<commit_message>
Correction: Recalculate merged Abhishek Shaji wage log using his actual daily rates
</commit_message>
<xml_diff>
--- a/Attendance_Payroll.xlsx
+++ b/Attendance_Payroll.xlsx
@@ -18564,13 +18564,13 @@
         <v>0</v>
       </c>
       <c r="L363">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M363">
         <v>0</v>
       </c>
       <c r="N363">
-        <v>140</v>
+        <v>466.67</v>
       </c>
       <c r="O363" t="str" xml:space="preserve">
         <v xml:space="preserve">Abhishek s

</xml_diff>

<commit_message>
feat: implement robust live recovery of missed WhatsApp messages on boot
</commit_message>
<xml_diff>
--- a/Attendance_Payroll.xlsx
+++ b/Attendance_Payroll.xlsx
@@ -405,7 +405,7 @@
     <col min="4" max="4" width="13.83203125" customWidth="1"/>
     <col min="5" max="5" width="31.83203125" customWidth="1"/>
     <col min="6" max="6" width="15.83203125" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="22.83203125" customWidth="1"/>
     <col min="8" max="8" width="20.83203125" customWidth="1"/>
     <col min="9" max="9" width="25.83203125" customWidth="1"/>
     <col min="10" max="10" width="25.83203125" customWidth="1"/>
@@ -414,7 +414,7 @@
     <col min="13" max="13" width="19.83203125" customWidth="1"/>
     <col min="14" max="14" width="22.83203125" customWidth="1"/>
     <col min="15" max="15" width="119.83203125" customWidth="1"/>
-    <col min="16" max="16" width="35.83203125" customWidth="1"/>
+    <col min="16" max="16" width="62.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -20042,16 +20042,16 @@
         <v>Maya Sunil</v>
       </c>
       <c r="D393" t="str">
-        <v>ABSENT</v>
+        <v>CHECKED-IN</v>
       </c>
       <c r="E393" t="str">
-        <v>—</v>
+        <v>INTEREXT OFFICE</v>
       </c>
       <c r="F393" t="str">
-        <v>—</v>
+        <v>12:11 PM</v>
       </c>
       <c r="G393" t="str">
-        <v>—</v>
+        <v>Currently Checked-In</v>
       </c>
       <c r="H393">
         <v>0</v>
@@ -20075,10 +20075,10 @@
         <v>0</v>
       </c>
       <c r="O393" t="str">
-        <v>—</v>
+        <v>Selfie caption</v>
       </c>
       <c r="P393" t="str">
-        <v>Auto-Marked Absent (Missing text)</v>
+        <v>[FLAGGED SELFIE] Location Mismatch via Location Pin (44637m)</v>
       </c>
     </row>
     <row r="394">

</xml_diff>

<commit_message>
feat: support parsing and logging worker leaves with tomorrow offset from WhatsApp
</commit_message>
<xml_diff>
--- a/Attendance_Payroll.xlsx
+++ b/Attendance_Payroll.xlsx
@@ -405,7 +405,7 @@
     <col min="4" max="4" width="13.83203125" customWidth="1"/>
     <col min="5" max="5" width="31.83203125" customWidth="1"/>
     <col min="6" max="6" width="15.83203125" customWidth="1"/>
-    <col min="7" max="7" width="22.83203125" customWidth="1"/>
+    <col min="7" max="7" width="16.83203125" customWidth="1"/>
     <col min="8" max="8" width="20.83203125" customWidth="1"/>
     <col min="9" max="9" width="25.83203125" customWidth="1"/>
     <col min="10" max="10" width="25.83203125" customWidth="1"/>
@@ -414,7 +414,7 @@
     <col min="13" max="13" width="19.83203125" customWidth="1"/>
     <col min="14" max="14" width="22.83203125" customWidth="1"/>
     <col min="15" max="15" width="119.83203125" customWidth="1"/>
-    <col min="16" max="16" width="62.83203125" customWidth="1"/>
+    <col min="16" max="16" width="35.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -20042,16 +20042,16 @@
         <v>Maya Sunil</v>
       </c>
       <c r="D393" t="str">
-        <v>CHECKED-IN</v>
+        <v>ABSENT</v>
       </c>
       <c r="E393" t="str">
-        <v>INTEREXT OFFICE</v>
+        <v>—</v>
       </c>
       <c r="F393" t="str">
-        <v>12:11 PM</v>
+        <v>—</v>
       </c>
       <c r="G393" t="str">
-        <v>Currently Checked-In</v>
+        <v>—</v>
       </c>
       <c r="H393">
         <v>0</v>
@@ -20075,10 +20075,10 @@
         <v>0</v>
       </c>
       <c r="O393" t="str">
-        <v>Selfie caption</v>
+        <v>—</v>
       </c>
       <c r="P393" t="str">
-        <v>[FLAGGED SELFIE] Location Mismatch via Location Pin (44637m)</v>
+        <v>Auto-Marked Absent (Missing text)</v>
       </c>
     </row>
     <row r="394">

</xml_diff>

<commit_message>
Fix duplicate initialization race condition, handle format-insensitive phone lookups, filter system events, and dump whatsapp group members list
</commit_message>
<xml_diff>
--- a/Attendance_Payroll.xlsx
+++ b/Attendance_Payroll.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P577"/>
+  <dimension ref="A1:P649"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="13.83203125" customWidth="1"/>
@@ -405,7 +405,7 @@
     <col min="4" max="4" width="13.83203125" customWidth="1"/>
     <col min="5" max="5" width="31.83203125" customWidth="1"/>
     <col min="6" max="6" width="15.83203125" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="22.83203125" customWidth="1"/>
     <col min="8" max="8" width="20.83203125" customWidth="1"/>
     <col min="9" max="9" width="25.83203125" customWidth="1"/>
     <col min="10" max="10" width="25.83203125" customWidth="1"/>
@@ -29277,9 +29277,3609 @@
         <v/>
       </c>
     </row>
+    <row r="578">
+      <c r="A578" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B578" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C578" t="str">
+        <v>Aamil</v>
+      </c>
+      <c r="D578" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E578" t="str">
+        <v>—</v>
+      </c>
+      <c r="F578" t="str">
+        <v>—</v>
+      </c>
+      <c r="G578" t="str">
+        <v>—</v>
+      </c>
+      <c r="H578">
+        <v>0</v>
+      </c>
+      <c r="I578">
+        <v>0</v>
+      </c>
+      <c r="J578">
+        <v>0</v>
+      </c>
+      <c r="K578">
+        <v>0</v>
+      </c>
+      <c r="L578">
+        <v>0</v>
+      </c>
+      <c r="M578">
+        <v>0</v>
+      </c>
+      <c r="N578">
+        <v>0</v>
+      </c>
+      <c r="O578" t="str">
+        <v>—</v>
+      </c>
+      <c r="P578" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B579" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C579" t="str">
+        <v>Abhishek Shaji</v>
+      </c>
+      <c r="D579" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E579" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F579" t="str">
+        <v>11:22 AM</v>
+      </c>
+      <c r="G579" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H579">
+        <v>0</v>
+      </c>
+      <c r="I579">
+        <v>0</v>
+      </c>
+      <c r="J579">
+        <v>0</v>
+      </c>
+      <c r="K579">
+        <v>0</v>
+      </c>
+      <c r="L579">
+        <v>0</v>
+      </c>
+      <c r="M579">
+        <v>0</v>
+      </c>
+      <c r="N579">
+        <v>0</v>
+      </c>
+      <c r="O579" t="str">
+        <v>Abhishek Shaji</v>
+      </c>
+      <c r="P579" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B580" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C580" t="str">
+        <v>AJEESH VIJAYAN</v>
+      </c>
+      <c r="D580" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E580" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F580" t="str">
+        <v>11:22 AM</v>
+      </c>
+      <c r="G580" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H580">
+        <v>0</v>
+      </c>
+      <c r="I580">
+        <v>0</v>
+      </c>
+      <c r="J580">
+        <v>0</v>
+      </c>
+      <c r="K580">
+        <v>0</v>
+      </c>
+      <c r="L580">
+        <v>0</v>
+      </c>
+      <c r="M580">
+        <v>0</v>
+      </c>
+      <c r="N580">
+        <v>0</v>
+      </c>
+      <c r="O580" t="str">
+        <v>Ajeesh Vijayan</v>
+      </c>
+      <c r="P580" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B581" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C581" t="str">
+        <v>Ajith Reghunath</v>
+      </c>
+      <c r="D581" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E581" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F581" t="str">
+        <v>11:22 AM</v>
+      </c>
+      <c r="G581" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H581">
+        <v>0</v>
+      </c>
+      <c r="I581">
+        <v>0</v>
+      </c>
+      <c r="J581">
+        <v>0</v>
+      </c>
+      <c r="K581">
+        <v>0</v>
+      </c>
+      <c r="L581">
+        <v>0</v>
+      </c>
+      <c r="M581">
+        <v>0</v>
+      </c>
+      <c r="N581">
+        <v>0</v>
+      </c>
+      <c r="O581" t="str">
+        <v>Ajith Reghunath</v>
+      </c>
+      <c r="P581" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B582" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C582" t="str">
+        <v>Ajmal K H</v>
+      </c>
+      <c r="D582" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E582" t="str">
+        <v>—</v>
+      </c>
+      <c r="F582" t="str">
+        <v>—</v>
+      </c>
+      <c r="G582" t="str">
+        <v>—</v>
+      </c>
+      <c r="H582">
+        <v>0</v>
+      </c>
+      <c r="I582">
+        <v>0</v>
+      </c>
+      <c r="J582">
+        <v>0</v>
+      </c>
+      <c r="K582">
+        <v>0</v>
+      </c>
+      <c r="L582">
+        <v>0</v>
+      </c>
+      <c r="M582">
+        <v>0</v>
+      </c>
+      <c r="N582">
+        <v>0</v>
+      </c>
+      <c r="O582" t="str">
+        <v>—</v>
+      </c>
+      <c r="P582" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B583" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C583" t="str">
+        <v>Akash</v>
+      </c>
+      <c r="D583" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E583" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F583" t="str">
+        <v>11:22 AM</v>
+      </c>
+      <c r="G583" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H583">
+        <v>0</v>
+      </c>
+      <c r="I583">
+        <v>0</v>
+      </c>
+      <c r="J583">
+        <v>0</v>
+      </c>
+      <c r="K583">
+        <v>0</v>
+      </c>
+      <c r="L583">
+        <v>0</v>
+      </c>
+      <c r="M583">
+        <v>0</v>
+      </c>
+      <c r="N583">
+        <v>0</v>
+      </c>
+      <c r="O583" t="str">
+        <v>Akash Rana</v>
+      </c>
+      <c r="P583" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B584" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C584" t="str">
+        <v>Akhil AK</v>
+      </c>
+      <c r="D584" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E584" t="str">
+        <v>—</v>
+      </c>
+      <c r="F584" t="str">
+        <v>—</v>
+      </c>
+      <c r="G584" t="str">
+        <v>—</v>
+      </c>
+      <c r="H584">
+        <v>0</v>
+      </c>
+      <c r="I584">
+        <v>0</v>
+      </c>
+      <c r="J584">
+        <v>0</v>
+      </c>
+      <c r="K584">
+        <v>0</v>
+      </c>
+      <c r="L584">
+        <v>0</v>
+      </c>
+      <c r="M584">
+        <v>0</v>
+      </c>
+      <c r="N584">
+        <v>0</v>
+      </c>
+      <c r="O584" t="str">
+        <v>—</v>
+      </c>
+      <c r="P584" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B585" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C585" t="str">
+        <v>AKHIL P KUMAR</v>
+      </c>
+      <c r="D585" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E585" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F585" t="str">
+        <v>11:22 AM</v>
+      </c>
+      <c r="G585" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H585">
+        <v>0</v>
+      </c>
+      <c r="I585">
+        <v>0</v>
+      </c>
+      <c r="J585">
+        <v>0</v>
+      </c>
+      <c r="K585">
+        <v>0</v>
+      </c>
+      <c r="L585">
+        <v>0</v>
+      </c>
+      <c r="M585">
+        <v>0</v>
+      </c>
+      <c r="N585">
+        <v>0</v>
+      </c>
+      <c r="O585" t="str">
+        <v>Akhil P Kumar</v>
+      </c>
+      <c r="P585" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B586" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C586" t="str">
+        <v>Alex Rajan</v>
+      </c>
+      <c r="D586" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E586" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F586" t="str">
+        <v>11:22 AM</v>
+      </c>
+      <c r="G586" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H586">
+        <v>0</v>
+      </c>
+      <c r="I586">
+        <v>0</v>
+      </c>
+      <c r="J586">
+        <v>0</v>
+      </c>
+      <c r="K586">
+        <v>0</v>
+      </c>
+      <c r="L586">
+        <v>0</v>
+      </c>
+      <c r="M586">
+        <v>0</v>
+      </c>
+      <c r="N586">
+        <v>0</v>
+      </c>
+      <c r="O586" t="str">
+        <v>Alex Gigi</v>
+      </c>
+      <c r="P586" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B587" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C587" t="str">
+        <v>ANADHU SUNIL</v>
+      </c>
+      <c r="D587" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E587" t="str">
+        <v>—</v>
+      </c>
+      <c r="F587" t="str">
+        <v>—</v>
+      </c>
+      <c r="G587" t="str">
+        <v>—</v>
+      </c>
+      <c r="H587">
+        <v>0</v>
+      </c>
+      <c r="I587">
+        <v>0</v>
+      </c>
+      <c r="J587">
+        <v>0</v>
+      </c>
+      <c r="K587">
+        <v>0</v>
+      </c>
+      <c r="L587">
+        <v>0</v>
+      </c>
+      <c r="M587">
+        <v>0</v>
+      </c>
+      <c r="N587">
+        <v>0</v>
+      </c>
+      <c r="O587" t="str">
+        <v>—</v>
+      </c>
+      <c r="P587" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B588" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C588" t="str">
+        <v>Anandhu Raj</v>
+      </c>
+      <c r="D588" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E588" t="str">
+        <v>—</v>
+      </c>
+      <c r="F588" t="str">
+        <v>—</v>
+      </c>
+      <c r="G588" t="str">
+        <v>—</v>
+      </c>
+      <c r="H588">
+        <v>0</v>
+      </c>
+      <c r="I588">
+        <v>0</v>
+      </c>
+      <c r="J588">
+        <v>0</v>
+      </c>
+      <c r="K588">
+        <v>0</v>
+      </c>
+      <c r="L588">
+        <v>0</v>
+      </c>
+      <c r="M588">
+        <v>0</v>
+      </c>
+      <c r="N588">
+        <v>0</v>
+      </c>
+      <c r="O588" t="str">
+        <v>—</v>
+      </c>
+      <c r="P588" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B589" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C589" t="str">
+        <v>Aneesh Ahammed</v>
+      </c>
+      <c r="D589" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E589" t="str">
+        <v>—</v>
+      </c>
+      <c r="F589" t="str">
+        <v>—</v>
+      </c>
+      <c r="G589" t="str">
+        <v>—</v>
+      </c>
+      <c r="H589">
+        <v>0</v>
+      </c>
+      <c r="I589">
+        <v>0</v>
+      </c>
+      <c r="J589">
+        <v>0</v>
+      </c>
+      <c r="K589">
+        <v>0</v>
+      </c>
+      <c r="L589">
+        <v>0</v>
+      </c>
+      <c r="M589">
+        <v>0</v>
+      </c>
+      <c r="N589">
+        <v>0</v>
+      </c>
+      <c r="O589" t="str">
+        <v>—</v>
+      </c>
+      <c r="P589" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B590" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C590" t="str">
+        <v>Anil Rana</v>
+      </c>
+      <c r="D590" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E590" t="str">
+        <v>—</v>
+      </c>
+      <c r="F590" t="str">
+        <v>—</v>
+      </c>
+      <c r="G590" t="str">
+        <v>—</v>
+      </c>
+      <c r="H590">
+        <v>0</v>
+      </c>
+      <c r="I590">
+        <v>0</v>
+      </c>
+      <c r="J590">
+        <v>0</v>
+      </c>
+      <c r="K590">
+        <v>0</v>
+      </c>
+      <c r="L590">
+        <v>0</v>
+      </c>
+      <c r="M590">
+        <v>0</v>
+      </c>
+      <c r="N590">
+        <v>0</v>
+      </c>
+      <c r="O590" t="str">
+        <v>—</v>
+      </c>
+      <c r="P590" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B591" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C591" t="str">
+        <v>Anish Viswanathan</v>
+      </c>
+      <c r="D591" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E591" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F591" t="str">
+        <v>11:22 AM</v>
+      </c>
+      <c r="G591" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H591">
+        <v>0</v>
+      </c>
+      <c r="I591">
+        <v>0</v>
+      </c>
+      <c r="J591">
+        <v>0</v>
+      </c>
+      <c r="K591">
+        <v>0</v>
+      </c>
+      <c r="L591">
+        <v>0</v>
+      </c>
+      <c r="M591">
+        <v>0</v>
+      </c>
+      <c r="N591">
+        <v>0</v>
+      </c>
+      <c r="O591" t="str">
+        <v>Anish Viswanathan</v>
+      </c>
+      <c r="P591" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B592" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C592" t="str">
+        <v>Anoop (Ancil K Grace)</v>
+      </c>
+      <c r="D592" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E592" t="str">
+        <v>—</v>
+      </c>
+      <c r="F592" t="str">
+        <v>—</v>
+      </c>
+      <c r="G592" t="str">
+        <v>—</v>
+      </c>
+      <c r="H592">
+        <v>0</v>
+      </c>
+      <c r="I592">
+        <v>0</v>
+      </c>
+      <c r="J592">
+        <v>0</v>
+      </c>
+      <c r="K592">
+        <v>0</v>
+      </c>
+      <c r="L592">
+        <v>0</v>
+      </c>
+      <c r="M592">
+        <v>0</v>
+      </c>
+      <c r="N592">
+        <v>0</v>
+      </c>
+      <c r="O592" t="str">
+        <v>—</v>
+      </c>
+      <c r="P592" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B593" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C593" t="str">
+        <v>Anusree Subramanian</v>
+      </c>
+      <c r="D593" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E593" t="str">
+        <v>—</v>
+      </c>
+      <c r="F593" t="str">
+        <v>—</v>
+      </c>
+      <c r="G593" t="str">
+        <v>—</v>
+      </c>
+      <c r="H593">
+        <v>0</v>
+      </c>
+      <c r="I593">
+        <v>0</v>
+      </c>
+      <c r="J593">
+        <v>0</v>
+      </c>
+      <c r="K593">
+        <v>0</v>
+      </c>
+      <c r="L593">
+        <v>0</v>
+      </c>
+      <c r="M593">
+        <v>0</v>
+      </c>
+      <c r="N593">
+        <v>0</v>
+      </c>
+      <c r="O593" t="str">
+        <v>—</v>
+      </c>
+      <c r="P593" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B594" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C594" t="str">
+        <v>Arun George</v>
+      </c>
+      <c r="D594" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E594" t="str">
+        <v>—</v>
+      </c>
+      <c r="F594" t="str">
+        <v>—</v>
+      </c>
+      <c r="G594" t="str">
+        <v>—</v>
+      </c>
+      <c r="H594">
+        <v>0</v>
+      </c>
+      <c r="I594">
+        <v>0</v>
+      </c>
+      <c r="J594">
+        <v>0</v>
+      </c>
+      <c r="K594">
+        <v>0</v>
+      </c>
+      <c r="L594">
+        <v>0</v>
+      </c>
+      <c r="M594">
+        <v>0</v>
+      </c>
+      <c r="N594">
+        <v>0</v>
+      </c>
+      <c r="O594" t="str">
+        <v>—</v>
+      </c>
+      <c r="P594" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B595" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C595" t="str">
+        <v>Arun P madhu</v>
+      </c>
+      <c r="D595" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E595" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F595" t="str">
+        <v>11:22 AM</v>
+      </c>
+      <c r="G595" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H595">
+        <v>0</v>
+      </c>
+      <c r="I595">
+        <v>0</v>
+      </c>
+      <c r="J595">
+        <v>0</v>
+      </c>
+      <c r="K595">
+        <v>0</v>
+      </c>
+      <c r="L595">
+        <v>0</v>
+      </c>
+      <c r="M595">
+        <v>0</v>
+      </c>
+      <c r="N595">
+        <v>0</v>
+      </c>
+      <c r="O595" t="str">
+        <v>Arun P Madhu</v>
+      </c>
+      <c r="P595" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B596" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C596" t="str">
+        <v>Bimal Rana</v>
+      </c>
+      <c r="D596" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E596" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F596" t="str">
+        <v>11:22 AM</v>
+      </c>
+      <c r="G596" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H596">
+        <v>0</v>
+      </c>
+      <c r="I596">
+        <v>0</v>
+      </c>
+      <c r="J596">
+        <v>0</v>
+      </c>
+      <c r="K596">
+        <v>0</v>
+      </c>
+      <c r="L596">
+        <v>0</v>
+      </c>
+      <c r="M596">
+        <v>0</v>
+      </c>
+      <c r="N596">
+        <v>0</v>
+      </c>
+      <c r="O596" t="str">
+        <v>Bimal Rana</v>
+      </c>
+      <c r="P596" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B597" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C597" t="str">
+        <v>BINDHU JOSE</v>
+      </c>
+      <c r="D597" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E597" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F597" t="str">
+        <v>11:22 AM</v>
+      </c>
+      <c r="G597" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H597">
+        <v>0</v>
+      </c>
+      <c r="I597">
+        <v>0</v>
+      </c>
+      <c r="J597">
+        <v>0</v>
+      </c>
+      <c r="K597">
+        <v>0</v>
+      </c>
+      <c r="L597">
+        <v>0</v>
+      </c>
+      <c r="M597">
+        <v>0</v>
+      </c>
+      <c r="N597">
+        <v>0</v>
+      </c>
+      <c r="O597" t="str">
+        <v>Bindhu Jose</v>
+      </c>
+      <c r="P597" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B598" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C598" t="str">
+        <v>Devadas E K</v>
+      </c>
+      <c r="D598" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E598" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F598" t="str">
+        <v>11:22 AM</v>
+      </c>
+      <c r="G598" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H598">
+        <v>0</v>
+      </c>
+      <c r="I598">
+        <v>0</v>
+      </c>
+      <c r="J598">
+        <v>0</v>
+      </c>
+      <c r="K598">
+        <v>0</v>
+      </c>
+      <c r="L598">
+        <v>0</v>
+      </c>
+      <c r="M598">
+        <v>0</v>
+      </c>
+      <c r="N598">
+        <v>0</v>
+      </c>
+      <c r="O598" t="str">
+        <v>Devadas E K</v>
+      </c>
+      <c r="P598" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B599" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C599" t="str">
+        <v>Faiyaj Ansari</v>
+      </c>
+      <c r="D599" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E599" t="str">
+        <v>—</v>
+      </c>
+      <c r="F599" t="str">
+        <v>—</v>
+      </c>
+      <c r="G599" t="str">
+        <v>—</v>
+      </c>
+      <c r="H599">
+        <v>0</v>
+      </c>
+      <c r="I599">
+        <v>0</v>
+      </c>
+      <c r="J599">
+        <v>0</v>
+      </c>
+      <c r="K599">
+        <v>0</v>
+      </c>
+      <c r="L599">
+        <v>0</v>
+      </c>
+      <c r="M599">
+        <v>0</v>
+      </c>
+      <c r="N599">
+        <v>0</v>
+      </c>
+      <c r="O599" t="str">
+        <v>—</v>
+      </c>
+      <c r="P599" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B600" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C600" t="str">
+        <v>GEORGE THOMAS</v>
+      </c>
+      <c r="D600" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E600" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F600" t="str">
+        <v>11:22 AM</v>
+      </c>
+      <c r="G600" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H600">
+        <v>0</v>
+      </c>
+      <c r="I600">
+        <v>0</v>
+      </c>
+      <c r="J600">
+        <v>0</v>
+      </c>
+      <c r="K600">
+        <v>0</v>
+      </c>
+      <c r="L600">
+        <v>0</v>
+      </c>
+      <c r="M600">
+        <v>0</v>
+      </c>
+      <c r="N600">
+        <v>0</v>
+      </c>
+      <c r="O600" t="str">
+        <v>George Thomas</v>
+      </c>
+      <c r="P600" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B601" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C601" t="str">
+        <v>GOKUL K</v>
+      </c>
+      <c r="D601" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E601" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F601" t="str">
+        <v>11:22 AM</v>
+      </c>
+      <c r="G601" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H601">
+        <v>0</v>
+      </c>
+      <c r="I601">
+        <v>0</v>
+      </c>
+      <c r="J601">
+        <v>0</v>
+      </c>
+      <c r="K601">
+        <v>0</v>
+      </c>
+      <c r="L601">
+        <v>0</v>
+      </c>
+      <c r="M601">
+        <v>0</v>
+      </c>
+      <c r="N601">
+        <v>0</v>
+      </c>
+      <c r="O601" t="str">
+        <v>Gokul K</v>
+      </c>
+      <c r="P601" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B602" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C602" t="str">
+        <v>Gokul Krishnan  E V</v>
+      </c>
+      <c r="D602" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E602" t="str">
+        <v>—</v>
+      </c>
+      <c r="F602" t="str">
+        <v>—</v>
+      </c>
+      <c r="G602" t="str">
+        <v>—</v>
+      </c>
+      <c r="H602">
+        <v>0</v>
+      </c>
+      <c r="I602">
+        <v>0</v>
+      </c>
+      <c r="J602">
+        <v>0</v>
+      </c>
+      <c r="K602">
+        <v>0</v>
+      </c>
+      <c r="L602">
+        <v>0</v>
+      </c>
+      <c r="M602">
+        <v>0</v>
+      </c>
+      <c r="N602">
+        <v>0</v>
+      </c>
+      <c r="O602" t="str">
+        <v>—</v>
+      </c>
+      <c r="P602" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B603" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C603" t="str">
+        <v>Gopal (soma)</v>
+      </c>
+      <c r="D603" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E603" t="str">
+        <v>—</v>
+      </c>
+      <c r="F603" t="str">
+        <v>—</v>
+      </c>
+      <c r="G603" t="str">
+        <v>—</v>
+      </c>
+      <c r="H603">
+        <v>0</v>
+      </c>
+      <c r="I603">
+        <v>0</v>
+      </c>
+      <c r="J603">
+        <v>0</v>
+      </c>
+      <c r="K603">
+        <v>0</v>
+      </c>
+      <c r="L603">
+        <v>0</v>
+      </c>
+      <c r="M603">
+        <v>0</v>
+      </c>
+      <c r="N603">
+        <v>0</v>
+      </c>
+      <c r="O603" t="str">
+        <v>—</v>
+      </c>
+      <c r="P603" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B604" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C604" t="str">
+        <v>James TM</v>
+      </c>
+      <c r="D604" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E604" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F604" t="str">
+        <v>11:22 AM</v>
+      </c>
+      <c r="G604" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H604">
+        <v>0</v>
+      </c>
+      <c r="I604">
+        <v>0</v>
+      </c>
+      <c r="J604">
+        <v>0</v>
+      </c>
+      <c r="K604">
+        <v>0</v>
+      </c>
+      <c r="L604">
+        <v>0</v>
+      </c>
+      <c r="M604">
+        <v>0</v>
+      </c>
+      <c r="N604">
+        <v>0</v>
+      </c>
+      <c r="O604" t="str">
+        <v>James T M</v>
+      </c>
+      <c r="P604" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B605" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C605" t="str">
+        <v>Jitendra Rana</v>
+      </c>
+      <c r="D605" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E605" t="str">
+        <v>—</v>
+      </c>
+      <c r="F605" t="str">
+        <v>—</v>
+      </c>
+      <c r="G605" t="str">
+        <v>—</v>
+      </c>
+      <c r="H605">
+        <v>0</v>
+      </c>
+      <c r="I605">
+        <v>0</v>
+      </c>
+      <c r="J605">
+        <v>0</v>
+      </c>
+      <c r="K605">
+        <v>0</v>
+      </c>
+      <c r="L605">
+        <v>0</v>
+      </c>
+      <c r="M605">
+        <v>0</v>
+      </c>
+      <c r="N605">
+        <v>0</v>
+      </c>
+      <c r="O605" t="str">
+        <v>—</v>
+      </c>
+      <c r="P605" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B606" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C606" t="str">
+        <v>Joshy</v>
+      </c>
+      <c r="D606" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E606" t="str">
+        <v>—</v>
+      </c>
+      <c r="F606" t="str">
+        <v>—</v>
+      </c>
+      <c r="G606" t="str">
+        <v>—</v>
+      </c>
+      <c r="H606">
+        <v>0</v>
+      </c>
+      <c r="I606">
+        <v>0</v>
+      </c>
+      <c r="J606">
+        <v>0</v>
+      </c>
+      <c r="K606">
+        <v>0</v>
+      </c>
+      <c r="L606">
+        <v>0</v>
+      </c>
+      <c r="M606">
+        <v>0</v>
+      </c>
+      <c r="N606">
+        <v>0</v>
+      </c>
+      <c r="O606" t="str">
+        <v>—</v>
+      </c>
+      <c r="P606" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B607" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C607" t="str">
+        <v>Mahin KJ</v>
+      </c>
+      <c r="D607" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E607" t="str">
+        <v>—</v>
+      </c>
+      <c r="F607" t="str">
+        <v>—</v>
+      </c>
+      <c r="G607" t="str">
+        <v>—</v>
+      </c>
+      <c r="H607">
+        <v>0</v>
+      </c>
+      <c r="I607">
+        <v>0</v>
+      </c>
+      <c r="J607">
+        <v>0</v>
+      </c>
+      <c r="K607">
+        <v>0</v>
+      </c>
+      <c r="L607">
+        <v>0</v>
+      </c>
+      <c r="M607">
+        <v>0</v>
+      </c>
+      <c r="N607">
+        <v>0</v>
+      </c>
+      <c r="O607" t="str">
+        <v>—</v>
+      </c>
+      <c r="P607" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B608" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C608" t="str">
+        <v>Manu Mahesh</v>
+      </c>
+      <c r="D608" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E608" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F608" t="str">
+        <v>11:22 AM</v>
+      </c>
+      <c r="G608" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H608">
+        <v>0</v>
+      </c>
+      <c r="I608">
+        <v>0</v>
+      </c>
+      <c r="J608">
+        <v>0</v>
+      </c>
+      <c r="K608">
+        <v>0</v>
+      </c>
+      <c r="L608">
+        <v>0</v>
+      </c>
+      <c r="M608">
+        <v>0</v>
+      </c>
+      <c r="N608">
+        <v>0</v>
+      </c>
+      <c r="O608" t="str">
+        <v>Manu Mahesh</v>
+      </c>
+      <c r="P608" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B609" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C609" t="str">
+        <v>Maya Sunil</v>
+      </c>
+      <c r="D609" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E609" t="str">
+        <v>—</v>
+      </c>
+      <c r="F609" t="str">
+        <v>—</v>
+      </c>
+      <c r="G609" t="str">
+        <v>—</v>
+      </c>
+      <c r="H609">
+        <v>0</v>
+      </c>
+      <c r="I609">
+        <v>0</v>
+      </c>
+      <c r="J609">
+        <v>0</v>
+      </c>
+      <c r="K609">
+        <v>0</v>
+      </c>
+      <c r="L609">
+        <v>0</v>
+      </c>
+      <c r="M609">
+        <v>0</v>
+      </c>
+      <c r="N609">
+        <v>0</v>
+      </c>
+      <c r="O609" t="str">
+        <v>—</v>
+      </c>
+      <c r="P609" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B610" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C610" t="str">
+        <v>Mohammed Gulfam</v>
+      </c>
+      <c r="D610" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E610" t="str">
+        <v>—</v>
+      </c>
+      <c r="F610" t="str">
+        <v>—</v>
+      </c>
+      <c r="G610" t="str">
+        <v>—</v>
+      </c>
+      <c r="H610">
+        <v>0</v>
+      </c>
+      <c r="I610">
+        <v>0</v>
+      </c>
+      <c r="J610">
+        <v>0</v>
+      </c>
+      <c r="K610">
+        <v>0</v>
+      </c>
+      <c r="L610">
+        <v>0</v>
+      </c>
+      <c r="M610">
+        <v>0</v>
+      </c>
+      <c r="N610">
+        <v>0</v>
+      </c>
+      <c r="O610" t="str">
+        <v>—</v>
+      </c>
+      <c r="P610" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B611" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C611" t="str">
+        <v>NIJI MANOJ</v>
+      </c>
+      <c r="D611" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E611" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F611" t="str">
+        <v>11:22 AM</v>
+      </c>
+      <c r="G611" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H611">
+        <v>0</v>
+      </c>
+      <c r="I611">
+        <v>0</v>
+      </c>
+      <c r="J611">
+        <v>0</v>
+      </c>
+      <c r="K611">
+        <v>0</v>
+      </c>
+      <c r="L611">
+        <v>0</v>
+      </c>
+      <c r="M611">
+        <v>0</v>
+      </c>
+      <c r="N611">
+        <v>0</v>
+      </c>
+      <c r="O611" t="str">
+        <v>Niji Manoj</v>
+      </c>
+      <c r="P611" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B612" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C612" t="str">
+        <v>Niranjan Bose</v>
+      </c>
+      <c r="D612" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E612" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F612" t="str">
+        <v>11:22 AM</v>
+      </c>
+      <c r="G612" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H612">
+        <v>0</v>
+      </c>
+      <c r="I612">
+        <v>0</v>
+      </c>
+      <c r="J612">
+        <v>0</v>
+      </c>
+      <c r="K612">
+        <v>0</v>
+      </c>
+      <c r="L612">
+        <v>0</v>
+      </c>
+      <c r="M612">
+        <v>0</v>
+      </c>
+      <c r="N612">
+        <v>0</v>
+      </c>
+      <c r="O612" t="str">
+        <v>Niranjan Bose</v>
+      </c>
+      <c r="P612" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B613" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C613" t="str">
+        <v>NOURIN SHAJI</v>
+      </c>
+      <c r="D613" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E613" t="str">
+        <v>—</v>
+      </c>
+      <c r="F613" t="str">
+        <v>—</v>
+      </c>
+      <c r="G613" t="str">
+        <v>—</v>
+      </c>
+      <c r="H613">
+        <v>0</v>
+      </c>
+      <c r="I613">
+        <v>0</v>
+      </c>
+      <c r="J613">
+        <v>0</v>
+      </c>
+      <c r="K613">
+        <v>0</v>
+      </c>
+      <c r="L613">
+        <v>0</v>
+      </c>
+      <c r="M613">
+        <v>0</v>
+      </c>
+      <c r="N613">
+        <v>0</v>
+      </c>
+      <c r="O613" t="str">
+        <v>—</v>
+      </c>
+      <c r="P613" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B614" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C614" t="str">
+        <v>Pappu Kumar Rana</v>
+      </c>
+      <c r="D614" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E614" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F614" t="str">
+        <v>11:22 AM</v>
+      </c>
+      <c r="G614" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H614">
+        <v>0</v>
+      </c>
+      <c r="I614">
+        <v>0</v>
+      </c>
+      <c r="J614">
+        <v>0</v>
+      </c>
+      <c r="K614">
+        <v>0</v>
+      </c>
+      <c r="L614">
+        <v>0</v>
+      </c>
+      <c r="M614">
+        <v>0</v>
+      </c>
+      <c r="N614">
+        <v>0</v>
+      </c>
+      <c r="O614" t="str">
+        <v>Pappu Kumar Rana</v>
+      </c>
+      <c r="P614" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B615" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C615" t="str">
+        <v>PRASANTH E.M</v>
+      </c>
+      <c r="D615" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E615" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F615" t="str">
+        <v>11:22 AM</v>
+      </c>
+      <c r="G615" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H615">
+        <v>0</v>
+      </c>
+      <c r="I615">
+        <v>0</v>
+      </c>
+      <c r="J615">
+        <v>0</v>
+      </c>
+      <c r="K615">
+        <v>0</v>
+      </c>
+      <c r="L615">
+        <v>0</v>
+      </c>
+      <c r="M615">
+        <v>0</v>
+      </c>
+      <c r="N615">
+        <v>0</v>
+      </c>
+      <c r="O615" t="str">
+        <v>Prasanth E M</v>
+      </c>
+      <c r="P615" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B616" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C616" t="str">
+        <v>PRATHEESH K S</v>
+      </c>
+      <c r="D616" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E616" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F616" t="str">
+        <v>11:22 AM</v>
+      </c>
+      <c r="G616" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H616">
+        <v>0</v>
+      </c>
+      <c r="I616">
+        <v>0</v>
+      </c>
+      <c r="J616">
+        <v>0</v>
+      </c>
+      <c r="K616">
+        <v>0</v>
+      </c>
+      <c r="L616">
+        <v>0</v>
+      </c>
+      <c r="M616">
+        <v>0</v>
+      </c>
+      <c r="N616">
+        <v>0</v>
+      </c>
+      <c r="O616" t="str">
+        <v>Pratheesh K S</v>
+      </c>
+      <c r="P616" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B617" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C617" t="str">
+        <v>Rahul Das</v>
+      </c>
+      <c r="D617" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E617" t="str">
+        <v>—</v>
+      </c>
+      <c r="F617" t="str">
+        <v>—</v>
+      </c>
+      <c r="G617" t="str">
+        <v>—</v>
+      </c>
+      <c r="H617">
+        <v>0</v>
+      </c>
+      <c r="I617">
+        <v>0</v>
+      </c>
+      <c r="J617">
+        <v>0</v>
+      </c>
+      <c r="K617">
+        <v>0</v>
+      </c>
+      <c r="L617">
+        <v>0</v>
+      </c>
+      <c r="M617">
+        <v>0</v>
+      </c>
+      <c r="N617">
+        <v>0</v>
+      </c>
+      <c r="O617" t="str">
+        <v>—</v>
+      </c>
+      <c r="P617" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B618" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C618" t="str">
+        <v>Rahul R Nair</v>
+      </c>
+      <c r="D618" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E618" t="str">
+        <v>—</v>
+      </c>
+      <c r="F618" t="str">
+        <v>—</v>
+      </c>
+      <c r="G618" t="str">
+        <v>—</v>
+      </c>
+      <c r="H618">
+        <v>0</v>
+      </c>
+      <c r="I618">
+        <v>0</v>
+      </c>
+      <c r="J618">
+        <v>0</v>
+      </c>
+      <c r="K618">
+        <v>0</v>
+      </c>
+      <c r="L618">
+        <v>0</v>
+      </c>
+      <c r="M618">
+        <v>0</v>
+      </c>
+      <c r="N618">
+        <v>0</v>
+      </c>
+      <c r="O618" t="str">
+        <v>—</v>
+      </c>
+      <c r="P618" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B619" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C619" t="str">
+        <v>RAHUL SUNDARAN</v>
+      </c>
+      <c r="D619" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E619" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F619" t="str">
+        <v>11:22 AM</v>
+      </c>
+      <c r="G619" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H619">
+        <v>0</v>
+      </c>
+      <c r="I619">
+        <v>0</v>
+      </c>
+      <c r="J619">
+        <v>0</v>
+      </c>
+      <c r="K619">
+        <v>0</v>
+      </c>
+      <c r="L619">
+        <v>0</v>
+      </c>
+      <c r="M619">
+        <v>0</v>
+      </c>
+      <c r="N619">
+        <v>0</v>
+      </c>
+      <c r="O619" t="str">
+        <v>Rahul Sundaran</v>
+      </c>
+      <c r="P619" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B620" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C620" t="str">
+        <v>Raj Kumar Rana</v>
+      </c>
+      <c r="D620" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E620" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F620" t="str">
+        <v>11:22 AM</v>
+      </c>
+      <c r="G620" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H620">
+        <v>0</v>
+      </c>
+      <c r="I620">
+        <v>0</v>
+      </c>
+      <c r="J620">
+        <v>0</v>
+      </c>
+      <c r="K620">
+        <v>0</v>
+      </c>
+      <c r="L620">
+        <v>0</v>
+      </c>
+      <c r="M620">
+        <v>0</v>
+      </c>
+      <c r="N620">
+        <v>0</v>
+      </c>
+      <c r="O620" t="str">
+        <v>Rajkumar Rana</v>
+      </c>
+      <c r="P620" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B621" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C621" t="str">
+        <v>RAJI KANNAN</v>
+      </c>
+      <c r="D621" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E621" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F621" t="str">
+        <v>11:22 AM</v>
+      </c>
+      <c r="G621" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H621">
+        <v>0</v>
+      </c>
+      <c r="I621">
+        <v>0</v>
+      </c>
+      <c r="J621">
+        <v>0</v>
+      </c>
+      <c r="K621">
+        <v>0</v>
+      </c>
+      <c r="L621">
+        <v>0</v>
+      </c>
+      <c r="M621">
+        <v>0</v>
+      </c>
+      <c r="N621">
+        <v>0</v>
+      </c>
+      <c r="O621" t="str">
+        <v>Raji Kannan</v>
+      </c>
+      <c r="P621" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B622" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C622" t="str">
+        <v>Raju Rana</v>
+      </c>
+      <c r="D622" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E622" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F622" t="str">
+        <v>11:22 AM</v>
+      </c>
+      <c r="G622" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H622">
+        <v>0</v>
+      </c>
+      <c r="I622">
+        <v>0</v>
+      </c>
+      <c r="J622">
+        <v>0</v>
+      </c>
+      <c r="K622">
+        <v>0</v>
+      </c>
+      <c r="L622">
+        <v>0</v>
+      </c>
+      <c r="M622">
+        <v>0</v>
+      </c>
+      <c r="N622">
+        <v>0</v>
+      </c>
+      <c r="O622" t="str">
+        <v>Raju Rana</v>
+      </c>
+      <c r="P622" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B623" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C623" t="str">
+        <v>Rakesh Sadhukha</v>
+      </c>
+      <c r="D623" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E623" t="str">
+        <v>—</v>
+      </c>
+      <c r="F623" t="str">
+        <v>—</v>
+      </c>
+      <c r="G623" t="str">
+        <v>—</v>
+      </c>
+      <c r="H623">
+        <v>0</v>
+      </c>
+      <c r="I623">
+        <v>0</v>
+      </c>
+      <c r="J623">
+        <v>0</v>
+      </c>
+      <c r="K623">
+        <v>0</v>
+      </c>
+      <c r="L623">
+        <v>0</v>
+      </c>
+      <c r="M623">
+        <v>0</v>
+      </c>
+      <c r="N623">
+        <v>0</v>
+      </c>
+      <c r="O623" t="str">
+        <v>—</v>
+      </c>
+      <c r="P623" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B624" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C624" t="str">
+        <v>Ratheesh K S</v>
+      </c>
+      <c r="D624" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E624" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F624" t="str">
+        <v>11:22 AM</v>
+      </c>
+      <c r="G624" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H624">
+        <v>0</v>
+      </c>
+      <c r="I624">
+        <v>0</v>
+      </c>
+      <c r="J624">
+        <v>0</v>
+      </c>
+      <c r="K624">
+        <v>0</v>
+      </c>
+      <c r="L624">
+        <v>0</v>
+      </c>
+      <c r="M624">
+        <v>0</v>
+      </c>
+      <c r="N624">
+        <v>0</v>
+      </c>
+      <c r="O624" t="str">
+        <v>Ratheesh K S</v>
+      </c>
+      <c r="P624" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B625" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C625" t="str">
+        <v>Ratheesh P R</v>
+      </c>
+      <c r="D625" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E625" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F625" t="str">
+        <v>11:22 AM</v>
+      </c>
+      <c r="G625" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H625">
+        <v>0</v>
+      </c>
+      <c r="I625">
+        <v>0</v>
+      </c>
+      <c r="J625">
+        <v>0</v>
+      </c>
+      <c r="K625">
+        <v>0</v>
+      </c>
+      <c r="L625">
+        <v>0</v>
+      </c>
+      <c r="M625">
+        <v>0</v>
+      </c>
+      <c r="N625">
+        <v>0</v>
+      </c>
+      <c r="O625" t="str">
+        <v>Ratheesh P R</v>
+      </c>
+      <c r="P625" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B626" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C626" t="str">
+        <v>REBEESH K S</v>
+      </c>
+      <c r="D626" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E626" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F626" t="str">
+        <v>11:22 AM</v>
+      </c>
+      <c r="G626" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H626">
+        <v>0</v>
+      </c>
+      <c r="I626">
+        <v>0</v>
+      </c>
+      <c r="J626">
+        <v>0</v>
+      </c>
+      <c r="K626">
+        <v>0</v>
+      </c>
+      <c r="L626">
+        <v>0</v>
+      </c>
+      <c r="M626">
+        <v>0</v>
+      </c>
+      <c r="N626">
+        <v>0</v>
+      </c>
+      <c r="O626" t="str">
+        <v>Rebeesh K S</v>
+      </c>
+      <c r="P626" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B627" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C627" t="str">
+        <v>REKHA MADHU</v>
+      </c>
+      <c r="D627" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E627" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F627" t="str">
+        <v>11:22 AM</v>
+      </c>
+      <c r="G627" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H627">
+        <v>0</v>
+      </c>
+      <c r="I627">
+        <v>0</v>
+      </c>
+      <c r="J627">
+        <v>0</v>
+      </c>
+      <c r="K627">
+        <v>0</v>
+      </c>
+      <c r="L627">
+        <v>0</v>
+      </c>
+      <c r="M627">
+        <v>0</v>
+      </c>
+      <c r="N627">
+        <v>0</v>
+      </c>
+      <c r="O627" t="str">
+        <v>Reksha Madhu</v>
+      </c>
+      <c r="P627" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B628" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C628" t="str">
+        <v>Remanan N N</v>
+      </c>
+      <c r="D628" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E628" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F628" t="str">
+        <v>11:22 AM</v>
+      </c>
+      <c r="G628" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H628">
+        <v>0</v>
+      </c>
+      <c r="I628">
+        <v>0</v>
+      </c>
+      <c r="J628">
+        <v>0</v>
+      </c>
+      <c r="K628">
+        <v>0</v>
+      </c>
+      <c r="L628">
+        <v>0</v>
+      </c>
+      <c r="M628">
+        <v>0</v>
+      </c>
+      <c r="N628">
+        <v>0</v>
+      </c>
+      <c r="O628" t="str">
+        <v>Remanan N N</v>
+      </c>
+      <c r="P628" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B629" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C629" t="str">
+        <v>Sabu (Joseph Antony)</v>
+      </c>
+      <c r="D629" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E629" t="str">
+        <v>—</v>
+      </c>
+      <c r="F629" t="str">
+        <v>—</v>
+      </c>
+      <c r="G629" t="str">
+        <v>—</v>
+      </c>
+      <c r="H629">
+        <v>0</v>
+      </c>
+      <c r="I629">
+        <v>0</v>
+      </c>
+      <c r="J629">
+        <v>0</v>
+      </c>
+      <c r="K629">
+        <v>0</v>
+      </c>
+      <c r="L629">
+        <v>0</v>
+      </c>
+      <c r="M629">
+        <v>0</v>
+      </c>
+      <c r="N629">
+        <v>0</v>
+      </c>
+      <c r="O629" t="str">
+        <v>—</v>
+      </c>
+      <c r="P629" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B630" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C630" t="str">
+        <v>Samshad Aalam</v>
+      </c>
+      <c r="D630" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E630" t="str">
+        <v>—</v>
+      </c>
+      <c r="F630" t="str">
+        <v>—</v>
+      </c>
+      <c r="G630" t="str">
+        <v>—</v>
+      </c>
+      <c r="H630">
+        <v>0</v>
+      </c>
+      <c r="I630">
+        <v>0</v>
+      </c>
+      <c r="J630">
+        <v>0</v>
+      </c>
+      <c r="K630">
+        <v>0</v>
+      </c>
+      <c r="L630">
+        <v>0</v>
+      </c>
+      <c r="M630">
+        <v>0</v>
+      </c>
+      <c r="N630">
+        <v>0</v>
+      </c>
+      <c r="O630" t="str">
+        <v>—</v>
+      </c>
+      <c r="P630" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B631" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C631" t="str">
+        <v>Sandeep C</v>
+      </c>
+      <c r="D631" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E631" t="str">
+        <v>—</v>
+      </c>
+      <c r="F631" t="str">
+        <v>—</v>
+      </c>
+      <c r="G631" t="str">
+        <v>—</v>
+      </c>
+      <c r="H631">
+        <v>0</v>
+      </c>
+      <c r="I631">
+        <v>0</v>
+      </c>
+      <c r="J631">
+        <v>0</v>
+      </c>
+      <c r="K631">
+        <v>0</v>
+      </c>
+      <c r="L631">
+        <v>0</v>
+      </c>
+      <c r="M631">
+        <v>0</v>
+      </c>
+      <c r="N631">
+        <v>0</v>
+      </c>
+      <c r="O631" t="str">
+        <v>—</v>
+      </c>
+      <c r="P631" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B632" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C632" t="str">
+        <v>SHAHANA JABBAR</v>
+      </c>
+      <c r="D632" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E632" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F632" t="str">
+        <v>11:22 AM</v>
+      </c>
+      <c r="G632" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H632">
+        <v>0</v>
+      </c>
+      <c r="I632">
+        <v>0</v>
+      </c>
+      <c r="J632">
+        <v>0</v>
+      </c>
+      <c r="K632">
+        <v>0</v>
+      </c>
+      <c r="L632">
+        <v>0</v>
+      </c>
+      <c r="M632">
+        <v>0</v>
+      </c>
+      <c r="N632">
+        <v>0</v>
+      </c>
+      <c r="O632" t="str">
+        <v>Shahana Jabbar</v>
+      </c>
+      <c r="P632" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B633" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C633" t="str">
+        <v>SHINODH N T</v>
+      </c>
+      <c r="D633" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E633" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F633" t="str">
+        <v>11:22 AM</v>
+      </c>
+      <c r="G633" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H633">
+        <v>0</v>
+      </c>
+      <c r="I633">
+        <v>0</v>
+      </c>
+      <c r="J633">
+        <v>0</v>
+      </c>
+      <c r="K633">
+        <v>0</v>
+      </c>
+      <c r="L633">
+        <v>0</v>
+      </c>
+      <c r="M633">
+        <v>0</v>
+      </c>
+      <c r="N633">
+        <v>0</v>
+      </c>
+      <c r="O633" t="str">
+        <v>Shinod N T</v>
+      </c>
+      <c r="P633" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B634" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C634" t="str">
+        <v>SHYAM MURALI</v>
+      </c>
+      <c r="D634" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E634" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F634" t="str">
+        <v>11:22 AM</v>
+      </c>
+      <c r="G634" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H634">
+        <v>0</v>
+      </c>
+      <c r="I634">
+        <v>0</v>
+      </c>
+      <c r="J634">
+        <v>0</v>
+      </c>
+      <c r="K634">
+        <v>0</v>
+      </c>
+      <c r="L634">
+        <v>0</v>
+      </c>
+      <c r="M634">
+        <v>0</v>
+      </c>
+      <c r="N634">
+        <v>0</v>
+      </c>
+      <c r="O634" t="str">
+        <v>Shyam Murali</v>
+      </c>
+      <c r="P634" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B635" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C635" t="str">
+        <v>Siju Thomas</v>
+      </c>
+      <c r="D635" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E635" t="str">
+        <v>—</v>
+      </c>
+      <c r="F635" t="str">
+        <v>—</v>
+      </c>
+      <c r="G635" t="str">
+        <v>—</v>
+      </c>
+      <c r="H635">
+        <v>0</v>
+      </c>
+      <c r="I635">
+        <v>0</v>
+      </c>
+      <c r="J635">
+        <v>0</v>
+      </c>
+      <c r="K635">
+        <v>0</v>
+      </c>
+      <c r="L635">
+        <v>0</v>
+      </c>
+      <c r="M635">
+        <v>0</v>
+      </c>
+      <c r="N635">
+        <v>0</v>
+      </c>
+      <c r="O635" t="str">
+        <v>—</v>
+      </c>
+      <c r="P635" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B636" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C636" t="str">
+        <v>Sineesh Sasi</v>
+      </c>
+      <c r="D636" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E636" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F636" t="str">
+        <v>11:22 AM</v>
+      </c>
+      <c r="G636" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H636">
+        <v>0</v>
+      </c>
+      <c r="I636">
+        <v>0</v>
+      </c>
+      <c r="J636">
+        <v>0</v>
+      </c>
+      <c r="K636">
+        <v>0</v>
+      </c>
+      <c r="L636">
+        <v>0</v>
+      </c>
+      <c r="M636">
+        <v>0</v>
+      </c>
+      <c r="N636">
+        <v>0</v>
+      </c>
+      <c r="O636" t="str">
+        <v>Sineesh Sasi</v>
+      </c>
+      <c r="P636" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B637" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C637" t="str">
+        <v>Sona Francis</v>
+      </c>
+      <c r="D637" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E637" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F637" t="str">
+        <v>11:22 AM</v>
+      </c>
+      <c r="G637" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H637">
+        <v>0</v>
+      </c>
+      <c r="I637">
+        <v>0</v>
+      </c>
+      <c r="J637">
+        <v>0</v>
+      </c>
+      <c r="K637">
+        <v>0</v>
+      </c>
+      <c r="L637">
+        <v>0</v>
+      </c>
+      <c r="M637">
+        <v>0</v>
+      </c>
+      <c r="N637">
+        <v>0</v>
+      </c>
+      <c r="O637" t="str">
+        <v>Sona Francis</v>
+      </c>
+      <c r="P637" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B638" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C638" t="str">
+        <v>Sreelakshmi R</v>
+      </c>
+      <c r="D638" t="str">
+        <v>LEAVE</v>
+      </c>
+      <c r="E638" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F638" t="str">
+        <v>—</v>
+      </c>
+      <c r="G638" t="str">
+        <v>—</v>
+      </c>
+      <c r="H638">
+        <v>0</v>
+      </c>
+      <c r="I638">
+        <v>0</v>
+      </c>
+      <c r="J638">
+        <v>0</v>
+      </c>
+      <c r="K638">
+        <v>0</v>
+      </c>
+      <c r="L638">
+        <v>0</v>
+      </c>
+      <c r="M638">
+        <v>0</v>
+      </c>
+      <c r="N638">
+        <v>0</v>
+      </c>
+      <c r="O638" t="str">
+        <v>Sreelakshmi R</v>
+      </c>
+      <c r="P638" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B639" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C639" t="str">
+        <v>Sreenath C V</v>
+      </c>
+      <c r="D639" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E639" t="str">
+        <v>—</v>
+      </c>
+      <c r="F639" t="str">
+        <v>—</v>
+      </c>
+      <c r="G639" t="str">
+        <v>—</v>
+      </c>
+      <c r="H639">
+        <v>0</v>
+      </c>
+      <c r="I639">
+        <v>0</v>
+      </c>
+      <c r="J639">
+        <v>0</v>
+      </c>
+      <c r="K639">
+        <v>0</v>
+      </c>
+      <c r="L639">
+        <v>0</v>
+      </c>
+      <c r="M639">
+        <v>0</v>
+      </c>
+      <c r="N639">
+        <v>0</v>
+      </c>
+      <c r="O639" t="str">
+        <v>—</v>
+      </c>
+      <c r="P639" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B640" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C640" t="str">
+        <v>Sreeraj V S</v>
+      </c>
+      <c r="D640" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E640" t="str">
+        <v>—</v>
+      </c>
+      <c r="F640" t="str">
+        <v>—</v>
+      </c>
+      <c r="G640" t="str">
+        <v>—</v>
+      </c>
+      <c r="H640">
+        <v>0</v>
+      </c>
+      <c r="I640">
+        <v>0</v>
+      </c>
+      <c r="J640">
+        <v>0</v>
+      </c>
+      <c r="K640">
+        <v>0</v>
+      </c>
+      <c r="L640">
+        <v>0</v>
+      </c>
+      <c r="M640">
+        <v>0</v>
+      </c>
+      <c r="N640">
+        <v>0</v>
+      </c>
+      <c r="O640" t="str">
+        <v>—</v>
+      </c>
+      <c r="P640" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B641" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C641" t="str">
+        <v>Stephin Pious</v>
+      </c>
+      <c r="D641" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E641" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F641" t="str">
+        <v>11:22 AM</v>
+      </c>
+      <c r="G641" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H641">
+        <v>0</v>
+      </c>
+      <c r="I641">
+        <v>0</v>
+      </c>
+      <c r="J641">
+        <v>0</v>
+      </c>
+      <c r="K641">
+        <v>0</v>
+      </c>
+      <c r="L641">
+        <v>0</v>
+      </c>
+      <c r="M641">
+        <v>0</v>
+      </c>
+      <c r="N641">
+        <v>0</v>
+      </c>
+      <c r="O641" t="str">
+        <v>Stephin Pious</v>
+      </c>
+      <c r="P641" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B642" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C642" t="str">
+        <v>Subodh Sha</v>
+      </c>
+      <c r="D642" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E642" t="str">
+        <v>—</v>
+      </c>
+      <c r="F642" t="str">
+        <v>—</v>
+      </c>
+      <c r="G642" t="str">
+        <v>—</v>
+      </c>
+      <c r="H642">
+        <v>0</v>
+      </c>
+      <c r="I642">
+        <v>0</v>
+      </c>
+      <c r="J642">
+        <v>0</v>
+      </c>
+      <c r="K642">
+        <v>0</v>
+      </c>
+      <c r="L642">
+        <v>0</v>
+      </c>
+      <c r="M642">
+        <v>0</v>
+      </c>
+      <c r="N642">
+        <v>0</v>
+      </c>
+      <c r="O642" t="str">
+        <v>—</v>
+      </c>
+      <c r="P642" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B643" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C643" t="str">
+        <v>Sukanto Mishal</v>
+      </c>
+      <c r="D643" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E643" t="str">
+        <v>—</v>
+      </c>
+      <c r="F643" t="str">
+        <v>—</v>
+      </c>
+      <c r="G643" t="str">
+        <v>—</v>
+      </c>
+      <c r="H643">
+        <v>0</v>
+      </c>
+      <c r="I643">
+        <v>0</v>
+      </c>
+      <c r="J643">
+        <v>0</v>
+      </c>
+      <c r="K643">
+        <v>0</v>
+      </c>
+      <c r="L643">
+        <v>0</v>
+      </c>
+      <c r="M643">
+        <v>0</v>
+      </c>
+      <c r="N643">
+        <v>0</v>
+      </c>
+      <c r="O643" t="str">
+        <v>—</v>
+      </c>
+      <c r="P643" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B644" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C644" t="str">
+        <v>Sumesh B</v>
+      </c>
+      <c r="D644" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E644" t="str">
+        <v>—</v>
+      </c>
+      <c r="F644" t="str">
+        <v>—</v>
+      </c>
+      <c r="G644" t="str">
+        <v>—</v>
+      </c>
+      <c r="H644">
+        <v>0</v>
+      </c>
+      <c r="I644">
+        <v>0</v>
+      </c>
+      <c r="J644">
+        <v>0</v>
+      </c>
+      <c r="K644">
+        <v>0</v>
+      </c>
+      <c r="L644">
+        <v>0</v>
+      </c>
+      <c r="M644">
+        <v>0</v>
+      </c>
+      <c r="N644">
+        <v>0</v>
+      </c>
+      <c r="O644" t="str">
+        <v>—</v>
+      </c>
+      <c r="P644" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B645" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C645" t="str">
+        <v>Sunil Aliyar</v>
+      </c>
+      <c r="D645" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E645" t="str">
+        <v>—</v>
+      </c>
+      <c r="F645" t="str">
+        <v>—</v>
+      </c>
+      <c r="G645" t="str">
+        <v>—</v>
+      </c>
+      <c r="H645">
+        <v>0</v>
+      </c>
+      <c r="I645">
+        <v>0</v>
+      </c>
+      <c r="J645">
+        <v>0</v>
+      </c>
+      <c r="K645">
+        <v>0</v>
+      </c>
+      <c r="L645">
+        <v>0</v>
+      </c>
+      <c r="M645">
+        <v>0</v>
+      </c>
+      <c r="N645">
+        <v>0</v>
+      </c>
+      <c r="O645" t="str">
+        <v>—</v>
+      </c>
+      <c r="P645" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B646" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C646" t="str">
+        <v>Sunil Rana</v>
+      </c>
+      <c r="D646" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E646" t="str">
+        <v>—</v>
+      </c>
+      <c r="F646" t="str">
+        <v>—</v>
+      </c>
+      <c r="G646" t="str">
+        <v>—</v>
+      </c>
+      <c r="H646">
+        <v>0</v>
+      </c>
+      <c r="I646">
+        <v>0</v>
+      </c>
+      <c r="J646">
+        <v>0</v>
+      </c>
+      <c r="K646">
+        <v>0</v>
+      </c>
+      <c r="L646">
+        <v>0</v>
+      </c>
+      <c r="M646">
+        <v>0</v>
+      </c>
+      <c r="N646">
+        <v>0</v>
+      </c>
+      <c r="O646" t="str">
+        <v>—</v>
+      </c>
+      <c r="P646" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B647" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C647" t="str">
+        <v>Sunil. C. M</v>
+      </c>
+      <c r="D647" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E647" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F647" t="str">
+        <v>11:22 AM</v>
+      </c>
+      <c r="G647" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H647">
+        <v>0</v>
+      </c>
+      <c r="I647">
+        <v>0</v>
+      </c>
+      <c r="J647">
+        <v>0</v>
+      </c>
+      <c r="K647">
+        <v>0</v>
+      </c>
+      <c r="L647">
+        <v>0</v>
+      </c>
+      <c r="M647">
+        <v>0</v>
+      </c>
+      <c r="N647">
+        <v>0</v>
+      </c>
+      <c r="O647" t="str">
+        <v>Sunil C M</v>
+      </c>
+      <c r="P647" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B648" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C648" t="str">
+        <v>Tufail Alam Danish</v>
+      </c>
+      <c r="D648" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E648" t="str">
+        <v>—</v>
+      </c>
+      <c r="F648" t="str">
+        <v>—</v>
+      </c>
+      <c r="G648" t="str">
+        <v>—</v>
+      </c>
+      <c r="H648">
+        <v>0</v>
+      </c>
+      <c r="I648">
+        <v>0</v>
+      </c>
+      <c r="J648">
+        <v>0</v>
+      </c>
+      <c r="K648">
+        <v>0</v>
+      </c>
+      <c r="L648">
+        <v>0</v>
+      </c>
+      <c r="M648">
+        <v>0</v>
+      </c>
+      <c r="N648">
+        <v>0</v>
+      </c>
+      <c r="O648" t="str">
+        <v>—</v>
+      </c>
+      <c r="P648" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="B649" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="C649" t="str">
+        <v>Vijesh A V</v>
+      </c>
+      <c r="D649" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E649" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F649" t="str">
+        <v>11:22 AM</v>
+      </c>
+      <c r="G649" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H649">
+        <v>0</v>
+      </c>
+      <c r="I649">
+        <v>0</v>
+      </c>
+      <c r="J649">
+        <v>0</v>
+      </c>
+      <c r="K649">
+        <v>0</v>
+      </c>
+      <c r="L649">
+        <v>0</v>
+      </c>
+      <c r="M649">
+        <v>0</v>
+      </c>
+      <c r="N649">
+        <v>0</v>
+      </c>
+      <c r="O649" t="str">
+        <v>Vijesh A V</v>
+      </c>
+      <c r="P649" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P577"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P649"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Support custom WhatsApp group names and monitoring of multiple groups simultaneously
- server.js changes:
  * Removed the hardcoded override forcing settingsData.whatsappGroupName to 'ATTENDANCE'.
  * Handled comma-separated lists of group names in settings save and raw message socket broadcasts.

- whatsapp.js changes:
  * Modified processMessage to match JIDs and names against comma-separated lists of target group JIDs/names.
  * Auto-heals missing group JIDs by appending newly matched group IDs to the settings.
  * Enhanced runStartupRoutines to resolve, load, map LIDs, and recover missed messages across all configured target groups.
  * Implemented resolveGroupIds to query and cache all JIDs matching target names, keeping resolveGroupId as a legacy wrapper.
  * Updated refreshChats and buildLidMapping to support scanning and processing multiple groups.
</commit_message>
<xml_diff>
--- a/Attendance_Payroll.xlsx
+++ b/Attendance_Payroll.xlsx
@@ -2178,7 +2178,7 @@
         <v>Mahin KJ</v>
       </c>
       <c r="D36" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E36" t="str">
         <v>INTEREXT OFFICE</v>
@@ -2187,10 +2187,10 @@
         <v>07:30 PM</v>
       </c>
       <c r="G36" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H36">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I36">
         <v>0</v>
@@ -2208,10 +2208,10 @@
         <v>0</v>
       </c>
       <c r="N36">
-        <v>0</v>
+        <v>389.43</v>
       </c>
       <c r="O36" t="str">
-        <v>7.30pm</v>
+        <v>7.30pm | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P36" t="str">
         <v/>
@@ -2628,7 +2628,7 @@
         <v>Rahul Das</v>
       </c>
       <c r="D45" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E45" t="str">
         <v>INTEREXT OFFICE</v>
@@ -2637,10 +2637,10 @@
         <v>07:00 PM</v>
       </c>
       <c r="G45" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H45">
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="I45">
         <v>0</v>
@@ -2658,10 +2658,10 @@
         <v>0</v>
       </c>
       <c r="N45">
-        <v>0</v>
+        <v>370.19</v>
       </c>
       <c r="O45" t="str">
-        <v>7:00pm</v>
+        <v>7:00pm | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P45" t="str">
         <v/>
@@ -4078,7 +4078,7 @@
         <v>Sunil Aliyar</v>
       </c>
       <c r="D74" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E74" t="str">
         <v>INTEREXT OFFICE</v>
@@ -4087,10 +4087,10 @@
         <v>07:04 PM</v>
       </c>
       <c r="G74" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H74">
-        <v>0</v>
+        <v>3.42</v>
       </c>
       <c r="I74">
         <v>0</v>
@@ -4108,10 +4108,10 @@
         <v>1</v>
       </c>
       <c r="N74">
-        <v>0</v>
+        <v>577.13</v>
       </c>
       <c r="O74" t="str">
-        <v xml:space="preserve">Sunil aliyar, Cavili choondy, </v>
+        <v>Sunil aliyar, Cavili choondy,  | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P74" t="str">
         <v/>
@@ -5028,7 +5028,7 @@
         <v>Anil Rana</v>
       </c>
       <c r="D93" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E93" t="str">
         <v>INTEREXT OFFICE</v>
@@ -5037,10 +5037,10 @@
         <v>08:14 PM</v>
       </c>
       <c r="G93" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H93">
-        <v>0</v>
+        <v>2.25</v>
       </c>
       <c r="I93">
         <v>0</v>
@@ -5058,10 +5058,10 @@
         <v>1</v>
       </c>
       <c r="N93">
-        <v>0</v>
+        <v>295.31</v>
       </c>
       <c r="O93" t="str">
-        <v xml:space="preserve">Anil rana, Cavili  choondy, </v>
+        <v>Anil rana, Cavili  choondy,  | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P93" t="str">
         <v/>
@@ -6028,7 +6028,7 @@
         <v>Mahin KJ</v>
       </c>
       <c r="D113" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E113" t="str">
         <v>INTEREXT OFFICE</v>
@@ -6037,10 +6037,10 @@
         <v>07:00 PM</v>
       </c>
       <c r="G113" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H113">
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="I113">
         <v>0</v>
@@ -6058,10 +6058,10 @@
         <v>0</v>
       </c>
       <c r="N113">
-        <v>0</v>
+        <v>454.34</v>
       </c>
       <c r="O113" t="str">
-        <v>7.00pm</v>
+        <v>7.00pm | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P113" t="str">
         <v/>
@@ -6478,7 +6478,7 @@
         <v>Rahul Das</v>
       </c>
       <c r="D122" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E122" t="str">
         <v>INTEREXT OFFICE</v>
@@ -6487,10 +6487,10 @@
         <v>08:40 PM</v>
       </c>
       <c r="G122" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H122">
-        <v>0</v>
+        <v>1.83</v>
       </c>
       <c r="I122">
         <v>0</v>
@@ -6508,10 +6508,10 @@
         <v>0</v>
       </c>
       <c r="N122">
-        <v>0</v>
+        <v>193.56</v>
       </c>
       <c r="O122" t="str">
-        <v>8:40pm</v>
+        <v>8:40pm | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P122" t="str">
         <v/>
@@ -7678,7 +7678,7 @@
         <v>Sreeraj V S</v>
       </c>
       <c r="D146" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E146" t="str">
         <v>INTEREXT OFFICE</v>
@@ -7687,10 +7687,10 @@
         <v>08:14 PM</v>
       </c>
       <c r="G146" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H146">
-        <v>0</v>
+        <v>2.25</v>
       </c>
       <c r="I146">
         <v>0</v>
@@ -7708,10 +7708,10 @@
         <v>1</v>
       </c>
       <c r="N146">
-        <v>0</v>
+        <v>295.31</v>
       </c>
       <c r="O146" t="str">
-        <v xml:space="preserve">Sreeraj, Cavili  choondy, </v>
+        <v>Sreeraj, Cavili  choondy,  | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P146" t="str">
         <v/>
@@ -7778,7 +7778,7 @@
         <v>Subodh Sha</v>
       </c>
       <c r="D148" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E148" t="str">
         <v>INTEREXT OFFICE</v>
@@ -7787,10 +7787,10 @@
         <v>08:14 PM</v>
       </c>
       <c r="G148" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H148">
-        <v>0</v>
+        <v>2.25</v>
       </c>
       <c r="I148">
         <v>0</v>
@@ -7808,10 +7808,10 @@
         <v>1</v>
       </c>
       <c r="N148">
-        <v>0</v>
+        <v>281.25</v>
       </c>
       <c r="O148" t="str">
-        <v xml:space="preserve">Subodsha, Cavili  choondy, </v>
+        <v>Subodsha, Cavili  choondy,  | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P148" t="str">
         <v/>
@@ -7928,7 +7928,7 @@
         <v>Sunil Aliyar</v>
       </c>
       <c r="D151" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E151" t="str">
         <v>INTEREXT OFFICE</v>
@@ -7937,10 +7937,10 @@
         <v>08:14 PM</v>
       </c>
       <c r="G151" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H151">
-        <v>0</v>
+        <v>2.25</v>
       </c>
       <c r="I151">
         <v>0</v>
@@ -7958,10 +7958,10 @@
         <v>1</v>
       </c>
       <c r="N151">
-        <v>0</v>
+        <v>379.69</v>
       </c>
       <c r="O151" t="str">
-        <v xml:space="preserve">Sunil aliyar, Cavili  choondy, </v>
+        <v>Sunil aliyar, Cavili  choondy,  | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P151" t="str">
         <v/>
@@ -8878,7 +8878,7 @@
         <v>Anil Rana</v>
       </c>
       <c r="D170" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E170" t="str">
         <v>INTEREXT OFFICE</v>
@@ -8887,10 +8887,10 @@
         <v>07:44 PM</v>
       </c>
       <c r="G170" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H170">
-        <v>0</v>
+        <v>2.75</v>
       </c>
       <c r="I170">
         <v>0</v>
@@ -8908,10 +8908,10 @@
         <v>1</v>
       </c>
       <c r="N170">
-        <v>0</v>
+        <v>360.94</v>
       </c>
       <c r="O170" t="str">
-        <v xml:space="preserve">Anil rana, Cavili choondy, </v>
+        <v>Anil rana, Cavili choondy,  | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P170" t="str">
         <v/>
@@ -9884,7 +9884,7 @@
         <v>INTEREXT OFFICE</v>
       </c>
       <c r="F190" t="str">
-        <v>09:30 PM</v>
+        <v>07:28 AM</v>
       </c>
       <c r="G190" t="str">
         <v>Currently Checked-In</v>
@@ -9911,7 +9911,7 @@
         <v>0</v>
       </c>
       <c r="O190" t="str">
-        <v>9.30pm</v>
+        <v>7.28am</v>
       </c>
       <c r="P190" t="str">
         <v/>
@@ -10328,7 +10328,7 @@
         <v>Rahul Das</v>
       </c>
       <c r="D199" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E199" t="str">
         <v>INTEREXT OFFICE</v>
@@ -10337,10 +10337,10 @@
         <v>07:00 PM</v>
       </c>
       <c r="G199" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H199">
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="I199">
         <v>0</v>
@@ -10358,10 +10358,10 @@
         <v>0</v>
       </c>
       <c r="N199">
-        <v>0</v>
+        <v>370.19</v>
       </c>
       <c r="O199" t="str">
-        <v>7:00pm</v>
+        <v>7:00pm | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P199" t="str">
         <v/>
@@ -10578,7 +10578,7 @@
         <v>Raju Rana</v>
       </c>
       <c r="D204" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E204" t="str">
         <v>INTEREXT OFFICE</v>
@@ -10587,7 +10587,7 @@
         <v>10:54 PM</v>
       </c>
       <c r="G204" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H204">
         <v>0</v>
@@ -10611,7 +10611,7 @@
         <v>0</v>
       </c>
       <c r="O204" t="str">
-        <v>Ratheesh ks. Akash, Raju rana, Rajkumar, Mahin Driver</v>
+        <v>Ratheesh ks. Akash, Raju rana, Rajkumar, Mahin Driver | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P204" t="str">
         <v/>
@@ -11628,7 +11628,7 @@
         <v>Subodh Sha</v>
       </c>
       <c r="D225" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E225" t="str">
         <v>INTEREXT OFFICE</v>
@@ -11637,10 +11637,10 @@
         <v>07:44 PM</v>
       </c>
       <c r="G225" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H225">
-        <v>0</v>
+        <v>2.75</v>
       </c>
       <c r="I225">
         <v>0</v>
@@ -11658,10 +11658,10 @@
         <v>1</v>
       </c>
       <c r="N225">
-        <v>0</v>
+        <v>343.75</v>
       </c>
       <c r="O225" t="str">
-        <v xml:space="preserve">Subodsha, Cavili choondy, </v>
+        <v>Subodsha, Cavili choondy,  | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P225" t="str">
         <v/>
@@ -11778,7 +11778,7 @@
         <v>Sunil Aliyar</v>
       </c>
       <c r="D228" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E228" t="str">
         <v>INTEREXT OFFICE</v>
@@ -11787,10 +11787,10 @@
         <v>07:44 PM</v>
       </c>
       <c r="G228" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H228">
-        <v>0</v>
+        <v>2.75</v>
       </c>
       <c r="I228">
         <v>0</v>
@@ -11808,10 +11808,10 @@
         <v>1</v>
       </c>
       <c r="N228">
-        <v>0</v>
+        <v>464.06</v>
       </c>
       <c r="O228" t="str">
-        <v xml:space="preserve">Sunil aliyar, Cavili choondy, </v>
+        <v>Sunil aliyar, Cavili choondy,  | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P228" t="str">
         <v/>
@@ -12682,7 +12682,7 @@
         <v>Aneesh Ahammed</v>
       </c>
       <c r="D246" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E246" t="str">
         <v>INTEREXT OFFICE</v>
@@ -12691,13 +12691,13 @@
         <v>07:00 AM</v>
       </c>
       <c r="G246" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H246">
-        <v>0</v>
+        <v>15.5</v>
       </c>
       <c r="I246">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J246">
         <v>0</v>
@@ -12706,16 +12706,16 @@
         <v>0</v>
       </c>
       <c r="L246">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="M246">
         <v>0</v>
       </c>
       <c r="N246">
-        <v>0</v>
+        <v>1870</v>
       </c>
       <c r="O246" t="str">
-        <v>7:pm</v>
+        <v>7:pm | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P246" t="str">
         <v/>
@@ -12732,7 +12732,7 @@
         <v>Anil Rana</v>
       </c>
       <c r="D247" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E247" t="str">
         <v>INTEREXT OFFICE</v>
@@ -12741,10 +12741,10 @@
         <v>08:36 PM</v>
       </c>
       <c r="G247" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H247">
-        <v>0</v>
+        <v>1.9</v>
       </c>
       <c r="I247">
         <v>0</v>
@@ -12762,10 +12762,10 @@
         <v>1</v>
       </c>
       <c r="N247">
-        <v>0</v>
+        <v>249.38</v>
       </c>
       <c r="O247" t="str">
-        <v xml:space="preserve">Anil rana, Cavili choondy, </v>
+        <v>Anil rana, Cavili choondy,  | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P247" t="str">
         <v/>
@@ -14182,7 +14182,7 @@
         <v>Rahul Das</v>
       </c>
       <c r="D276" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E276" t="str">
         <v>INTEREXT OFFICE</v>
@@ -14191,10 +14191,10 @@
         <v>07:00 PM</v>
       </c>
       <c r="G276" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H276">
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="I276">
         <v>0</v>
@@ -14212,10 +14212,10 @@
         <v>0</v>
       </c>
       <c r="N276">
-        <v>0</v>
+        <v>370.19</v>
       </c>
       <c r="O276" t="str">
-        <v>7:00pm</v>
+        <v>7:00pm | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P276" t="str">
         <v/>
@@ -15232,7 +15232,7 @@
         <v>Sona Francis</v>
       </c>
       <c r="D297" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E297" t="str">
         <v>INTEREXT OFFICE</v>
@@ -15241,13 +15241,13 @@
         <v>09:30 AM</v>
       </c>
       <c r="G297" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H297">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="I297">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J297">
         <v>0</v>
@@ -15262,10 +15262,10 @@
         <v>0</v>
       </c>
       <c r="N297">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="O297" t="str">
-        <v>I'm half hour late to reach office today hospital case</v>
+        <v>I'm half hour late to reach office today hospital case | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P297" t="str">
         <v/>
@@ -15482,7 +15482,7 @@
         <v>Subodh Sha</v>
       </c>
       <c r="D302" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E302" t="str">
         <v>INTEREXT OFFICE</v>
@@ -15491,10 +15491,10 @@
         <v>08:36 PM</v>
       </c>
       <c r="G302" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H302">
-        <v>0</v>
+        <v>1.9</v>
       </c>
       <c r="I302">
         <v>0</v>
@@ -15512,10 +15512,10 @@
         <v>1</v>
       </c>
       <c r="N302">
-        <v>0</v>
+        <v>237.5</v>
       </c>
       <c r="O302" t="str">
-        <v xml:space="preserve">Subodsha, Cavili choondy, </v>
+        <v>Subodsha, Cavili choondy,  | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P302" t="str">
         <v/>
@@ -16532,7 +16532,7 @@
         <v>Aneesh Ahammed</v>
       </c>
       <c r="D323" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E323" t="str">
         <v>INTEREXT OFFICE</v>
@@ -16541,13 +16541,13 @@
         <v>09:22 AM</v>
       </c>
       <c r="G323" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H323">
-        <v>0</v>
+        <v>13.13</v>
       </c>
       <c r="I323">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J323">
         <v>0</v>
@@ -16556,16 +16556,16 @@
         <v>0</v>
       </c>
       <c r="L323">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="M323">
         <v>0</v>
       </c>
       <c r="N323">
-        <v>0</v>
+        <v>1650</v>
       </c>
       <c r="O323" t="str">
-        <v>9:22</v>
+        <v>9:22 | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P323" t="str">
         <v/>
@@ -16582,7 +16582,7 @@
         <v>Anil Rana</v>
       </c>
       <c r="D324" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E324" t="str">
         <v>INTEREXT OFFICE</v>
@@ -16591,10 +16591,10 @@
         <v>08:11 PM</v>
       </c>
       <c r="G324" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H324">
-        <v>0</v>
+        <v>2.3</v>
       </c>
       <c r="I324">
         <v>0</v>
@@ -16612,10 +16612,10 @@
         <v>1</v>
       </c>
       <c r="N324">
-        <v>0</v>
+        <v>301.88</v>
       </c>
       <c r="O324" t="str">
-        <v xml:space="preserve">Anil rana, Cavili choondy, </v>
+        <v>Anil rana, Cavili choondy,  | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P324" t="str">
         <v/>
@@ -17332,7 +17332,7 @@
         <v>James TM</v>
       </c>
       <c r="D339" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E339" t="str">
         <v>INTEREXT OFFICE</v>
@@ -17341,13 +17341,13 @@
         <v>09:30 AM</v>
       </c>
       <c r="G339" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H339">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="I339">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J339">
         <v>0</v>
@@ -17356,16 +17356,16 @@
         <v>0</v>
       </c>
       <c r="L339">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="M339">
         <v>0</v>
       </c>
       <c r="N339">
-        <v>0</v>
+        <v>1442.31</v>
       </c>
       <c r="O339" t="str">
-        <v>Iam half an hour late</v>
+        <v>Iam half an hour late | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P339" t="str">
         <v/>
@@ -17582,7 +17582,7 @@
         <v>Mahin KJ</v>
       </c>
       <c r="D344" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E344" t="str">
         <v>INTEREXT OFFICE</v>
@@ -17591,10 +17591,10 @@
         <v>07:00 PM</v>
       </c>
       <c r="G344" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H344">
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="I344">
         <v>0</v>
@@ -17612,10 +17612,10 @@
         <v>0</v>
       </c>
       <c r="N344">
-        <v>0</v>
+        <v>454.34</v>
       </c>
       <c r="O344" t="str">
-        <v>7.00pm</v>
+        <v>7.00pm | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P344" t="str">
         <v/>
@@ -17932,7 +17932,7 @@
         <v>PRASANTH E.M</v>
       </c>
       <c r="D351" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E351" t="str">
         <v>INTEREXT OFFICE</v>
@@ -17941,10 +17941,10 @@
         <v>08:30 PM</v>
       </c>
       <c r="G351" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H351">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I351">
         <v>0</v>
@@ -17962,10 +17962,10 @@
         <v>0</v>
       </c>
       <c r="N351">
-        <v>0</v>
+        <v>298.08</v>
       </c>
       <c r="O351" t="str">
-        <v>8.30 pm</v>
+        <v>8.30 pm | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P351" t="str">
         <v/>
@@ -19332,7 +19332,7 @@
         <v>Subodh Sha</v>
       </c>
       <c r="D379" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E379" t="str">
         <v>INTEREXT OFFICE</v>
@@ -19341,10 +19341,10 @@
         <v>08:11 PM</v>
       </c>
       <c r="G379" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H379">
-        <v>0</v>
+        <v>2.3</v>
       </c>
       <c r="I379">
         <v>0</v>
@@ -19362,10 +19362,10 @@
         <v>1</v>
       </c>
       <c r="N379">
-        <v>0</v>
+        <v>287.5</v>
       </c>
       <c r="O379" t="str">
-        <v xml:space="preserve">Subodsha, Cavili choondy, </v>
+        <v>Subodsha, Cavili choondy,  | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P379" t="str">
         <v/>
@@ -19482,7 +19482,7 @@
         <v>Sunil Aliyar</v>
       </c>
       <c r="D382" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E382" t="str">
         <v>INTEREXT OFFICE</v>
@@ -19491,10 +19491,10 @@
         <v>08:11 PM</v>
       </c>
       <c r="G382" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H382">
-        <v>0</v>
+        <v>2.3</v>
       </c>
       <c r="I382">
         <v>0</v>
@@ -19512,10 +19512,10 @@
         <v>1</v>
       </c>
       <c r="N382">
-        <v>0</v>
+        <v>388.12</v>
       </c>
       <c r="O382" t="str">
-        <v xml:space="preserve">Sunil aliyar, Cavili choondy, </v>
+        <v>Sunil aliyar, Cavili choondy,  | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P382" t="str">
         <v/>
@@ -20282,7 +20282,7 @@
         <v>ANADHU SUNIL</v>
       </c>
       <c r="D398" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E398" t="str">
         <v>INTEREXT OFFICE</v>
@@ -20291,13 +20291,13 @@
         <v>12:08 PM</v>
       </c>
       <c r="G398" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H398">
-        <v>0</v>
+        <v>10.35</v>
       </c>
       <c r="I398">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J398">
         <v>0</v>
@@ -20312,10 +20312,10 @@
         <v>0</v>
       </c>
       <c r="N398">
-        <v>0</v>
+        <v>961.54</v>
       </c>
       <c r="O398" t="str">
-        <v xml:space="preserve">Anadhu, (Inter ext office), </v>
+        <v>Anadhu, (Inter ext office),  | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P398" t="str">
         <v/>
@@ -20982,7 +20982,7 @@
         <v>GEORGE THOMAS</v>
       </c>
       <c r="D412" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E412" t="str">
         <v>INTEREXT OFFICE</v>
@@ -20991,13 +20991,13 @@
         <v>06:00 AM</v>
       </c>
       <c r="G412" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H412">
-        <v>0</v>
+        <v>16.5</v>
       </c>
       <c r="I412">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J412">
         <v>0</v>
@@ -21012,10 +21012,10 @@
         <v>0</v>
       </c>
       <c r="N412">
-        <v>0</v>
+        <v>1300</v>
       </c>
       <c r="O412" t="str">
-        <v>I am 30 mints late to reach office..</v>
+        <v>I am 30 mints late to reach office.. | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P412" t="str">
         <v/>
@@ -21432,7 +21432,7 @@
         <v>Mahin KJ</v>
       </c>
       <c r="D421" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E421" t="str">
         <v>INTEREXT OFFICE</v>
@@ -21441,13 +21441,13 @@
         <v>02:00 PM</v>
       </c>
       <c r="G421" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H421">
-        <v>0</v>
+        <v>8.5</v>
       </c>
       <c r="I421">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J421">
         <v>0</v>
@@ -21462,10 +21462,10 @@
         <v>0</v>
       </c>
       <c r="N421">
-        <v>0</v>
+        <v>1038.46</v>
       </c>
       <c r="O421" t="str">
-        <v>2.00pm</v>
+        <v>2.00pm | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P421" t="str">
         <v/>
@@ -22282,7 +22282,7 @@
         <v>Ratheesh K S</v>
       </c>
       <c r="D438" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E438" t="str">
         <v>INTEREXT OFFICE</v>
@@ -22291,13 +22291,13 @@
         <v>08:40 AM</v>
       </c>
       <c r="G438" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H438">
-        <v>0</v>
+        <v>13.82</v>
       </c>
       <c r="I438">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J438">
         <v>0</v>
@@ -22306,16 +22306,16 @@
         <v>0</v>
       </c>
       <c r="L438">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="M438">
         <v>0</v>
       </c>
       <c r="N438">
-        <v>0</v>
+        <v>2192.31</v>
       </c>
       <c r="O438" t="str">
-        <v>Ratheesh ks, Anish driver</v>
+        <v>Ratheesh ks, Anish driver | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P438" t="str">
         <v/>
@@ -23132,7 +23132,7 @@
         <v>Stephin Pious</v>
       </c>
       <c r="D455" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E455" t="str">
         <v>INTEREXT OFFICE</v>
@@ -23141,13 +23141,13 @@
         <v>12:08 PM</v>
       </c>
       <c r="G455" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H455">
-        <v>0</v>
+        <v>10.35</v>
       </c>
       <c r="I455">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J455">
         <v>0</v>
@@ -23162,10 +23162,10 @@
         <v>0</v>
       </c>
       <c r="N455">
-        <v>0</v>
+        <v>961.54</v>
       </c>
       <c r="O455" t="str">
-        <v xml:space="preserve">(Sathyan kanjar -stephan, (Inter ext office), </v>
+        <v>(Sathyan kanjar -stephan, (Inter ext office),  | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P455" t="str">
         <v/>
@@ -23282,7 +23282,7 @@
         <v>Sumesh B</v>
       </c>
       <c r="D458" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E458" t="str">
         <v>INTEREXT OFFICE</v>
@@ -23291,13 +23291,13 @@
         <v>12:08 PM</v>
       </c>
       <c r="G458" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H458">
-        <v>0</v>
+        <v>10.35</v>
       </c>
       <c r="I458">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J458">
         <v>0</v>
@@ -23306,16 +23306,16 @@
         <v>0</v>
       </c>
       <c r="L458">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M458">
         <v>0</v>
       </c>
       <c r="N458">
-        <v>0</v>
+        <v>1560</v>
       </c>
       <c r="O458" t="str">
-        <v xml:space="preserve">Sumesh, (Inter ext office), </v>
+        <v>Sumesh, (Inter ext office),  | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P458" t="str">
         <v/>
@@ -24282,7 +24282,7 @@
         <v>Anil Rana</v>
       </c>
       <c r="D478" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E478" t="str">
         <v>INTEREXT OFFICE</v>
@@ -24291,10 +24291,10 @@
         <v>07:32 PM</v>
       </c>
       <c r="G478" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H478">
-        <v>0</v>
+        <v>2.97</v>
       </c>
       <c r="I478">
         <v>0</v>
@@ -24312,10 +24312,10 @@
         <v>1</v>
       </c>
       <c r="N478">
-        <v>0</v>
+        <v>389.81</v>
       </c>
       <c r="O478" t="str">
-        <v xml:space="preserve">Anil rana, Cavili choondy, </v>
+        <v>Anil rana, Cavili choondy,  | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P478" t="str">
         <v/>
@@ -27032,7 +27032,7 @@
         <v>Subodh Sha</v>
       </c>
       <c r="D533" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E533" t="str">
         <v>INTEREXT OFFICE</v>
@@ -27041,10 +27041,10 @@
         <v>07:32 PM</v>
       </c>
       <c r="G533" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H533">
-        <v>0</v>
+        <v>2.97</v>
       </c>
       <c r="I533">
         <v>0</v>
@@ -27062,10 +27062,10 @@
         <v>1</v>
       </c>
       <c r="N533">
-        <v>0</v>
+        <v>371.25</v>
       </c>
       <c r="O533" t="str">
-        <v xml:space="preserve">Subodsha, Cavili choondy, </v>
+        <v>Subodsha, Cavili choondy,  | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P533" t="str">
         <v/>
@@ -27734,7 +27734,7 @@
         <v>Akash</v>
       </c>
       <c r="D547" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E547" t="str">
         <v>INTEREXT OFFICE</v>
@@ -27743,19 +27743,19 @@
         <v>02:38 PM</v>
       </c>
       <c r="G547" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H547">
-        <v>0</v>
+        <v>7.85</v>
       </c>
       <c r="I547">
         <v>0</v>
       </c>
       <c r="J547">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K547">
-        <v>0</v>
+        <v>3.85</v>
       </c>
       <c r="L547">
         <v>0</v>
@@ -27764,10 +27764,10 @@
         <v>0</v>
       </c>
       <c r="N547">
-        <v>0</v>
+        <v>1070.53</v>
       </c>
       <c r="O547" t="str">
-        <v>Okay 👍</v>
+        <v>Okay 👍 | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P547" t="str">
         <v/>
@@ -28084,7 +28084,7 @@
         <v>Aneesh Ahammed</v>
       </c>
       <c r="D554" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E554" t="str">
         <v>INTEREXT OFFICE</v>
@@ -28093,10 +28093,10 @@
         <v>08:10 PM</v>
       </c>
       <c r="G554" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H554">
-        <v>0</v>
+        <v>2.33</v>
       </c>
       <c r="I554">
         <v>0</v>
@@ -28114,10 +28114,10 @@
         <v>0</v>
       </c>
       <c r="N554">
-        <v>0</v>
+        <v>320.38</v>
       </c>
       <c r="O554" t="str">
-        <v>8:10pm</v>
+        <v>8:10pm | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P554" t="str">
         <v/>
@@ -28884,7 +28884,7 @@
         <v>James TM</v>
       </c>
       <c r="D570" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E570" t="str">
         <v>INTEREXT OFFICE</v>
@@ -28893,13 +28893,13 @@
         <v>09:30 AM</v>
       </c>
       <c r="G570" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H570">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="I570">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J570">
         <v>0</v>
@@ -28908,16 +28908,16 @@
         <v>0</v>
       </c>
       <c r="L570">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="M570">
         <v>0</v>
       </c>
       <c r="N570">
-        <v>0</v>
+        <v>1442.31</v>
       </c>
       <c r="O570" t="str">
-        <v>Iam half an hour late</v>
+        <v>Iam half an hour late | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P570" t="str">
         <v/>
@@ -29134,7 +29134,7 @@
         <v>Mahin KJ</v>
       </c>
       <c r="D575" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E575" t="str">
         <v>INTEREXT OFFICE</v>
@@ -29143,10 +29143,10 @@
         <v>07:00 PM</v>
       </c>
       <c r="G575" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H575">
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="I575">
         <v>0</v>
@@ -29164,10 +29164,10 @@
         <v>0</v>
       </c>
       <c r="N575">
-        <v>0</v>
+        <v>454.34</v>
       </c>
       <c r="O575" t="str">
-        <v>7.00pm</v>
+        <v>7.00pm | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P575" t="str">
         <v/>
@@ -29484,7 +29484,7 @@
         <v>PRASANTH E.M</v>
       </c>
       <c r="D582" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E582" t="str">
         <v>INTEREXT OFFICE</v>
@@ -29493,13 +29493,13 @@
         <v>12:53 PM</v>
       </c>
       <c r="G582" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H582">
-        <v>0</v>
+        <v>9.6</v>
       </c>
       <c r="I582">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J582">
         <v>0</v>
@@ -29514,10 +29514,10 @@
         <v>0</v>
       </c>
       <c r="N582">
-        <v>0</v>
+        <v>1192.31</v>
       </c>
       <c r="O582" t="str">
-        <v>👍</v>
+        <v>👍 | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P582" t="str">
         <v/>
@@ -29584,7 +29584,7 @@
         <v>Rahul Das</v>
       </c>
       <c r="D584" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E584" t="str">
         <v>INTEREXT OFFICE</v>
@@ -29593,10 +29593,10 @@
         <v>07:00 PM</v>
       </c>
       <c r="G584" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H584">
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="I584">
         <v>0</v>
@@ -29614,10 +29614,10 @@
         <v>0</v>
       </c>
       <c r="N584">
-        <v>0</v>
+        <v>370.19</v>
       </c>
       <c r="O584" t="str">
-        <v>7:00pm</v>
+        <v>7:00pm | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P584" t="str">
         <v/>
@@ -30384,7 +30384,7 @@
         <v>SHAHANA JABBAR</v>
       </c>
       <c r="D600" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E600" t="str">
         <v>INTEREXT OFFICE</v>
@@ -30393,10 +30393,10 @@
         <v>08:00 PM</v>
       </c>
       <c r="G600" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H600">
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="I600">
         <v>0</v>
@@ -30414,10 +30414,10 @@
         <v>0</v>
       </c>
       <c r="N600">
-        <v>0</v>
+        <v>312.5</v>
       </c>
       <c r="O600" t="str">
-        <v>I am on 20 mnts late morning</v>
+        <v>I am on 20 mnts late morning | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P600" t="str">
         <v/>
@@ -30534,7 +30534,7 @@
         <v>Siju Thomas</v>
       </c>
       <c r="D603" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E603" t="str">
         <v>INTEREXT OFFICE</v>
@@ -30543,16 +30543,16 @@
         <v>03:00 PM</v>
       </c>
       <c r="G603" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H603">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="I603">
         <v>0</v>
       </c>
       <c r="J603">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K603">
         <v>0</v>
@@ -30564,10 +30564,10 @@
         <v>0</v>
       </c>
       <c r="N603">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="O603" t="str">
-        <v>3.am Gokulam medical college Venjaramoodu</v>
+        <v>3.am Gokulam medical college Venjaramoodu | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P603" t="str">
         <v/>
@@ -30834,7 +30834,7 @@
         <v>Stephin Pious</v>
       </c>
       <c r="D609" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E609" t="str">
         <v>INTEREXT OFFICE</v>
@@ -30843,10 +30843,10 @@
         <v>07:00 PM</v>
       </c>
       <c r="G609" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H609">
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="I609">
         <v>0</v>
@@ -30864,10 +30864,10 @@
         <v>0</v>
       </c>
       <c r="N609">
-        <v>0</v>
+        <v>420.66</v>
       </c>
       <c r="O609" t="str">
-        <v>7 pm</v>
+        <v>7 pm | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P609" t="str">
         <v/>
@@ -31334,7 +31334,7 @@
         <v>Abhishek Shaji</v>
       </c>
       <c r="D619" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E619" t="str">
         <v>INTEREXT OFFICE</v>
@@ -31343,13 +31343,13 @@
         <v>11:22 AM</v>
       </c>
       <c r="G619" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H619">
-        <v>0</v>
+        <v>11.12</v>
       </c>
       <c r="I619">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J619">
         <v>0</v>
@@ -31364,10 +31364,10 @@
         <v>0</v>
       </c>
       <c r="N619">
-        <v>0</v>
+        <v>466.67</v>
       </c>
       <c r="O619" t="str">
-        <v>Abhishek Shaji</v>
+        <v>Abhishek Shaji | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P619" t="str">
         <v/>
@@ -31434,7 +31434,7 @@
         <v>AJEESH VIJAYAN</v>
       </c>
       <c r="D621" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E621" t="str">
         <v>INTEREXT OFFICE</v>
@@ -31443,13 +31443,13 @@
         <v>11:22 AM</v>
       </c>
       <c r="G621" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H621">
-        <v>0</v>
+        <v>11.12</v>
       </c>
       <c r="I621">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J621">
         <v>0</v>
@@ -31464,10 +31464,10 @@
         <v>0</v>
       </c>
       <c r="N621">
-        <v>0</v>
+        <v>1066.67</v>
       </c>
       <c r="O621" t="str">
-        <v>Ajeesh Vijayan</v>
+        <v>Ajeesh Vijayan | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P621" t="str">
         <v/>
@@ -31484,7 +31484,7 @@
         <v>Ajith Reghunath</v>
       </c>
       <c r="D622" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E622" t="str">
         <v>INTEREXT OFFICE</v>
@@ -31493,13 +31493,13 @@
         <v>11:22 AM</v>
       </c>
       <c r="G622" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H622">
-        <v>0</v>
+        <v>11.12</v>
       </c>
       <c r="I622">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J622">
         <v>0</v>
@@ -31514,10 +31514,10 @@
         <v>0</v>
       </c>
       <c r="N622">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="O622" t="str">
-        <v>Ajith Reghunath</v>
+        <v>Ajith Reghunath | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P622" t="str">
         <v/>
@@ -31584,7 +31584,7 @@
         <v>Akash</v>
       </c>
       <c r="D624" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E624" t="str">
         <v>INTEREXT OFFICE</v>
@@ -31593,13 +31593,13 @@
         <v>11:22 AM</v>
       </c>
       <c r="G624" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H624">
-        <v>0</v>
+        <v>11.12</v>
       </c>
       <c r="I624">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J624">
         <v>0</v>
@@ -31608,16 +31608,16 @@
         <v>0</v>
       </c>
       <c r="L624">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M624">
         <v>0</v>
       </c>
       <c r="N624">
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c r="O624" t="str">
-        <v>Akash Rana</v>
+        <v>Akash Rana | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P624" t="str">
         <v/>
@@ -31734,7 +31734,7 @@
         <v>Alex Gigi</v>
       </c>
       <c r="D627" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E627" t="str">
         <v>INTEREXT OFFICE</v>
@@ -31743,13 +31743,13 @@
         <v>11:22 AM</v>
       </c>
       <c r="G627" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H627">
-        <v>0</v>
+        <v>11.12</v>
       </c>
       <c r="I627">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J627">
         <v>0</v>
@@ -31758,16 +31758,16 @@
         <v>0</v>
       </c>
       <c r="L627">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M627">
         <v>0</v>
       </c>
       <c r="N627">
-        <v>0</v>
+        <v>845</v>
       </c>
       <c r="O627" t="str">
-        <v>Alex Gigi</v>
+        <v>Alex Gigi | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P627" t="str">
         <v/>
@@ -31784,7 +31784,7 @@
         <v>Alex Rajan</v>
       </c>
       <c r="D628" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E628" t="str">
         <v>INTEREXT OFFICE</v>
@@ -31793,13 +31793,13 @@
         <v>11:22 AM</v>
       </c>
       <c r="G628" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H628">
-        <v>0</v>
+        <v>11.12</v>
       </c>
       <c r="I628">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J628">
         <v>0</v>
@@ -31814,10 +31814,10 @@
         <v>0</v>
       </c>
       <c r="N628">
-        <v>0</v>
+        <v>666.67</v>
       </c>
       <c r="O628" t="str">
-        <v>Alex Rajan</v>
+        <v>Alex Rajan | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P628" t="str">
         <v/>
@@ -32034,7 +32034,7 @@
         <v>Anish Viswanathan</v>
       </c>
       <c r="D633" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E633" t="str">
         <v>INTEREXT OFFICE</v>
@@ -32043,13 +32043,13 @@
         <v>11:22 AM</v>
       </c>
       <c r="G633" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H633">
-        <v>0</v>
+        <v>11.12</v>
       </c>
       <c r="I633">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J633">
         <v>0</v>
@@ -32064,10 +32064,10 @@
         <v>0</v>
       </c>
       <c r="N633">
-        <v>0</v>
+        <v>846.15</v>
       </c>
       <c r="O633" t="str">
-        <v>Anish Viswanathan</v>
+        <v>Anish Viswanathan | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P633" t="str">
         <v/>
@@ -32234,7 +32234,7 @@
         <v>Arun P madhu</v>
       </c>
       <c r="D637" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E637" t="str">
         <v>INTEREXT OFFICE</v>
@@ -32243,13 +32243,13 @@
         <v>11:22 AM</v>
       </c>
       <c r="G637" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H637">
-        <v>0</v>
+        <v>11.12</v>
       </c>
       <c r="I637">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J637">
         <v>0</v>
@@ -32258,16 +32258,16 @@
         <v>0</v>
       </c>
       <c r="L637">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M637">
         <v>0</v>
       </c>
       <c r="N637">
-        <v>0</v>
+        <v>1690</v>
       </c>
       <c r="O637" t="str">
-        <v>Arun P Madhu</v>
+        <v>Arun P Madhu | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P637" t="str">
         <v/>
@@ -32284,7 +32284,7 @@
         <v>Bimal Rana</v>
       </c>
       <c r="D638" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E638" t="str">
         <v>INTEREXT OFFICE</v>
@@ -32293,13 +32293,13 @@
         <v>11:22 AM</v>
       </c>
       <c r="G638" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H638">
-        <v>0</v>
+        <v>11.12</v>
       </c>
       <c r="I638">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J638">
         <v>0</v>
@@ -32308,16 +32308,16 @@
         <v>0</v>
       </c>
       <c r="L638">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M638">
         <v>0</v>
       </c>
       <c r="N638">
-        <v>0</v>
+        <v>750</v>
       </c>
       <c r="O638" t="str">
-        <v>Bimal Rana</v>
+        <v>Bimal Rana | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P638" t="str">
         <v/>
@@ -32334,7 +32334,7 @@
         <v>BINDHU JOSE</v>
       </c>
       <c r="D639" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E639" t="str">
         <v>INTEREXT OFFICE</v>
@@ -32343,13 +32343,13 @@
         <v>11:22 AM</v>
       </c>
       <c r="G639" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H639">
-        <v>0</v>
+        <v>11.12</v>
       </c>
       <c r="I639">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J639">
         <v>0</v>
@@ -32364,10 +32364,10 @@
         <v>0</v>
       </c>
       <c r="N639">
-        <v>0</v>
+        <v>700</v>
       </c>
       <c r="O639" t="str">
-        <v>Bindhu Jose</v>
+        <v>Bindhu Jose | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P639" t="str">
         <v/>
@@ -32434,7 +32434,7 @@
         <v>Devadas E K</v>
       </c>
       <c r="D641" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E641" t="str">
         <v>INTEREXT OFFICE</v>
@@ -32443,13 +32443,13 @@
         <v>11:22 AM</v>
       </c>
       <c r="G641" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H641">
-        <v>0</v>
+        <v>11.12</v>
       </c>
       <c r="I641">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J641">
         <v>0</v>
@@ -32458,16 +32458,16 @@
         <v>0</v>
       </c>
       <c r="L641">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M641">
         <v>0</v>
       </c>
       <c r="N641">
-        <v>0</v>
+        <v>1650</v>
       </c>
       <c r="O641" t="str">
-        <v>Devadas E K</v>
+        <v>Devadas E K | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P641" t="str">
         <v/>
@@ -32534,7 +32534,7 @@
         <v>GEORGE THOMAS</v>
       </c>
       <c r="D643" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E643" t="str">
         <v>INTEREXT OFFICE</v>
@@ -32543,13 +32543,13 @@
         <v>11:22 AM</v>
       </c>
       <c r="G643" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H643">
-        <v>0</v>
+        <v>11.12</v>
       </c>
       <c r="I643">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J643">
         <v>0</v>
@@ -32564,10 +32564,10 @@
         <v>0</v>
       </c>
       <c r="N643">
-        <v>0</v>
+        <v>1300</v>
       </c>
       <c r="O643" t="str">
-        <v>George Thomas</v>
+        <v>George Thomas | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P643" t="str">
         <v/>
@@ -32584,7 +32584,7 @@
         <v>GOKUL K</v>
       </c>
       <c r="D644" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E644" t="str">
         <v>INTEREXT OFFICE</v>
@@ -32593,13 +32593,13 @@
         <v>11:22 AM</v>
       </c>
       <c r="G644" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H644">
-        <v>0</v>
+        <v>11.12</v>
       </c>
       <c r="I644">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J644">
         <v>0</v>
@@ -32614,10 +32614,10 @@
         <v>0</v>
       </c>
       <c r="N644">
-        <v>0</v>
+        <v>900</v>
       </c>
       <c r="O644" t="str">
-        <v>Gokul K</v>
+        <v>Gokul K | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P644" t="str">
         <v/>
@@ -32734,7 +32734,7 @@
         <v>James TM</v>
       </c>
       <c r="D647" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E647" t="str">
         <v>INTEREXT OFFICE</v>
@@ -32743,13 +32743,13 @@
         <v>11:22 AM</v>
       </c>
       <c r="G647" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H647">
-        <v>0</v>
+        <v>11.12</v>
       </c>
       <c r="I647">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J647">
         <v>0</v>
@@ -32758,16 +32758,16 @@
         <v>0</v>
       </c>
       <c r="L647">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M647">
         <v>0</v>
       </c>
       <c r="N647">
-        <v>0</v>
+        <v>1250</v>
       </c>
       <c r="O647" t="str">
-        <v>James T M</v>
+        <v>James T M | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P647" t="str">
         <v/>
@@ -32984,7 +32984,7 @@
         <v>Mahin KJ</v>
       </c>
       <c r="D652" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E652" t="str">
         <v>INTEREXT OFFICE</v>
@@ -32993,10 +32993,10 @@
         <v>07:00 PM</v>
       </c>
       <c r="G652" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H652">
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="I652">
         <v>0</v>
@@ -33014,10 +33014,10 @@
         <v>0</v>
       </c>
       <c r="N652">
-        <v>0</v>
+        <v>454.34</v>
       </c>
       <c r="O652" t="str">
-        <v>7.00pm</v>
+        <v>7.00pm | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P652" t="str">
         <v/>
@@ -33034,7 +33034,7 @@
         <v>Manu Mahesh</v>
       </c>
       <c r="D653" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E653" t="str">
         <v>INTEREXT OFFICE</v>
@@ -33043,13 +33043,13 @@
         <v>11:22 AM</v>
       </c>
       <c r="G653" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H653">
-        <v>0</v>
+        <v>11.12</v>
       </c>
       <c r="I653">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J653">
         <v>0</v>
@@ -33064,10 +33064,10 @@
         <v>0</v>
       </c>
       <c r="N653">
-        <v>0</v>
+        <v>1333.33</v>
       </c>
       <c r="O653" t="str">
-        <v>Manu Mahesh</v>
+        <v>Manu Mahesh | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P653" t="str">
         <v/>
@@ -33134,7 +33134,7 @@
         <v>NIJI MANOJ</v>
       </c>
       <c r="D655" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E655" t="str">
         <v>INTEREXT OFFICE</v>
@@ -33143,13 +33143,13 @@
         <v>11:22 AM</v>
       </c>
       <c r="G655" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H655">
-        <v>0</v>
+        <v>11.12</v>
       </c>
       <c r="I655">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J655">
         <v>0</v>
@@ -33158,16 +33158,16 @@
         <v>0</v>
       </c>
       <c r="L655">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M655">
         <v>0</v>
       </c>
       <c r="N655">
-        <v>0</v>
+        <v>750</v>
       </c>
       <c r="O655" t="str">
-        <v>Niji Manoj</v>
+        <v>Niji Manoj | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P655" t="str">
         <v/>
@@ -33184,7 +33184,7 @@
         <v>Niranjan Bose</v>
       </c>
       <c r="D656" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E656" t="str">
         <v>INTEREXT OFFICE</v>
@@ -33193,13 +33193,13 @@
         <v>11:22 AM</v>
       </c>
       <c r="G656" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H656">
-        <v>0</v>
+        <v>11.12</v>
       </c>
       <c r="I656">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J656">
         <v>0</v>
@@ -33214,10 +33214,10 @@
         <v>0</v>
       </c>
       <c r="N656">
-        <v>0</v>
+        <v>866.67</v>
       </c>
       <c r="O656" t="str">
-        <v>Niranjan Bose</v>
+        <v>Niranjan Bose | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P656" t="str">
         <v/>
@@ -33284,7 +33284,7 @@
         <v>Pappu Kumar Rana</v>
       </c>
       <c r="D658" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E658" t="str">
         <v>INTEREXT OFFICE</v>
@@ -33293,13 +33293,13 @@
         <v>11:22 AM</v>
       </c>
       <c r="G658" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H658">
-        <v>0</v>
+        <v>11.12</v>
       </c>
       <c r="I658">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J658">
         <v>0</v>
@@ -33308,16 +33308,16 @@
         <v>0</v>
       </c>
       <c r="L658">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M658">
         <v>0</v>
       </c>
       <c r="N658">
-        <v>0</v>
+        <v>1350</v>
       </c>
       <c r="O658" t="str">
-        <v>Pappu Kumar Rana</v>
+        <v>Pappu Kumar Rana | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P658" t="str">
         <v/>
@@ -33334,7 +33334,7 @@
         <v>PRASANTH E.M</v>
       </c>
       <c r="D659" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E659" t="str">
         <v>INTEREXT OFFICE</v>
@@ -33343,13 +33343,13 @@
         <v>11:22 AM</v>
       </c>
       <c r="G659" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H659">
-        <v>0</v>
+        <v>11.12</v>
       </c>
       <c r="I659">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J659">
         <v>0</v>
@@ -33364,10 +33364,10 @@
         <v>0</v>
       </c>
       <c r="N659">
-        <v>0</v>
+        <v>1192.31</v>
       </c>
       <c r="O659" t="str">
-        <v>Prasanth E M</v>
+        <v>Prasanth E M | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P659" t="str">
         <v/>
@@ -33384,7 +33384,7 @@
         <v>PRATHEESH K S</v>
       </c>
       <c r="D660" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E660" t="str">
         <v>INTEREXT OFFICE</v>
@@ -33393,13 +33393,13 @@
         <v>11:22 AM</v>
       </c>
       <c r="G660" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H660">
-        <v>0</v>
+        <v>11.12</v>
       </c>
       <c r="I660">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J660">
         <v>0</v>
@@ -33414,10 +33414,10 @@
         <v>0</v>
       </c>
       <c r="N660">
-        <v>0</v>
+        <v>1900</v>
       </c>
       <c r="O660" t="str">
-        <v>Pratheesh K S</v>
+        <v>Pratheesh K S | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P660" t="str">
         <v/>
@@ -33434,7 +33434,7 @@
         <v>Rahul Das</v>
       </c>
       <c r="D661" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E661" t="str">
         <v>INTEREXT OFFICE</v>
@@ -33443,10 +33443,10 @@
         <v>07:00 PM</v>
       </c>
       <c r="G661" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H661">
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="I661">
         <v>0</v>
@@ -33464,10 +33464,10 @@
         <v>0</v>
       </c>
       <c r="N661">
-        <v>0</v>
+        <v>370.19</v>
       </c>
       <c r="O661" t="str">
-        <v>7:00pm</v>
+        <v>7:00pm | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P661" t="str">
         <v/>
@@ -33534,7 +33534,7 @@
         <v>RAHUL SUNDARAN</v>
       </c>
       <c r="D663" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E663" t="str">
         <v>INTEREXT OFFICE</v>
@@ -33543,13 +33543,13 @@
         <v>11:22 AM</v>
       </c>
       <c r="G663" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H663">
-        <v>0</v>
+        <v>11.12</v>
       </c>
       <c r="I663">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J663">
         <v>0</v>
@@ -33564,10 +33564,10 @@
         <v>0</v>
       </c>
       <c r="N663">
-        <v>0</v>
+        <v>1166.67</v>
       </c>
       <c r="O663" t="str">
-        <v>Rahul Sundaran</v>
+        <v>Rahul Sundaran | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P663" t="str">
         <v/>
@@ -33584,7 +33584,7 @@
         <v>Raj Kumar Rana</v>
       </c>
       <c r="D664" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E664" t="str">
         <v>INTEREXT OFFICE</v>
@@ -33593,13 +33593,13 @@
         <v>11:22 AM</v>
       </c>
       <c r="G664" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H664">
-        <v>0</v>
+        <v>11.12</v>
       </c>
       <c r="I664">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J664">
         <v>0</v>
@@ -33608,16 +33608,16 @@
         <v>0</v>
       </c>
       <c r="L664">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M664">
         <v>0</v>
       </c>
       <c r="N664">
-        <v>0</v>
+        <v>1105</v>
       </c>
       <c r="O664" t="str">
-        <v>Rajkumar Rana</v>
+        <v>Rajkumar Rana | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P664" t="str">
         <v/>
@@ -33634,7 +33634,7 @@
         <v>RAJI KANNAN</v>
       </c>
       <c r="D665" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E665" t="str">
         <v>INTEREXT OFFICE</v>
@@ -33643,13 +33643,13 @@
         <v>11:22 AM</v>
       </c>
       <c r="G665" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H665">
-        <v>0</v>
+        <v>11.12</v>
       </c>
       <c r="I665">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J665">
         <v>0</v>
@@ -33658,16 +33658,16 @@
         <v>0</v>
       </c>
       <c r="L665">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M665">
         <v>0</v>
       </c>
       <c r="N665">
-        <v>0</v>
+        <v>750</v>
       </c>
       <c r="O665" t="str">
-        <v>Raji Kannan</v>
+        <v>Raji Kannan | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P665" t="str">
         <v/>
@@ -33684,7 +33684,7 @@
         <v>Raju Rana</v>
       </c>
       <c r="D666" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E666" t="str">
         <v>INTEREXT OFFICE</v>
@@ -33693,13 +33693,13 @@
         <v>11:22 AM</v>
       </c>
       <c r="G666" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H666">
-        <v>0</v>
+        <v>11.12</v>
       </c>
       <c r="I666">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J666">
         <v>0</v>
@@ -33708,16 +33708,16 @@
         <v>0</v>
       </c>
       <c r="L666">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M666">
         <v>0</v>
       </c>
       <c r="N666">
-        <v>0</v>
+        <v>1175.01</v>
       </c>
       <c r="O666" t="str">
-        <v>Raju Rana</v>
+        <v>Raju Rana | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P666" t="str">
         <v/>
@@ -33834,7 +33834,7 @@
         <v>Ratheesh K S</v>
       </c>
       <c r="D669" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E669" t="str">
         <v>INTEREXT OFFICE</v>
@@ -33843,13 +33843,13 @@
         <v>11:22 AM</v>
       </c>
       <c r="G669" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H669">
-        <v>0</v>
+        <v>11.12</v>
       </c>
       <c r="I669">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J669">
         <v>0</v>
@@ -33858,16 +33858,16 @@
         <v>0</v>
       </c>
       <c r="L669">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M669">
         <v>0</v>
       </c>
       <c r="N669">
-        <v>0</v>
+        <v>1900</v>
       </c>
       <c r="O669" t="str">
-        <v>Ratheesh K S</v>
+        <v>Ratheesh K S | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P669" t="str">
         <v/>
@@ -33884,7 +33884,7 @@
         <v>Ratheesh P R</v>
       </c>
       <c r="D670" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E670" t="str">
         <v>INTEREXT OFFICE</v>
@@ -33893,13 +33893,13 @@
         <v>11:22 AM</v>
       </c>
       <c r="G670" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H670">
-        <v>0</v>
+        <v>11.12</v>
       </c>
       <c r="I670">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J670">
         <v>0</v>
@@ -33908,16 +33908,16 @@
         <v>0</v>
       </c>
       <c r="L670">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M670">
         <v>0</v>
       </c>
       <c r="N670">
-        <v>0</v>
+        <v>1690</v>
       </c>
       <c r="O670" t="str">
-        <v>Ratheesh P R</v>
+        <v>Ratheesh P R | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P670" t="str">
         <v/>
@@ -33934,7 +33934,7 @@
         <v>REBEESH K S</v>
       </c>
       <c r="D671" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E671" t="str">
         <v>INTEREXT OFFICE</v>
@@ -33943,13 +33943,13 @@
         <v>11:22 AM</v>
       </c>
       <c r="G671" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H671">
-        <v>0</v>
+        <v>11.12</v>
       </c>
       <c r="I671">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J671">
         <v>0</v>
@@ -33964,10 +33964,10 @@
         <v>0</v>
       </c>
       <c r="N671">
-        <v>0</v>
+        <v>1266.67</v>
       </c>
       <c r="O671" t="str">
-        <v>Rebeesh K S</v>
+        <v>Rebeesh K S | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P671" t="str">
         <v/>
@@ -33984,7 +33984,7 @@
         <v>REKHA MADHU</v>
       </c>
       <c r="D672" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E672" t="str">
         <v>INTEREXT OFFICE</v>
@@ -33993,13 +33993,13 @@
         <v>11:22 AM</v>
       </c>
       <c r="G672" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H672">
-        <v>0</v>
+        <v>11.12</v>
       </c>
       <c r="I672">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J672">
         <v>0</v>
@@ -34008,16 +34008,16 @@
         <v>0</v>
       </c>
       <c r="L672">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M672">
         <v>0</v>
       </c>
       <c r="N672">
-        <v>0</v>
+        <v>750</v>
       </c>
       <c r="O672" t="str">
-        <v>Reksha Madhu</v>
+        <v>Reksha Madhu | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P672" t="str">
         <v/>
@@ -34034,7 +34034,7 @@
         <v>Remanan N N</v>
       </c>
       <c r="D673" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E673" t="str">
         <v>INTEREXT OFFICE</v>
@@ -34043,13 +34043,13 @@
         <v>11:22 AM</v>
       </c>
       <c r="G673" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H673">
-        <v>0</v>
+        <v>11.12</v>
       </c>
       <c r="I673">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J673">
         <v>0</v>
@@ -34064,10 +34064,10 @@
         <v>0</v>
       </c>
       <c r="N673">
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="O673" t="str">
-        <v>Remanan N N</v>
+        <v>Remanan N N | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P673" t="str">
         <v/>
@@ -34234,7 +34234,7 @@
         <v>SHAHANA JABBAR</v>
       </c>
       <c r="D677" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E677" t="str">
         <v>INTEREXT OFFICE</v>
@@ -34243,13 +34243,13 @@
         <v>11:22 AM</v>
       </c>
       <c r="G677" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H677">
-        <v>0</v>
+        <v>11.12</v>
       </c>
       <c r="I677">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J677">
         <v>0</v>
@@ -34264,10 +34264,10 @@
         <v>0</v>
       </c>
       <c r="N677">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="O677" t="str">
-        <v>Shahana Jabbar</v>
+        <v>Shahana Jabbar | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P677" t="str">
         <v/>
@@ -34284,7 +34284,7 @@
         <v>SHINODH N T</v>
       </c>
       <c r="D678" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E678" t="str">
         <v>INTEREXT OFFICE</v>
@@ -34293,13 +34293,13 @@
         <v>11:22 AM</v>
       </c>
       <c r="G678" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H678">
-        <v>0</v>
+        <v>11.12</v>
       </c>
       <c r="I678">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J678">
         <v>0</v>
@@ -34314,10 +34314,10 @@
         <v>0</v>
       </c>
       <c r="N678">
-        <v>0</v>
+        <v>1666.67</v>
       </c>
       <c r="O678" t="str">
-        <v>Shinod N T</v>
+        <v>Shinod N T | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P678" t="str">
         <v/>
@@ -34334,7 +34334,7 @@
         <v>SHYAM MURALI</v>
       </c>
       <c r="D679" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E679" t="str">
         <v>INTEREXT OFFICE</v>
@@ -34343,13 +34343,13 @@
         <v>11:22 AM</v>
       </c>
       <c r="G679" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H679">
-        <v>0</v>
+        <v>11.12</v>
       </c>
       <c r="I679">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J679">
         <v>0</v>
@@ -34364,10 +34364,10 @@
         <v>0</v>
       </c>
       <c r="N679">
-        <v>0</v>
+        <v>1366.67</v>
       </c>
       <c r="O679" t="str">
-        <v>Shyam Murali</v>
+        <v>Shyam Murali | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P679" t="str">
         <v/>
@@ -34434,7 +34434,7 @@
         <v>Sineesh Sasi</v>
       </c>
       <c r="D681" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E681" t="str">
         <v>INTEREXT OFFICE</v>
@@ -34443,13 +34443,13 @@
         <v>11:22 AM</v>
       </c>
       <c r="G681" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H681">
-        <v>0</v>
+        <v>11.12</v>
       </c>
       <c r="I681">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J681">
         <v>0</v>
@@ -34464,10 +34464,10 @@
         <v>0</v>
       </c>
       <c r="N681">
-        <v>0</v>
+        <v>966.67</v>
       </c>
       <c r="O681" t="str">
-        <v>Sineesh Sasi</v>
+        <v>Sineesh Sasi | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P681" t="str">
         <v/>
@@ -34484,7 +34484,7 @@
         <v>Sona Francis</v>
       </c>
       <c r="D682" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E682" t="str">
         <v>INTEREXT OFFICE</v>
@@ -34493,13 +34493,13 @@
         <v>11:22 AM</v>
       </c>
       <c r="G682" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H682">
-        <v>0</v>
+        <v>11.12</v>
       </c>
       <c r="I682">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J682">
         <v>0</v>
@@ -34514,10 +34514,10 @@
         <v>0</v>
       </c>
       <c r="N682">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="O682" t="str">
-        <v>Sona Francis</v>
+        <v>Sona Francis | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P682" t="str">
         <v/>
@@ -34684,7 +34684,7 @@
         <v>Stephin Pious</v>
       </c>
       <c r="D686" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E686" t="str">
         <v>INTEREXT OFFICE</v>
@@ -34693,13 +34693,13 @@
         <v>11:22 AM</v>
       </c>
       <c r="G686" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H686">
-        <v>0</v>
+        <v>11.12</v>
       </c>
       <c r="I686">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J686">
         <v>0</v>
@@ -34714,10 +34714,10 @@
         <v>0</v>
       </c>
       <c r="N686">
-        <v>0</v>
+        <v>961.54</v>
       </c>
       <c r="O686" t="str">
-        <v>Stephin Pious</v>
+        <v>Stephin Pious | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P686" t="str">
         <v/>
@@ -34984,7 +34984,7 @@
         <v>Sunil. C. M</v>
       </c>
       <c r="D692" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E692" t="str">
         <v>INTEREXT OFFICE</v>
@@ -34993,13 +34993,13 @@
         <v>11:22 AM</v>
       </c>
       <c r="G692" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H692">
-        <v>0</v>
+        <v>11.12</v>
       </c>
       <c r="I692">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J692">
         <v>0</v>
@@ -35008,16 +35008,16 @@
         <v>0</v>
       </c>
       <c r="L692">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M692">
         <v>0</v>
       </c>
       <c r="N692">
-        <v>0</v>
+        <v>1300</v>
       </c>
       <c r="O692" t="str">
-        <v>Sunil C M</v>
+        <v>Sunil C M | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P692" t="str">
         <v/>
@@ -35134,7 +35134,7 @@
         <v>Aamil</v>
       </c>
       <c r="D695" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E695" t="str">
         <v>INTEREXT OFFICE</v>
@@ -35143,13 +35143,13 @@
         <v>12:36 PM</v>
       </c>
       <c r="G695" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H695">
-        <v>0</v>
+        <v>9.88</v>
       </c>
       <c r="I695">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J695">
         <v>0</v>
@@ -35158,16 +35158,16 @@
         <v>0</v>
       </c>
       <c r="L695">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M695">
         <v>0</v>
       </c>
       <c r="N695">
-        <v>0</v>
+        <v>1440</v>
       </c>
       <c r="O695" t="str">
-        <v>Aamil</v>
+        <v>Aamil | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P695" t="str">
         <v/>
@@ -35384,7 +35384,7 @@
         <v>Ajmal K H</v>
       </c>
       <c r="D700" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E700" t="str">
         <v>INTEREXT OFFICE</v>
@@ -35393,13 +35393,13 @@
         <v>12:36 PM</v>
       </c>
       <c r="G700" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H700">
-        <v>0</v>
+        <v>9.88</v>
       </c>
       <c r="I700">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J700">
         <v>0</v>
@@ -35408,16 +35408,16 @@
         <v>0</v>
       </c>
       <c r="L700">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M700">
         <v>0</v>
       </c>
       <c r="N700">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="O700" t="str">
-        <v>Ajmal K H</v>
+        <v>Ajmal K H | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P700" t="str">
         <v/>
@@ -35484,7 +35484,7 @@
         <v>Akhil AK</v>
       </c>
       <c r="D702" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E702" t="str">
         <v>INTEREXT OFFICE</v>
@@ -35493,13 +35493,13 @@
         <v>12:36 PM</v>
       </c>
       <c r="G702" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H702">
-        <v>0</v>
+        <v>9.88</v>
       </c>
       <c r="I702">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J702">
         <v>0</v>
@@ -35508,16 +35508,16 @@
         <v>0</v>
       </c>
       <c r="L702">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M702">
         <v>0</v>
       </c>
       <c r="N702">
-        <v>0</v>
+        <v>1560</v>
       </c>
       <c r="O702" t="str">
-        <v>Akhil AK</v>
+        <v>Akhil AK | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P702" t="str">
         <v/>
@@ -35734,7 +35734,7 @@
         <v>Anandhu Raj</v>
       </c>
       <c r="D707" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E707" t="str">
         <v>INTEREXT OFFICE</v>
@@ -35743,13 +35743,13 @@
         <v>12:36 PM</v>
       </c>
       <c r="G707" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H707">
-        <v>0</v>
+        <v>9.88</v>
       </c>
       <c r="I707">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J707">
         <v>0</v>
@@ -35758,16 +35758,16 @@
         <v>0</v>
       </c>
       <c r="L707">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M707">
         <v>0</v>
       </c>
       <c r="N707">
-        <v>0</v>
+        <v>1260</v>
       </c>
       <c r="O707" t="str">
-        <v>Anandhu Raj</v>
+        <v>Anandhu Raj | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P707" t="str">
         <v/>
@@ -35784,7 +35784,7 @@
         <v>Aneesh Ahammed</v>
       </c>
       <c r="D708" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E708" t="str">
         <v>INTEREXT OFFICE</v>
@@ -35793,13 +35793,13 @@
         <v>07:00 AM</v>
       </c>
       <c r="G708" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H708">
-        <v>0</v>
+        <v>15.5</v>
       </c>
       <c r="I708">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J708">
         <v>0</v>
@@ -35808,16 +35808,16 @@
         <v>0</v>
       </c>
       <c r="L708">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="M708">
         <v>0</v>
       </c>
       <c r="N708">
-        <v>0</v>
+        <v>1870</v>
       </c>
       <c r="O708" t="str">
-        <v>7:pm</v>
+        <v>7:pm | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P708" t="str">
         <v/>
@@ -35834,7 +35834,7 @@
         <v>Anil Rana</v>
       </c>
       <c r="D709" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E709" t="str">
         <v>INTEREXT OFFICE</v>
@@ -35843,13 +35843,13 @@
         <v>12:36 PM</v>
       </c>
       <c r="G709" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H709">
-        <v>0</v>
+        <v>9.88</v>
       </c>
       <c r="I709">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J709">
         <v>0</v>
@@ -35858,16 +35858,16 @@
         <v>0</v>
       </c>
       <c r="L709">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M709">
         <v>0</v>
       </c>
       <c r="N709">
-        <v>0</v>
+        <v>1260</v>
       </c>
       <c r="O709" t="str">
-        <v>Anil Rana</v>
+        <v>Anil Rana | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P709" t="str">
         <v/>
@@ -35984,7 +35984,7 @@
         <v>Anusree Subramanian</v>
       </c>
       <c r="D712" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E712" t="str">
         <v>INTEREXT OFFICE</v>
@@ -35993,13 +35993,13 @@
         <v>12:36 PM</v>
       </c>
       <c r="G712" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H712">
-        <v>0</v>
+        <v>9.88</v>
       </c>
       <c r="I712">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J712">
         <v>0</v>
@@ -36014,10 +36014,10 @@
         <v>0</v>
       </c>
       <c r="N712">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="O712" t="str">
-        <v>Anusree Subramanian</v>
+        <v>Anusree Subramanian | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P712" t="str">
         <v/>
@@ -36334,7 +36334,7 @@
         <v>Faiyaj Ansari</v>
       </c>
       <c r="D719" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E719" t="str">
         <v>INTEREXT OFFICE</v>
@@ -36343,13 +36343,13 @@
         <v>12:36 PM</v>
       </c>
       <c r="G719" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H719">
-        <v>0</v>
+        <v>9.88</v>
       </c>
       <c r="I719">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J719">
         <v>0</v>
@@ -36358,16 +36358,16 @@
         <v>0</v>
       </c>
       <c r="L719">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M719">
         <v>0</v>
       </c>
       <c r="N719">
-        <v>0</v>
+        <v>1080</v>
       </c>
       <c r="O719" t="str">
-        <v>Faiyaj Ansari</v>
+        <v>Faiyaj Ansari | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P719" t="str">
         <v/>
@@ -36384,7 +36384,7 @@
         <v>GEORGE THOMAS</v>
       </c>
       <c r="D720" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E720" t="str">
         <v>INTEREXT OFFICE</v>
@@ -36393,13 +36393,13 @@
         <v>11:00 AM</v>
       </c>
       <c r="G720" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H720">
-        <v>0</v>
+        <v>11.5</v>
       </c>
       <c r="I720">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J720">
         <v>0</v>
@@ -36414,10 +36414,10 @@
         <v>0</v>
       </c>
       <c r="N720">
-        <v>0</v>
+        <v>1300</v>
       </c>
       <c r="O720" t="str">
-        <v>I am 2 hour late to reach office today ( hospital case )</v>
+        <v>I am 2 hour late to reach office today ( hospital case ) | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P720" t="str">
         <v/>
@@ -36434,7 +36434,7 @@
         <v>GOKUL K</v>
       </c>
       <c r="D721" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E721" t="str">
         <v>INTEREXT OFFICE</v>
@@ -36443,13 +36443,13 @@
         <v>12:36 PM</v>
       </c>
       <c r="G721" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H721">
-        <v>0</v>
+        <v>9.88</v>
       </c>
       <c r="I721">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J721">
         <v>0</v>
@@ -36464,10 +36464,10 @@
         <v>0</v>
       </c>
       <c r="N721">
-        <v>0</v>
+        <v>900</v>
       </c>
       <c r="O721" t="str">
-        <v>Gokul Krishnan E V</v>
+        <v>Gokul Krishnan E V | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P721" t="str">
         <v/>
@@ -36584,7 +36584,7 @@
         <v>James TM</v>
       </c>
       <c r="D724" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E724" t="str">
         <v>INTEREXT OFFICE</v>
@@ -36593,13 +36593,13 @@
         <v>09:28 AM</v>
       </c>
       <c r="G724" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H724">
-        <v>0</v>
+        <v>13.02</v>
       </c>
       <c r="I724">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J724">
         <v>0</v>
@@ -36608,16 +36608,16 @@
         <v>0</v>
       </c>
       <c r="L724">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="M724">
         <v>0</v>
       </c>
       <c r="N724">
-        <v>0</v>
+        <v>1442.31</v>
       </c>
       <c r="O724" t="str">
-        <v>Iam an hour late</v>
+        <v>Iam an hour late | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P724" t="str">
         <v/>
@@ -36634,7 +36634,7 @@
         <v>Jitendra Rana</v>
       </c>
       <c r="D725" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E725" t="str">
         <v>INTEREXT OFFICE</v>
@@ -36643,13 +36643,13 @@
         <v>12:36 PM</v>
       </c>
       <c r="G725" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H725">
-        <v>0</v>
+        <v>9.88</v>
       </c>
       <c r="I725">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J725">
         <v>0</v>
@@ -36658,16 +36658,16 @@
         <v>0</v>
       </c>
       <c r="L725">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M725">
         <v>0</v>
       </c>
       <c r="N725">
-        <v>0</v>
+        <v>692.3</v>
       </c>
       <c r="O725" t="str">
-        <v>Jitendra Rana</v>
+        <v>Jitendra Rana | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P725" t="str">
         <v/>
@@ -36684,7 +36684,7 @@
         <v>Joshy</v>
       </c>
       <c r="D726" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E726" t="str">
         <v>INTEREXT OFFICE</v>
@@ -36693,13 +36693,13 @@
         <v>12:36 PM</v>
       </c>
       <c r="G726" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H726">
-        <v>0</v>
+        <v>9.88</v>
       </c>
       <c r="I726">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J726">
         <v>0</v>
@@ -36708,16 +36708,16 @@
         <v>0</v>
       </c>
       <c r="L726">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M726">
         <v>0</v>
       </c>
       <c r="N726">
-        <v>0</v>
+        <v>1620</v>
       </c>
       <c r="O726" t="str">
-        <v>Joshy</v>
+        <v>Joshy | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P726" t="str">
         <v/>
@@ -36834,7 +36834,7 @@
         <v>Mahin KJ</v>
       </c>
       <c r="D729" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E729" t="str">
         <v>INTEREXT OFFICE</v>
@@ -36843,10 +36843,10 @@
         <v>09:00 PM</v>
       </c>
       <c r="G729" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H729">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I729">
         <v>0</v>
@@ -36864,10 +36864,10 @@
         <v>0</v>
       </c>
       <c r="N729">
-        <v>0</v>
+        <v>194.72</v>
       </c>
       <c r="O729" t="str">
-        <v>9.00pm</v>
+        <v>9.00pm | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P729" t="str">
         <v/>
@@ -36934,7 +36934,7 @@
         <v>Mohammed Gulfam</v>
       </c>
       <c r="D731" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E731" t="str">
         <v>INTEREXT OFFICE</v>
@@ -36943,13 +36943,13 @@
         <v>12:36 PM</v>
       </c>
       <c r="G731" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H731">
-        <v>0</v>
+        <v>9.88</v>
       </c>
       <c r="I731">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J731">
         <v>0</v>
@@ -36958,16 +36958,16 @@
         <v>0</v>
       </c>
       <c r="L731">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M731">
         <v>0</v>
       </c>
       <c r="N731">
-        <v>0</v>
+        <v>1440</v>
       </c>
       <c r="O731" t="str">
-        <v>Mohammed Gulfam</v>
+        <v>Mohammed Gulfam | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P731" t="str">
         <v/>
@@ -37034,7 +37034,7 @@
         <v>Niranjan Bose</v>
       </c>
       <c r="D733" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E733" t="str">
         <v>INTEREXT OFFICE</v>
@@ -37043,13 +37043,13 @@
         <v>06:00 AM</v>
       </c>
       <c r="G733" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H733">
-        <v>0</v>
+        <v>16.5</v>
       </c>
       <c r="I733">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J733">
         <v>0</v>
@@ -37064,10 +37064,10 @@
         <v>0</v>
       </c>
       <c r="N733">
-        <v>0</v>
+        <v>866.67</v>
       </c>
       <c r="O733" t="str">
-        <v>30 minutes late</v>
+        <v>30 minutes late | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P733" t="str">
         <v/>
@@ -37084,7 +37084,7 @@
         <v>NOURIN SHAJI</v>
       </c>
       <c r="D734" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E734" t="str">
         <v>INTEREXT OFFICE</v>
@@ -37093,13 +37093,13 @@
         <v>12:36 PM</v>
       </c>
       <c r="G734" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H734">
-        <v>0</v>
+        <v>9.88</v>
       </c>
       <c r="I734">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J734">
         <v>0</v>
@@ -37114,10 +37114,10 @@
         <v>0</v>
       </c>
       <c r="N734">
-        <v>0</v>
+        <v>666.67</v>
       </c>
       <c r="O734" t="str">
-        <v>NOURIN SHAJI</v>
+        <v>NOURIN SHAJI | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P734" t="str">
         <v/>
@@ -37134,7 +37134,7 @@
         <v>Pappu Kumar Rana</v>
       </c>
       <c r="D735" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E735" t="str">
         <v>INTEREXT OFFICE</v>
@@ -37143,13 +37143,13 @@
         <v>12:36 PM</v>
       </c>
       <c r="G735" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H735">
-        <v>0</v>
+        <v>9.88</v>
       </c>
       <c r="I735">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J735">
         <v>0</v>
@@ -37158,16 +37158,16 @@
         <v>0</v>
       </c>
       <c r="L735">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M735">
         <v>0</v>
       </c>
       <c r="N735">
-        <v>0</v>
+        <v>1246.15</v>
       </c>
       <c r="O735" t="str">
-        <v>Pappu Kumar Rana</v>
+        <v>Pappu Kumar Rana | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P735" t="str">
         <v/>
@@ -37284,7 +37284,7 @@
         <v>Rahul Das</v>
       </c>
       <c r="D738" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E738" t="str">
         <v>INTEREXT OFFICE</v>
@@ -37293,10 +37293,10 @@
         <v>09:00 PM</v>
       </c>
       <c r="G738" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H738">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I738">
         <v>0</v>
@@ -37314,10 +37314,10 @@
         <v>0</v>
       </c>
       <c r="N738">
-        <v>0</v>
+        <v>158.66</v>
       </c>
       <c r="O738" t="str">
-        <v>9:00 PM</v>
+        <v>9:00 PM | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P738" t="str">
         <v/>
@@ -37334,7 +37334,7 @@
         <v>Rahul R Nair</v>
       </c>
       <c r="D739" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E739" t="str">
         <v>INTEREXT OFFICE</v>
@@ -37343,13 +37343,13 @@
         <v>12:36 PM</v>
       </c>
       <c r="G739" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H739">
-        <v>0</v>
+        <v>9.88</v>
       </c>
       <c r="I739">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J739">
         <v>0</v>
@@ -37358,16 +37358,16 @@
         <v>0</v>
       </c>
       <c r="L739">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M739">
         <v>0</v>
       </c>
       <c r="N739">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="O739" t="str">
-        <v>Rahul R Nair</v>
+        <v>Rahul R Nair | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P739" t="str">
         <v/>
@@ -37984,7 +37984,7 @@
         <v>Samshad Aalam</v>
       </c>
       <c r="D752" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E752" t="str">
         <v>INTEREXT OFFICE</v>
@@ -37993,13 +37993,13 @@
         <v>12:36 PM</v>
       </c>
       <c r="G752" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H752">
-        <v>0</v>
+        <v>9.88</v>
       </c>
       <c r="I752">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J752">
         <v>0</v>
@@ -38008,16 +38008,16 @@
         <v>0</v>
       </c>
       <c r="L752">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M752">
         <v>0</v>
       </c>
       <c r="N752">
-        <v>0</v>
+        <v>1080</v>
       </c>
       <c r="O752" t="str">
-        <v>Samshad Aalam</v>
+        <v>Samshad Aalam | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P752" t="str">
         <v/>
@@ -38434,7 +38434,7 @@
         <v>Sreenath C V</v>
       </c>
       <c r="D761" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E761" t="str">
         <v>INTEREXT OFFICE</v>
@@ -38443,13 +38443,13 @@
         <v>12:36 PM</v>
       </c>
       <c r="G761" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H761">
-        <v>0</v>
+        <v>9.88</v>
       </c>
       <c r="I761">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J761">
         <v>0</v>
@@ -38458,16 +38458,16 @@
         <v>0</v>
       </c>
       <c r="L761">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M761">
         <v>0</v>
       </c>
       <c r="N761">
-        <v>0</v>
+        <v>692.3</v>
       </c>
       <c r="O761" t="str">
-        <v>Sreenath C V</v>
+        <v>Sreenath C V | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P761" t="str">
         <v/>
@@ -38484,7 +38484,7 @@
         <v>Sreeraj V S</v>
       </c>
       <c r="D762" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E762" t="str">
         <v>INTEREXT OFFICE</v>
@@ -38493,13 +38493,13 @@
         <v>12:36 PM</v>
       </c>
       <c r="G762" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H762">
-        <v>0</v>
+        <v>9.88</v>
       </c>
       <c r="I762">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J762">
         <v>0</v>
@@ -38508,16 +38508,16 @@
         <v>0</v>
       </c>
       <c r="L762">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M762">
         <v>0</v>
       </c>
       <c r="N762">
-        <v>0</v>
+        <v>1260</v>
       </c>
       <c r="O762" t="str">
-        <v>Sreeraj V S</v>
+        <v>Sreeraj V S | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P762" t="str">
         <v/>
@@ -38534,7 +38534,7 @@
         <v>Stephin Pious</v>
       </c>
       <c r="D763" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E763" t="str">
         <v>INTEREXT OFFICE</v>
@@ -38543,7 +38543,7 @@
         <v>03:15 AM</v>
       </c>
       <c r="G763" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H763">
         <v>0</v>
@@ -38567,7 +38567,7 @@
         <v>0</v>
       </c>
       <c r="O763" t="str">
-        <v>3.15 am</v>
+        <v>3.15 am | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P763" t="str">
         <v/>
@@ -38584,7 +38584,7 @@
         <v>Subodh Sha</v>
       </c>
       <c r="D764" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E764" t="str">
         <v>INTEREXT OFFICE</v>
@@ -38593,13 +38593,13 @@
         <v>12:36 PM</v>
       </c>
       <c r="G764" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H764">
-        <v>0</v>
+        <v>9.88</v>
       </c>
       <c r="I764">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J764">
         <v>0</v>
@@ -38608,16 +38608,16 @@
         <v>0</v>
       </c>
       <c r="L764">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M764">
         <v>0</v>
       </c>
       <c r="N764">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="O764" t="str">
-        <v>Subodh Sha</v>
+        <v>Subodh Sha | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P764" t="str">
         <v/>
@@ -38684,7 +38684,7 @@
         <v>Sumesh B</v>
       </c>
       <c r="D766" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E766" t="str">
         <v>INTEREXT OFFICE</v>
@@ -38693,13 +38693,13 @@
         <v>12:36 PM</v>
       </c>
       <c r="G766" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H766">
-        <v>0</v>
+        <v>9.88</v>
       </c>
       <c r="I766">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J766">
         <v>0</v>
@@ -38708,16 +38708,16 @@
         <v>0</v>
       </c>
       <c r="L766">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M766">
         <v>0</v>
       </c>
       <c r="N766">
-        <v>0</v>
+        <v>1560</v>
       </c>
       <c r="O766" t="str">
-        <v>Sumesh B</v>
+        <v>Sumesh B | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P766" t="str">
         <v/>
@@ -38884,7 +38884,7 @@
         <v>Tufail Alam Danish</v>
       </c>
       <c r="D770" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E770" t="str">
         <v>INTEREXT OFFICE</v>
@@ -38893,13 +38893,13 @@
         <v>12:36 PM</v>
       </c>
       <c r="G770" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H770">
-        <v>0</v>
+        <v>9.88</v>
       </c>
       <c r="I770">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J770">
         <v>0</v>
@@ -38908,16 +38908,16 @@
         <v>0</v>
       </c>
       <c r="L770">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M770">
         <v>0</v>
       </c>
       <c r="N770">
-        <v>0</v>
+        <v>1080</v>
       </c>
       <c r="O770" t="str">
-        <v>Tufail Alam Danish</v>
+        <v>Tufail Alam Danish | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P770" t="str">
         <v/>
@@ -39284,7 +39284,7 @@
         <v>Akash</v>
       </c>
       <c r="D778" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E778" t="str">
         <v>INTEREXT OFFICE</v>
@@ -39293,7 +39293,7 @@
         <v>03:22 AM</v>
       </c>
       <c r="G778" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H778">
         <v>0</v>
@@ -39317,7 +39317,7 @@
         <v>0</v>
       </c>
       <c r="O778" t="str">
-        <v>Akash, Raju, Rajkumar, Bimal, stephin driver</v>
+        <v>Akash, Raju, Rajkumar, Bimal, stephin driver | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P778" t="str">
         <v/>
@@ -39634,7 +39634,7 @@
         <v>Aneesh Ahammed</v>
       </c>
       <c r="D785" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E785" t="str">
         <v>INTEREXT OFFICE</v>
@@ -39643,10 +39643,10 @@
         <v>07:00 PM</v>
       </c>
       <c r="G785" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H785">
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="I785">
         <v>0</v>
@@ -39664,10 +39664,10 @@
         <v>0</v>
       </c>
       <c r="N785">
-        <v>0</v>
+        <v>481.25</v>
       </c>
       <c r="O785" t="str">
-        <v>7:00pm</v>
+        <v>7:00pm | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P785" t="str">
         <v/>
@@ -40684,7 +40684,7 @@
         <v>Mahin KJ</v>
       </c>
       <c r="D806" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E806" t="str">
         <v>INTEREXT OFFICE</v>
@@ -40693,10 +40693,10 @@
         <v>09:35 PM</v>
       </c>
       <c r="G806" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H806">
-        <v>0</v>
+        <v>0.92</v>
       </c>
       <c r="I806">
         <v>0</v>
@@ -40714,10 +40714,10 @@
         <v>0</v>
       </c>
       <c r="N806">
-        <v>0</v>
+        <v>119.43</v>
       </c>
       <c r="O806" t="str">
-        <v>9.35pm</v>
+        <v>9.35pm | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P806" t="str">
         <v/>
@@ -41134,7 +41134,7 @@
         <v>Rahul Das</v>
       </c>
       <c r="D815" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E815" t="str">
         <v>INTEREXT OFFICE</v>
@@ -41143,10 +41143,10 @@
         <v>07:00 PM</v>
       </c>
       <c r="G815" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H815">
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="I815">
         <v>0</v>
@@ -41164,10 +41164,10 @@
         <v>0</v>
       </c>
       <c r="N815">
-        <v>0</v>
+        <v>370.19</v>
       </c>
       <c r="O815" t="str">
-        <v>7:00pm</v>
+        <v>7:00pm | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P815" t="str">
         <v/>
@@ -41434,7 +41434,7 @@
         <v>Rakesh Sadhukha</v>
       </c>
       <c r="D821" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E821" t="str">
         <v>INTEREXT OFFICE</v>
@@ -41443,13 +41443,13 @@
         <v>08:44 AM</v>
       </c>
       <c r="G821" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H821">
-        <v>0</v>
+        <v>13.75</v>
       </c>
       <c r="I821">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J821">
         <v>0</v>
@@ -41464,10 +41464,10 @@
         <v>0</v>
       </c>
       <c r="N821">
-        <v>0</v>
+        <v>1538.46</v>
       </c>
       <c r="O821" t="str">
-        <v>Rakesh Sadhukha, Sukant Mishal</v>
+        <v>Rakesh Sadhukha, Sukant Mishal | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P821" t="str">
         <v/>
@@ -43234,7 +43234,7 @@
         <v>AKHIL P KUMAR</v>
       </c>
       <c r="D857" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E857" t="str">
         <v>INTEREXT OFFICE</v>
@@ -43243,13 +43243,13 @@
         <v>10:00 AM</v>
       </c>
       <c r="G857" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H857">
-        <v>0</v>
+        <v>12.5</v>
       </c>
       <c r="I857">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J857">
         <v>0</v>
@@ -43264,10 +43264,10 @@
         <v>0</v>
       </c>
       <c r="N857">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="O857" t="str">
-        <v>I am 1 hr late to reach office today</v>
+        <v>I am 1 hr late to reach office today | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P857" t="str">
         <v/>
@@ -43484,7 +43484,7 @@
         <v>Aneesh Ahammed</v>
       </c>
       <c r="D862" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E862" t="str">
         <v>INTEREXT OFFICE</v>
@@ -43493,10 +43493,10 @@
         <v>10:00 PM</v>
       </c>
       <c r="G862" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H862">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I862">
         <v>0</v>
@@ -43514,10 +43514,10 @@
         <v>0</v>
       </c>
       <c r="N862">
-        <v>0</v>
+        <v>68.75</v>
       </c>
       <c r="O862" t="str">
-        <v>10:00PM</v>
+        <v>10:00PM | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P862" t="str">
         <v/>
@@ -44534,7 +44534,7 @@
         <v>Mahin KJ</v>
       </c>
       <c r="D883" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E883" t="str">
         <v>INTEREXT OFFICE</v>
@@ -44543,10 +44543,10 @@
         <v>07:00 PM</v>
       </c>
       <c r="G883" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H883">
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="I883">
         <v>0</v>
@@ -44564,10 +44564,10 @@
         <v>0</v>
       </c>
       <c r="N883">
-        <v>0</v>
+        <v>454.34</v>
       </c>
       <c r="O883" t="str">
-        <v>7.00pm</v>
+        <v>7.00pm | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P883" t="str">
         <v/>
@@ -44984,7 +44984,7 @@
         <v>Rahul Das</v>
       </c>
       <c r="D892" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E892" t="str">
         <v>INTEREXT OFFICE</v>
@@ -44993,10 +44993,10 @@
         <v>07:00 PM</v>
       </c>
       <c r="G892" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H892">
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="I892">
         <v>0</v>
@@ -45014,10 +45014,10 @@
         <v>0</v>
       </c>
       <c r="N892">
-        <v>0</v>
+        <v>370.19</v>
       </c>
       <c r="O892" t="str">
-        <v>7:00pm</v>
+        <v>7:00pm | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P892" t="str">
         <v/>
@@ -45284,7 +45284,7 @@
         <v>Rakesh Sadhukha</v>
       </c>
       <c r="D898" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E898" t="str">
         <v>INTEREXT OFFICE</v>
@@ -45293,13 +45293,13 @@
         <v>09:29 AM</v>
       </c>
       <c r="G898" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H898">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="I898">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J898">
         <v>0</v>
@@ -45314,10 +45314,10 @@
         <v>0</v>
       </c>
       <c r="N898">
-        <v>0</v>
+        <v>1538.46</v>
       </c>
       <c r="O898" t="str">
-        <v>Rakesh Sadhukha, Sukant Mishal</v>
+        <v>Rakesh Sadhukha, Sukant Mishal | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P898" t="str">
         <v/>

</xml_diff>

<commit_message>
Cache resolved WhatsApp group JIDs and re-sync spreadsheet
</commit_message>
<xml_diff>
--- a/Attendance_Payroll.xlsx
+++ b/Attendance_Payroll.xlsx
@@ -46934,10 +46934,10 @@
         <v>Ajmal K H</v>
       </c>
       <c r="D931" t="str">
-        <v>ABSENT</v>
+        <v>LEAVE</v>
       </c>
       <c r="E931" t="str">
-        <v>—</v>
+        <v>INTEREXT OFFICE</v>
       </c>
       <c r="F931" t="str">
         <v>—</v>
@@ -46967,10 +46967,10 @@
         <v>0</v>
       </c>
       <c r="O931" t="str">
-        <v>—</v>
+        <v>Completed</v>
       </c>
       <c r="P931" t="str">
-        <v>Auto-Marked Absent (Missing text)</v>
+        <v/>
       </c>
     </row>
     <row r="932">

</xml_diff>

<commit_message>
feat: enforce Title Case formatting for all employee names in database and spreadsheet
</commit_message>
<xml_diff>
--- a/Attendance_Payroll.xlsx
+++ b/Attendance_Payroll.xlsx
@@ -625,7 +625,7 @@
         <v>Monday</v>
       </c>
       <c r="C5" t="str">
-        <v>AJEESH VIJAYAN</v>
+        <v>Ajeesh Vijayan</v>
       </c>
       <c r="D5" t="str">
         <v>ABSENT</v>
@@ -825,7 +825,7 @@
         <v>Monday</v>
       </c>
       <c r="C9" t="str">
-        <v>Akhil AK</v>
+        <v>Akhil Ak</v>
       </c>
       <c r="D9" t="str">
         <v>ABSENT</v>
@@ -875,7 +875,7 @@
         <v>Monday</v>
       </c>
       <c r="C10" t="str">
-        <v>AKHIL P KUMAR</v>
+        <v>Akhil P Kumar</v>
       </c>
       <c r="D10" t="str">
         <v>ABSENT</v>
@@ -1025,7 +1025,7 @@
         <v>Monday</v>
       </c>
       <c r="C13" t="str">
-        <v>ANADHU SUNIL</v>
+        <v>Anadhu Sunil</v>
       </c>
       <c r="D13" t="str">
         <v>ABSENT</v>
@@ -1411,7 +1411,7 @@
         <v>1320</v>
       </c>
       <c r="O20" t="str">
-        <v>Subodsha, Sandeep Arun George Sabu Anadhu Gopal, 9-6 pm. Joseph lukose)</v>
+        <v>Arun, Vengalloor, 9-6</v>
       </c>
       <c r="P20" t="str">
         <v/>
@@ -1425,7 +1425,7 @@
         <v>Monday</v>
       </c>
       <c r="C21" t="str">
-        <v>Arun P madhu</v>
+        <v>Arun P Madhu</v>
       </c>
       <c r="D21" t="str">
         <v>ABSENT</v>
@@ -1525,7 +1525,7 @@
         <v>Monday</v>
       </c>
       <c r="C23" t="str">
-        <v>BINDHU JOSE</v>
+        <v>Bindhu Jose</v>
       </c>
       <c r="D23" t="str">
         <v>ABSENT</v>
@@ -1725,7 +1725,7 @@
         <v>Monday</v>
       </c>
       <c r="C27" t="str">
-        <v>GEORGE THOMAS</v>
+        <v>George Thomas</v>
       </c>
       <c r="D27" t="str">
         <v>ABSENT</v>
@@ -1775,7 +1775,7 @@
         <v>Monday</v>
       </c>
       <c r="C28" t="str">
-        <v>GOKUL K</v>
+        <v>Gokul K</v>
       </c>
       <c r="D28" t="str">
         <v>ABSENT</v>
@@ -1825,7 +1825,7 @@
         <v>Monday</v>
       </c>
       <c r="C29" t="str">
-        <v>Gokul Krishnan  E V</v>
+        <v>Gokul Krishnan E V</v>
       </c>
       <c r="D29" t="str">
         <v>ABSENT</v>
@@ -1875,7 +1875,7 @@
         <v>Monday</v>
       </c>
       <c r="C30" t="str">
-        <v>Gopal (soma)</v>
+        <v>Gopal (Soma)</v>
       </c>
       <c r="D30" t="str">
         <v>ABSENT</v>
@@ -1925,7 +1925,7 @@
         <v>Monday</v>
       </c>
       <c r="C31" t="str">
-        <v>James TM</v>
+        <v>James Tm</v>
       </c>
       <c r="D31" t="str">
         <v>ABSENT</v>
@@ -2128,22 +2128,22 @@
         <v>M S Arjun</v>
       </c>
       <c r="D35" t="str">
-        <v>LEAVE</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E35" t="str">
         <v>INTEREXT OFFICE</v>
       </c>
       <c r="F35" t="str">
-        <v>—</v>
+        <v>08:00 AM</v>
       </c>
       <c r="G35" t="str">
-        <v>—</v>
+        <v>06:00 PM</v>
       </c>
       <c r="H35">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I35">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J35">
         <v>0</v>
@@ -2158,10 +2158,10 @@
         <v>0</v>
       </c>
       <c r="N35">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="O35" t="str">
-        <v>https://interext-image-collection.vercel.app</v>
+        <v>Arjun, 8-6</v>
       </c>
       <c r="P35" t="str">
         <v/>
@@ -2175,7 +2175,7 @@
         <v>Monday</v>
       </c>
       <c r="C36" t="str">
-        <v>Mahin KJ</v>
+        <v>Mahin Kj</v>
       </c>
       <c r="D36" t="str">
         <v>COMPLETED</v>
@@ -2325,7 +2325,7 @@
         <v>Monday</v>
       </c>
       <c r="C39" t="str">
-        <v>NIJI MANOJ</v>
+        <v>Niji Manoj</v>
       </c>
       <c r="D39" t="str">
         <v>ABSENT</v>
@@ -2425,7 +2425,7 @@
         <v>Monday</v>
       </c>
       <c r="C41" t="str">
-        <v>NOURIN SHAJI</v>
+        <v>Nourin Shaji</v>
       </c>
       <c r="D41" t="str">
         <v>ABSENT</v>
@@ -2525,7 +2525,7 @@
         <v>Monday</v>
       </c>
       <c r="C43" t="str">
-        <v>PRASANTH E.M</v>
+        <v>Prasanth E.M</v>
       </c>
       <c r="D43" t="str">
         <v>ABSENT</v>
@@ -2575,7 +2575,7 @@
         <v>Monday</v>
       </c>
       <c r="C44" t="str">
-        <v>PRATHEESH K S</v>
+        <v>Pratheesh K S</v>
       </c>
       <c r="D44" t="str">
         <v>ABSENT</v>
@@ -2725,7 +2725,7 @@
         <v>Monday</v>
       </c>
       <c r="C47" t="str">
-        <v>RAHUL SUNDARAN</v>
+        <v>Rahul Sundaran</v>
       </c>
       <c r="D47" t="str">
         <v>ABSENT</v>
@@ -2825,7 +2825,7 @@
         <v>Monday</v>
       </c>
       <c r="C49" t="str">
-        <v>RAJI KANNAN</v>
+        <v>Raji Kannan</v>
       </c>
       <c r="D49" t="str">
         <v>ABSENT</v>
@@ -3125,7 +3125,7 @@
         <v>Monday</v>
       </c>
       <c r="C55" t="str">
-        <v>REBEESH K S</v>
+        <v>Rebeesh K S</v>
       </c>
       <c r="D55" t="str">
         <v>ABSENT</v>
@@ -3175,7 +3175,7 @@
         <v>Monday</v>
       </c>
       <c r="C56" t="str">
-        <v>REKHA MADHU</v>
+        <v>Rekha Madhu</v>
       </c>
       <c r="D56" t="str">
         <v>ABSENT</v>
@@ -3425,7 +3425,7 @@
         <v>Monday</v>
       </c>
       <c r="C61" t="str">
-        <v>SHAHANA JABBAR</v>
+        <v>Shahana Jabbar</v>
       </c>
       <c r="D61" t="str">
         <v>ABSENT</v>
@@ -3475,7 +3475,7 @@
         <v>Monday</v>
       </c>
       <c r="C62" t="str">
-        <v>SHINODH N T</v>
+        <v>Shinodh N T</v>
       </c>
       <c r="D62" t="str">
         <v>ABSENT</v>
@@ -3525,7 +3525,7 @@
         <v>Monday</v>
       </c>
       <c r="C63" t="str">
-        <v>SHYAM MURALI</v>
+        <v>Shyam Murali</v>
       </c>
       <c r="D63" t="str">
         <v>ABSENT</v>
@@ -4317,7 +4317,7 @@
         <v/>
       </c>
     </row>
-    <row r="79">
+    <row r="79" xml:space="preserve">
       <c r="A79" t="str">
         <v>2026-05-26</v>
       </c>
@@ -4360,8 +4360,10 @@
       <c r="N79">
         <v>1320</v>
       </c>
-      <c r="O79" t="str">
-        <v>Aamil, Sunilrana, (9-6 pm milou)</v>
+      <c r="O79" t="str" xml:space="preserve">
+        <v xml:space="preserve">Aamil
+Office
+9-6</v>
       </c>
       <c r="P79" t="str">
         <v/>
@@ -4467,7 +4469,7 @@
         <v>Auto-Marked Absent (Missing text)</v>
       </c>
     </row>
-    <row r="82">
+    <row r="82" xml:space="preserve">
       <c r="A82" t="str">
         <v>2026-05-26</v>
       </c>
@@ -4475,25 +4477,25 @@
         <v>Tuesday</v>
       </c>
       <c r="C82" t="str">
-        <v>AJEESH VIJAYAN</v>
+        <v>Ajeesh Vijayan</v>
       </c>
       <c r="D82" t="str">
-        <v>LEAVE</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E82" t="str">
         <v>INTEREXT OFFICE</v>
       </c>
       <c r="F82" t="str">
-        <v>—</v>
+        <v>09:00 AM</v>
       </c>
       <c r="G82" t="str">
-        <v>—</v>
+        <v>06:00 PM</v>
       </c>
       <c r="H82">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I82">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J82">
         <v>0</v>
@@ -4508,10 +4510,12 @@
         <v>0</v>
       </c>
       <c r="N82">
-        <v>0</v>
-      </c>
-      <c r="O82" t="str">
-        <v>*half day leave tomorrow after noon session*</v>
+        <v>1066.67</v>
+      </c>
+      <c r="O82" t="str" xml:space="preserve">
+        <v xml:space="preserve">Ajeesh
+Office
+9-6</v>
       </c>
       <c r="P82" t="str">
         <v/>
@@ -4675,7 +4679,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C86" t="str">
-        <v>Akhil AK</v>
+        <v>Akhil Ak</v>
       </c>
       <c r="D86" t="str">
         <v>ABSENT</v>
@@ -4717,7 +4721,7 @@
         <v>Auto-Marked Absent (Missing text)</v>
       </c>
     </row>
-    <row r="87">
+    <row r="87" xml:space="preserve">
       <c r="A87" t="str">
         <v>2026-05-26</v>
       </c>
@@ -4725,25 +4729,25 @@
         <v>Tuesday</v>
       </c>
       <c r="C87" t="str">
-        <v>AKHIL P KUMAR</v>
+        <v>Akhil P Kumar</v>
       </c>
       <c r="D87" t="str">
-        <v>LEAVE</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E87" t="str">
         <v>INTEREXT OFFICE</v>
       </c>
       <c r="F87" t="str">
-        <v>—</v>
+        <v>09:00 AM</v>
       </c>
       <c r="G87" t="str">
-        <v>—</v>
+        <v>06:00 PM</v>
       </c>
       <c r="H87">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I87">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J87">
         <v>0</v>
@@ -4758,10 +4762,12 @@
         <v>0</v>
       </c>
       <c r="N87">
-        <v>0</v>
-      </c>
-      <c r="O87" t="str">
-        <v>I am on leave today</v>
+        <v>1200</v>
+      </c>
+      <c r="O87" t="str" xml:space="preserve">
+        <v xml:space="preserve">Akhil
+Kaloor
+9-6</v>
       </c>
       <c r="P87" t="str">
         <v/>
@@ -4875,7 +4881,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C90" t="str">
-        <v>ANADHU SUNIL</v>
+        <v>Anadhu Sunil</v>
       </c>
       <c r="D90" t="str">
         <v>ABSENT</v>
@@ -5261,7 +5267,7 @@
         <v>1320</v>
       </c>
       <c r="O97" t="str">
-        <v>Arun George, Sunilrana, (9-6 pm milou)</v>
+        <v>Arun, Vengalloor, 9-6</v>
       </c>
       <c r="P97" t="str">
         <v/>
@@ -5275,7 +5281,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C98" t="str">
-        <v>Arun P madhu</v>
+        <v>Arun P Madhu</v>
       </c>
       <c r="D98" t="str">
         <v>ABSENT</v>
@@ -5375,7 +5381,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C100" t="str">
-        <v>BINDHU JOSE</v>
+        <v>Bindhu Jose</v>
       </c>
       <c r="D100" t="str">
         <v>ABSENT</v>
@@ -5575,7 +5581,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C104" t="str">
-        <v>GEORGE THOMAS</v>
+        <v>George Thomas</v>
       </c>
       <c r="D104" t="str">
         <v>ABSENT</v>
@@ -5625,7 +5631,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C105" t="str">
-        <v>GOKUL K</v>
+        <v>Gokul K</v>
       </c>
       <c r="D105" t="str">
         <v>ABSENT</v>
@@ -5675,7 +5681,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C106" t="str">
-        <v>Gokul Krishnan  E V</v>
+        <v>Gokul Krishnan E V</v>
       </c>
       <c r="D106" t="str">
         <v>ABSENT</v>
@@ -5725,7 +5731,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C107" t="str">
-        <v>Gopal (soma)</v>
+        <v>Gopal (Soma)</v>
       </c>
       <c r="D107" t="str">
         <v>ABSENT</v>
@@ -5775,7 +5781,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C108" t="str">
-        <v>James TM</v>
+        <v>James Tm</v>
       </c>
       <c r="D108" t="str">
         <v>LEAVE</v>
@@ -5967,7 +5973,7 @@
         <v>Auto-Marked Absent (Missing text)</v>
       </c>
     </row>
-    <row r="112">
+    <row r="112" xml:space="preserve">
       <c r="A112" t="str">
         <v>2026-05-26</v>
       </c>
@@ -5978,22 +5984,22 @@
         <v>M S Arjun</v>
       </c>
       <c r="D112" t="str">
-        <v>ABSENT</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E112" t="str">
-        <v>—</v>
+        <v>Kottayam</v>
       </c>
       <c r="F112" t="str">
-        <v>—</v>
+        <v>08:00 AM</v>
       </c>
       <c r="G112" t="str">
-        <v>—</v>
+        <v>06:00 PM</v>
       </c>
       <c r="H112">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I112">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J112">
         <v>0</v>
@@ -6008,13 +6014,16 @@
         <v>0</v>
       </c>
       <c r="N112">
-        <v>0</v>
-      </c>
-      <c r="O112" t="str">
-        <v>—</v>
+        <v>1000</v>
+      </c>
+      <c r="O112" t="str" xml:space="preserve">
+        <v xml:space="preserve">Arjun
+Site : Kottayam
+In : 8:00 am
+Out : 6:00 pm</v>
       </c>
       <c r="P112" t="str">
-        <v>Auto-Marked Absent (Missing text)</v>
+        <v/>
       </c>
     </row>
     <row r="113">
@@ -6025,7 +6034,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C113" t="str">
-        <v>Mahin KJ</v>
+        <v>Mahin Kj</v>
       </c>
       <c r="D113" t="str">
         <v>COMPLETED</v>
@@ -6175,7 +6184,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C116" t="str">
-        <v>NIJI MANOJ</v>
+        <v>Niji Manoj</v>
       </c>
       <c r="D116" t="str">
         <v>ABSENT</v>
@@ -6275,7 +6284,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C118" t="str">
-        <v>NOURIN SHAJI</v>
+        <v>Nourin Shaji</v>
       </c>
       <c r="D118" t="str">
         <v>ABSENT</v>
@@ -6375,7 +6384,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C120" t="str">
-        <v>PRASANTH E.M</v>
+        <v>Prasanth E.M</v>
       </c>
       <c r="D120" t="str">
         <v>LEAVE</v>
@@ -6425,7 +6434,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C121" t="str">
-        <v>PRATHEESH K S</v>
+        <v>Pratheesh K S</v>
       </c>
       <c r="D121" t="str">
         <v>ABSENT</v>
@@ -6467,7 +6476,7 @@
         <v>Auto-Marked Absent (Missing text)</v>
       </c>
     </row>
-    <row r="122">
+    <row r="122" xml:space="preserve">
       <c r="A122" t="str">
         <v>2026-05-26</v>
       </c>
@@ -6484,16 +6493,16 @@
         <v>INTEREXT OFFICE</v>
       </c>
       <c r="F122" t="str">
-        <v>08:40 PM</v>
+        <v>09:00 AM</v>
       </c>
       <c r="G122" t="str">
-        <v>10:30 PM</v>
+        <v>06:00 PM</v>
       </c>
       <c r="H122">
-        <v>1.83</v>
+        <v>9</v>
       </c>
       <c r="I122">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J122">
         <v>0</v>
@@ -6508,10 +6517,12 @@
         <v>0</v>
       </c>
       <c r="N122">
-        <v>193.56</v>
-      </c>
-      <c r="O122" t="str">
-        <v>8:40pm | [System Auto-Checkout: Missed check-out]</v>
+        <v>846.15</v>
+      </c>
+      <c r="O122" t="str" xml:space="preserve">
+        <v xml:space="preserve">Rahul
+Muvattupuzha 
+9-6</v>
       </c>
       <c r="P122" t="str">
         <v/>
@@ -6575,7 +6586,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C124" t="str">
-        <v>RAHUL SUNDARAN</v>
+        <v>Rahul Sundaran</v>
       </c>
       <c r="D124" t="str">
         <v>ABSENT</v>
@@ -6675,7 +6686,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C126" t="str">
-        <v>RAJI KANNAN</v>
+        <v>Raji Kannan</v>
       </c>
       <c r="D126" t="str">
         <v>ABSENT</v>
@@ -6975,7 +6986,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C132" t="str">
-        <v>REBEESH K S</v>
+        <v>Rebeesh K S</v>
       </c>
       <c r="D132" t="str">
         <v>ABSENT</v>
@@ -7025,7 +7036,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C133" t="str">
-        <v>REKHA MADHU</v>
+        <v>Rekha Madhu</v>
       </c>
       <c r="D133" t="str">
         <v>ABSENT</v>
@@ -7275,7 +7286,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C138" t="str">
-        <v>SHAHANA JABBAR</v>
+        <v>Shahana Jabbar</v>
       </c>
       <c r="D138" t="str">
         <v>ABSENT</v>
@@ -7325,7 +7336,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C139" t="str">
-        <v>SHINODH N T</v>
+        <v>Shinodh N T</v>
       </c>
       <c r="D139" t="str">
         <v>ABSENT</v>
@@ -7375,25 +7386,25 @@
         <v>Tuesday</v>
       </c>
       <c r="C140" t="str">
-        <v>SHYAM MURALI</v>
+        <v>Shyam Murali</v>
       </c>
       <c r="D140" t="str">
-        <v>ABSENT</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E140" t="str">
-        <v>—</v>
+        <v>INTEREXT OFFICE</v>
       </c>
       <c r="F140" t="str">
-        <v>—</v>
+        <v>10:00 AM</v>
       </c>
       <c r="G140" t="str">
-        <v>—</v>
+        <v>06:00 PM</v>
       </c>
       <c r="H140">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I140">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J140">
         <v>0</v>
@@ -7408,13 +7419,13 @@
         <v>0</v>
       </c>
       <c r="N140">
-        <v>0</v>
+        <v>1366.67</v>
       </c>
       <c r="O140" t="str">
-        <v>—</v>
+        <v>Shyam, —, 10-6</v>
       </c>
       <c r="P140" t="str">
-        <v>Auto-Marked Absent (Missing text)</v>
+        <v/>
       </c>
     </row>
     <row r="141">
@@ -7428,22 +7439,22 @@
         <v>Siju Thomas</v>
       </c>
       <c r="D141" t="str">
-        <v>LEAVE</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E141" t="str">
         <v>INTEREXT OFFICE</v>
       </c>
       <c r="F141" t="str">
-        <v>—</v>
+        <v>09:00 AM</v>
       </c>
       <c r="G141" t="str">
-        <v>—</v>
+        <v>05:00 PM</v>
       </c>
       <c r="H141">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I141">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J141">
         <v>0</v>
@@ -7458,10 +7469,10 @@
         <v>0</v>
       </c>
       <c r="N141">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="O141" t="str">
-        <v>I am on leave tomorrow (Hospital case)</v>
+        <v>Thomas, Kalady, 9-5</v>
       </c>
       <c r="P141" t="str">
         <v/>
@@ -7934,16 +7945,16 @@
         <v>INTEREXT OFFICE</v>
       </c>
       <c r="F151" t="str">
-        <v>08:14 PM</v>
+        <v>11:16 AM</v>
       </c>
       <c r="G151" t="str">
         <v>10:30 PM</v>
       </c>
       <c r="H151">
-        <v>2.25</v>
+        <v>11.22</v>
       </c>
       <c r="I151">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J151">
         <v>0</v>
@@ -7952,16 +7963,16 @@
         <v>0</v>
       </c>
       <c r="L151">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M151">
         <v>1</v>
       </c>
       <c r="N151">
-        <v>379.69</v>
+        <v>1755</v>
       </c>
       <c r="O151" t="str">
-        <v>Sunil aliyar, Cavili  choondy,  | [System Auto-Checkout: Missed check-out]</v>
+        <v>Sunil aliyar, Cavili choondy,  | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P151" t="str">
         <v/>
@@ -8325,7 +8336,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C159" t="str">
-        <v>AJEESH VIJAYAN</v>
+        <v>Ajeesh Vijayan</v>
       </c>
       <c r="D159" t="str">
         <v>ABSENT</v>
@@ -8525,7 +8536,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C163" t="str">
-        <v>Akhil AK</v>
+        <v>Akhil Ak</v>
       </c>
       <c r="D163" t="str">
         <v>COMPLETED</v>
@@ -8575,7 +8586,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C164" t="str">
-        <v>AKHIL P KUMAR</v>
+        <v>Akhil P Kumar</v>
       </c>
       <c r="D164" t="str">
         <v>ABSENT</v>
@@ -8725,7 +8736,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C167" t="str">
-        <v>ANADHU SUNIL</v>
+        <v>Anadhu Sunil</v>
       </c>
       <c r="D167" t="str">
         <v>ABSENT</v>
@@ -9125,7 +9136,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C175" t="str">
-        <v>Arun P madhu</v>
+        <v>Arun P Madhu</v>
       </c>
       <c r="D175" t="str">
         <v>ABSENT</v>
@@ -9225,7 +9236,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C177" t="str">
-        <v>BINDHU JOSE</v>
+        <v>Bindhu Jose</v>
       </c>
       <c r="D177" t="str">
         <v>ABSENT</v>
@@ -9425,7 +9436,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C181" t="str">
-        <v>GEORGE THOMAS</v>
+        <v>George Thomas</v>
       </c>
       <c r="D181" t="str">
         <v>ABSENT</v>
@@ -9475,7 +9486,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C182" t="str">
-        <v>GOKUL K</v>
+        <v>Gokul K</v>
       </c>
       <c r="D182" t="str">
         <v>ABSENT</v>
@@ -9525,7 +9536,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C183" t="str">
-        <v>Gokul Krishnan  E V</v>
+        <v>Gokul Krishnan E V</v>
       </c>
       <c r="D183" t="str">
         <v>ABSENT</v>
@@ -9575,7 +9586,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C184" t="str">
-        <v>Gopal (soma)</v>
+        <v>Gopal (Soma)</v>
       </c>
       <c r="D184" t="str">
         <v>ABSENT</v>
@@ -9625,7 +9636,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C185" t="str">
-        <v>James TM</v>
+        <v>James Tm</v>
       </c>
       <c r="D185" t="str">
         <v>ABSENT</v>
@@ -9875,10 +9886,10 @@
         <v>Wednesday</v>
       </c>
       <c r="C190" t="str">
-        <v>Mahin KJ</v>
+        <v>Mahin Kj</v>
       </c>
       <c r="D190" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E190" t="str">
         <v>INTEREXT OFFICE</v>
@@ -9887,13 +9898,13 @@
         <v>07:28 AM</v>
       </c>
       <c r="G190" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H190">
-        <v>0</v>
+        <v>15.03</v>
       </c>
       <c r="I190">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J190">
         <v>0</v>
@@ -9908,10 +9919,10 @@
         <v>0</v>
       </c>
       <c r="N190">
-        <v>0</v>
+        <v>1038.46</v>
       </c>
       <c r="O190" t="str">
-        <v>7.28am</v>
+        <v>7.28am | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P190" t="str">
         <v/>
@@ -10025,7 +10036,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C193" t="str">
-        <v>NIJI MANOJ</v>
+        <v>Niji Manoj</v>
       </c>
       <c r="D193" t="str">
         <v>ABSENT</v>
@@ -10125,7 +10136,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C195" t="str">
-        <v>NOURIN SHAJI</v>
+        <v>Nourin Shaji</v>
       </c>
       <c r="D195" t="str">
         <v>ABSENT</v>
@@ -10225,7 +10236,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C197" t="str">
-        <v>PRASANTH E.M</v>
+        <v>Prasanth E.M</v>
       </c>
       <c r="D197" t="str">
         <v>ABSENT</v>
@@ -10275,7 +10286,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C198" t="str">
-        <v>PRATHEESH K S</v>
+        <v>Pratheesh K S</v>
       </c>
       <c r="D198" t="str">
         <v>ABSENT</v>
@@ -10425,7 +10436,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C201" t="str">
-        <v>RAHUL SUNDARAN</v>
+        <v>Rahul Sundaran</v>
       </c>
       <c r="D201" t="str">
         <v>ABSENT</v>
@@ -10525,7 +10536,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C203" t="str">
-        <v>RAJI KANNAN</v>
+        <v>Raji Kannan</v>
       </c>
       <c r="D203" t="str">
         <v>ABSENT</v>
@@ -10825,7 +10836,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C209" t="str">
-        <v>REBEESH K S</v>
+        <v>Rebeesh K S</v>
       </c>
       <c r="D209" t="str">
         <v>ABSENT</v>
@@ -10875,7 +10886,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C210" t="str">
-        <v>REKHA MADHU</v>
+        <v>Rekha Madhu</v>
       </c>
       <c r="D210" t="str">
         <v>ABSENT</v>
@@ -11125,7 +11136,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C215" t="str">
-        <v>SHAHANA JABBAR</v>
+        <v>Shahana Jabbar</v>
       </c>
       <c r="D215" t="str">
         <v>ABSENT</v>
@@ -11175,7 +11186,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C216" t="str">
-        <v>SHINODH N T</v>
+        <v>Shinodh N T</v>
       </c>
       <c r="D216" t="str">
         <v>ABSENT</v>
@@ -11225,7 +11236,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C217" t="str">
-        <v>SHYAM MURALI</v>
+        <v>Shyam Murali</v>
       </c>
       <c r="D217" t="str">
         <v>ABSENT</v>
@@ -12031,7 +12042,7 @@
         <v>COMPLETED</v>
       </c>
       <c r="E233" t="str">
-        <v>Kochi</v>
+        <v>INTEREXT OFFICE</v>
       </c>
       <c r="F233" t="str">
         <v>09:00 AM</v>
@@ -12058,7 +12069,7 @@
         <v>0</v>
       </c>
       <c r="N233">
-        <v>1500</v>
+        <v>1440</v>
       </c>
       <c r="O233" t="str" xml:space="preserve">
         <v xml:space="preserve">Aamil
@@ -12177,13 +12188,13 @@
         <v>Thursday</v>
       </c>
       <c r="C236" t="str">
-        <v>AJEESH VIJAYAN</v>
+        <v>Ajeesh Vijayan</v>
       </c>
       <c r="D236" t="str">
         <v>COMPLETED</v>
       </c>
       <c r="E236" t="str">
-        <v>Office</v>
+        <v>INTEREXT OFFICE</v>
       </c>
       <c r="F236" t="str">
         <v>09:00 AM</v>
@@ -12379,7 +12390,7 @@
         <v>Thursday</v>
       </c>
       <c r="C240" t="str">
-        <v>Akhil AK</v>
+        <v>Akhil Ak</v>
       </c>
       <c r="D240" t="str">
         <v>COMPLETED</v>
@@ -12421,7 +12432,7 @@
         <v/>
       </c>
     </row>
-    <row r="241">
+    <row r="241" xml:space="preserve">
       <c r="A241" t="str">
         <v>2026-05-28</v>
       </c>
@@ -12429,25 +12440,25 @@
         <v>Thursday</v>
       </c>
       <c r="C241" t="str">
-        <v>AKHIL P KUMAR</v>
+        <v>Akhil P Kumar</v>
       </c>
       <c r="D241" t="str">
-        <v>LEAVE</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E241" t="str">
         <v>INTEREXT OFFICE</v>
       </c>
       <c r="F241" t="str">
-        <v>—</v>
+        <v>09:00 AM</v>
       </c>
       <c r="G241" t="str">
-        <v>—</v>
+        <v>06:00 PM</v>
       </c>
       <c r="H241">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I241">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J241">
         <v>0</v>
@@ -12462,10 +12473,12 @@
         <v>0</v>
       </c>
       <c r="N241">
-        <v>0</v>
-      </c>
-      <c r="O241" t="str">
-        <v>I'm on leave friday &amp; saturday</v>
+        <v>1200</v>
+      </c>
+      <c r="O241" t="str" xml:space="preserve">
+        <v xml:space="preserve">Akhil p
+Office 
+9-6</v>
       </c>
       <c r="P241" t="str">
         <v/>
@@ -12579,7 +12592,7 @@
         <v>Thursday</v>
       </c>
       <c r="C244" t="str">
-        <v>ANADHU SUNIL</v>
+        <v>Anadhu Sunil</v>
       </c>
       <c r="D244" t="str">
         <v>ABSENT</v>
@@ -12979,7 +12992,7 @@
         <v>Thursday</v>
       </c>
       <c r="C252" t="str">
-        <v>Arun P madhu</v>
+        <v>Arun P Madhu</v>
       </c>
       <c r="D252" t="str">
         <v>ABSENT</v>
@@ -13079,7 +13092,7 @@
         <v>Thursday</v>
       </c>
       <c r="C254" t="str">
-        <v>BINDHU JOSE</v>
+        <v>Bindhu Jose</v>
       </c>
       <c r="D254" t="str">
         <v>ABSENT</v>
@@ -13279,7 +13292,7 @@
         <v>Thursday</v>
       </c>
       <c r="C258" t="str">
-        <v>GEORGE THOMAS</v>
+        <v>George Thomas</v>
       </c>
       <c r="D258" t="str">
         <v>ABSENT</v>
@@ -13329,7 +13342,7 @@
         <v>Thursday</v>
       </c>
       <c r="C259" t="str">
-        <v>GOKUL K</v>
+        <v>Gokul K</v>
       </c>
       <c r="D259" t="str">
         <v>ABSENT</v>
@@ -13379,7 +13392,7 @@
         <v>Thursday</v>
       </c>
       <c r="C260" t="str">
-        <v>Gokul Krishnan  E V</v>
+        <v>Gokul Krishnan E V</v>
       </c>
       <c r="D260" t="str">
         <v>ABSENT</v>
@@ -13429,7 +13442,7 @@
         <v>Thursday</v>
       </c>
       <c r="C261" t="str">
-        <v>Gopal (soma)</v>
+        <v>Gopal (Soma)</v>
       </c>
       <c r="D261" t="str">
         <v>ABSENT</v>
@@ -13479,7 +13492,7 @@
         <v>Thursday</v>
       </c>
       <c r="C262" t="str">
-        <v>James TM</v>
+        <v>James Tm</v>
       </c>
       <c r="D262" t="str">
         <v>ABSENT</v>
@@ -13729,7 +13742,7 @@
         <v>Thursday</v>
       </c>
       <c r="C267" t="str">
-        <v>Mahin KJ</v>
+        <v>Mahin Kj</v>
       </c>
       <c r="D267" t="str">
         <v>LEAVE</v>
@@ -13879,7 +13892,7 @@
         <v>Thursday</v>
       </c>
       <c r="C270" t="str">
-        <v>NIJI MANOJ</v>
+        <v>Niji Manoj</v>
       </c>
       <c r="D270" t="str">
         <v>ABSENT</v>
@@ -13979,7 +13992,7 @@
         <v>Thursday</v>
       </c>
       <c r="C272" t="str">
-        <v>NOURIN SHAJI</v>
+        <v>Nourin Shaji</v>
       </c>
       <c r="D272" t="str">
         <v>ABSENT</v>
@@ -14079,7 +14092,7 @@
         <v>Thursday</v>
       </c>
       <c r="C274" t="str">
-        <v>PRASANTH E.M</v>
+        <v>Prasanth E.M</v>
       </c>
       <c r="D274" t="str">
         <v>ABSENT</v>
@@ -14129,7 +14142,7 @@
         <v>Thursday</v>
       </c>
       <c r="C275" t="str">
-        <v>PRATHEESH K S</v>
+        <v>Pratheesh K S</v>
       </c>
       <c r="D275" t="str">
         <v>ABSENT</v>
@@ -14279,7 +14292,7 @@
         <v>Thursday</v>
       </c>
       <c r="C278" t="str">
-        <v>RAHUL SUNDARAN</v>
+        <v>Rahul Sundaran</v>
       </c>
       <c r="D278" t="str">
         <v>ABSENT</v>
@@ -14379,7 +14392,7 @@
         <v>Thursday</v>
       </c>
       <c r="C280" t="str">
-        <v>RAJI KANNAN</v>
+        <v>Raji Kannan</v>
       </c>
       <c r="D280" t="str">
         <v>ABSENT</v>
@@ -14679,7 +14692,7 @@
         <v>Thursday</v>
       </c>
       <c r="C286" t="str">
-        <v>REBEESH K S</v>
+        <v>Rebeesh K S</v>
       </c>
       <c r="D286" t="str">
         <v>ABSENT</v>
@@ -14729,7 +14742,7 @@
         <v>Thursday</v>
       </c>
       <c r="C287" t="str">
-        <v>REKHA MADHU</v>
+        <v>Rekha Madhu</v>
       </c>
       <c r="D287" t="str">
         <v>LEAVE</v>
@@ -14979,7 +14992,7 @@
         <v>Thursday</v>
       </c>
       <c r="C292" t="str">
-        <v>SHAHANA JABBAR</v>
+        <v>Shahana Jabbar</v>
       </c>
       <c r="D292" t="str">
         <v>ABSENT</v>
@@ -15029,7 +15042,7 @@
         <v>Thursday</v>
       </c>
       <c r="C293" t="str">
-        <v>SHINODH N T</v>
+        <v>Shinodh N T</v>
       </c>
       <c r="D293" t="str">
         <v>ABSENT</v>
@@ -15079,7 +15092,7 @@
         <v>Thursday</v>
       </c>
       <c r="C294" t="str">
-        <v>SHYAM MURALI</v>
+        <v>Shyam Murali</v>
       </c>
       <c r="D294" t="str">
         <v>ABSENT</v>
@@ -16029,7 +16042,7 @@
         <v>Friday</v>
       </c>
       <c r="C313" t="str">
-        <v>AJEESH VIJAYAN</v>
+        <v>Ajeesh Vijayan</v>
       </c>
       <c r="D313" t="str">
         <v>ABSENT</v>
@@ -16229,7 +16242,7 @@
         <v>Friday</v>
       </c>
       <c r="C317" t="str">
-        <v>Akhil AK</v>
+        <v>Akhil Ak</v>
       </c>
       <c r="D317" t="str">
         <v>ABSENT</v>
@@ -16279,7 +16292,7 @@
         <v>Friday</v>
       </c>
       <c r="C318" t="str">
-        <v>AKHIL P KUMAR</v>
+        <v>Akhil P Kumar</v>
       </c>
       <c r="D318" t="str">
         <v>COMPLETED</v>
@@ -16429,7 +16442,7 @@
         <v>Friday</v>
       </c>
       <c r="C321" t="str">
-        <v>ANADHU SUNIL</v>
+        <v>Anadhu Sunil</v>
       </c>
       <c r="D321" t="str">
         <v>ABSENT</v>
@@ -16588,22 +16601,22 @@
         <v>INTEREXT OFFICE</v>
       </c>
       <c r="F324" t="str">
-        <v>08:11 PM</v>
+        <v>04:46 PM</v>
       </c>
       <c r="G324" t="str">
         <v>10:30 PM</v>
       </c>
       <c r="H324">
-        <v>2.3</v>
+        <v>5.72</v>
       </c>
       <c r="I324">
         <v>0</v>
       </c>
       <c r="J324">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K324">
-        <v>0</v>
+        <v>1.72</v>
       </c>
       <c r="L324">
         <v>0</v>
@@ -16612,7 +16625,7 @@
         <v>1</v>
       </c>
       <c r="N324">
-        <v>301.88</v>
+        <v>750.75</v>
       </c>
       <c r="O324" t="str">
         <v>Anil rana, Cavili choondy,  | [System Auto-Checkout: Missed check-out]</v>
@@ -16829,7 +16842,7 @@
         <v>Friday</v>
       </c>
       <c r="C329" t="str">
-        <v>Arun P madhu</v>
+        <v>Arun P Madhu</v>
       </c>
       <c r="D329" t="str">
         <v>ABSENT</v>
@@ -16929,7 +16942,7 @@
         <v>Friday</v>
       </c>
       <c r="C331" t="str">
-        <v>BINDHU JOSE</v>
+        <v>Bindhu Jose</v>
       </c>
       <c r="D331" t="str">
         <v>ABSENT</v>
@@ -17129,7 +17142,7 @@
         <v>Friday</v>
       </c>
       <c r="C335" t="str">
-        <v>GEORGE THOMAS</v>
+        <v>George Thomas</v>
       </c>
       <c r="D335" t="str">
         <v>ABSENT</v>
@@ -17179,7 +17192,7 @@
         <v>Friday</v>
       </c>
       <c r="C336" t="str">
-        <v>GOKUL K</v>
+        <v>Gokul K</v>
       </c>
       <c r="D336" t="str">
         <v>ABSENT</v>
@@ -17229,7 +17242,7 @@
         <v>Friday</v>
       </c>
       <c r="C337" t="str">
-        <v>Gokul Krishnan  E V</v>
+        <v>Gokul Krishnan E V</v>
       </c>
       <c r="D337" t="str">
         <v>ABSENT</v>
@@ -17279,7 +17292,7 @@
         <v>Friday</v>
       </c>
       <c r="C338" t="str">
-        <v>Gopal (soma)</v>
+        <v>Gopal (Soma)</v>
       </c>
       <c r="D338" t="str">
         <v>ABSENT</v>
@@ -17329,7 +17342,7 @@
         <v>Friday</v>
       </c>
       <c r="C339" t="str">
-        <v>James TM</v>
+        <v>James Tm</v>
       </c>
       <c r="D339" t="str">
         <v>COMPLETED</v>
@@ -17532,25 +17545,25 @@
         <v>M S Arjun</v>
       </c>
       <c r="D343" t="str">
-        <v>ABSENT</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E343" t="str">
-        <v>—</v>
+        <v>INTEREXT OFFICE</v>
       </c>
       <c r="F343" t="str">
-        <v>—</v>
+        <v>02:41 PM</v>
       </c>
       <c r="G343" t="str">
-        <v>—</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H343">
-        <v>0</v>
+        <v>7.82</v>
       </c>
       <c r="I343">
         <v>0</v>
       </c>
       <c r="J343">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K343">
         <v>0</v>
@@ -17562,13 +17575,13 @@
         <v>0</v>
       </c>
       <c r="N343">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="O343" t="str">
-        <v>—</v>
+        <v>http://192.168.2.41:3000/checkin | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P343" t="str">
-        <v>Auto-Marked Absent (Missing text)</v>
+        <v/>
       </c>
     </row>
     <row r="344">
@@ -17579,7 +17592,7 @@
         <v>Friday</v>
       </c>
       <c r="C344" t="str">
-        <v>Mahin KJ</v>
+        <v>Mahin Kj</v>
       </c>
       <c r="D344" t="str">
         <v>COMPLETED</v>
@@ -17729,7 +17742,7 @@
         <v>Friday</v>
       </c>
       <c r="C347" t="str">
-        <v>NIJI MANOJ</v>
+        <v>Niji Manoj</v>
       </c>
       <c r="D347" t="str">
         <v>ABSENT</v>
@@ -17829,7 +17842,7 @@
         <v>Friday</v>
       </c>
       <c r="C349" t="str">
-        <v>NOURIN SHAJI</v>
+        <v>Nourin Shaji</v>
       </c>
       <c r="D349" t="str">
         <v>ABSENT</v>
@@ -17929,7 +17942,7 @@
         <v>Friday</v>
       </c>
       <c r="C351" t="str">
-        <v>PRASANTH E.M</v>
+        <v>Prasanth E.M</v>
       </c>
       <c r="D351" t="str">
         <v>COMPLETED</v>
@@ -17979,7 +17992,7 @@
         <v>Friday</v>
       </c>
       <c r="C352" t="str">
-        <v>PRATHEESH K S</v>
+        <v>Pratheesh K S</v>
       </c>
       <c r="D352" t="str">
         <v>ABSENT</v>
@@ -18129,7 +18142,7 @@
         <v>Friday</v>
       </c>
       <c r="C355" t="str">
-        <v>RAHUL SUNDARAN</v>
+        <v>Rahul Sundaran</v>
       </c>
       <c r="D355" t="str">
         <v>ABSENT</v>
@@ -18229,7 +18242,7 @@
         <v>Friday</v>
       </c>
       <c r="C357" t="str">
-        <v>RAJI KANNAN</v>
+        <v>Raji Kannan</v>
       </c>
       <c r="D357" t="str">
         <v>ABSENT</v>
@@ -18529,7 +18542,7 @@
         <v>Friday</v>
       </c>
       <c r="C363" t="str">
-        <v>REBEESH K S</v>
+        <v>Rebeesh K S</v>
       </c>
       <c r="D363" t="str">
         <v>ABSENT</v>
@@ -18579,7 +18592,7 @@
         <v>Friday</v>
       </c>
       <c r="C364" t="str">
-        <v>REKHA MADHU</v>
+        <v>Rekha Madhu</v>
       </c>
       <c r="D364" t="str">
         <v>ABSENT</v>
@@ -18829,7 +18842,7 @@
         <v>Friday</v>
       </c>
       <c r="C369" t="str">
-        <v>SHAHANA JABBAR</v>
+        <v>Shahana Jabbar</v>
       </c>
       <c r="D369" t="str">
         <v>ABSENT</v>
@@ -18879,7 +18892,7 @@
         <v>Friday</v>
       </c>
       <c r="C370" t="str">
-        <v>SHINODH N T</v>
+        <v>Shinodh N T</v>
       </c>
       <c r="D370" t="str">
         <v>LEAVE</v>
@@ -18929,7 +18942,7 @@
         <v>Friday</v>
       </c>
       <c r="C371" t="str">
-        <v>SHYAM MURALI</v>
+        <v>Shyam Murali</v>
       </c>
       <c r="D371" t="str">
         <v>ABSENT</v>
@@ -19338,22 +19351,22 @@
         <v>INTEREXT OFFICE</v>
       </c>
       <c r="F379" t="str">
-        <v>08:11 PM</v>
+        <v>04:46 PM</v>
       </c>
       <c r="G379" t="str">
         <v>10:30 PM</v>
       </c>
       <c r="H379">
-        <v>2.3</v>
+        <v>5.72</v>
       </c>
       <c r="I379">
         <v>0</v>
       </c>
       <c r="J379">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K379">
-        <v>0</v>
+        <v>1.72</v>
       </c>
       <c r="L379">
         <v>0</v>
@@ -19362,7 +19375,7 @@
         <v>1</v>
       </c>
       <c r="N379">
-        <v>287.5</v>
+        <v>715</v>
       </c>
       <c r="O379" t="str">
         <v>Subodsha, Cavili choondy,  | [System Auto-Checkout: Missed check-out]</v>
@@ -19879,7 +19892,7 @@
         <v>Saturday</v>
       </c>
       <c r="C390" t="str">
-        <v>AJEESH VIJAYAN</v>
+        <v>Ajeesh Vijayan</v>
       </c>
       <c r="D390" t="str">
         <v>ABSENT</v>
@@ -20079,7 +20092,7 @@
         <v>Saturday</v>
       </c>
       <c r="C394" t="str">
-        <v>Akhil AK</v>
+        <v>Akhil Ak</v>
       </c>
       <c r="D394" t="str">
         <v>ABSENT</v>
@@ -20129,7 +20142,7 @@
         <v>Saturday</v>
       </c>
       <c r="C395" t="str">
-        <v>AKHIL P KUMAR</v>
+        <v>Akhil P Kumar</v>
       </c>
       <c r="D395" t="str">
         <v>COMPLETED</v>
@@ -20279,7 +20292,7 @@
         <v>Saturday</v>
       </c>
       <c r="C398" t="str">
-        <v>ANADHU SUNIL</v>
+        <v>Anadhu Sunil</v>
       </c>
       <c r="D398" t="str">
         <v>COMPLETED</v>
@@ -20679,7 +20692,7 @@
         <v>Saturday</v>
       </c>
       <c r="C406" t="str">
-        <v>Arun P madhu</v>
+        <v>Arun P Madhu</v>
       </c>
       <c r="D406" t="str">
         <v>ABSENT</v>
@@ -20779,7 +20792,7 @@
         <v>Saturday</v>
       </c>
       <c r="C408" t="str">
-        <v>BINDHU JOSE</v>
+        <v>Bindhu Jose</v>
       </c>
       <c r="D408" t="str">
         <v>ABSENT</v>
@@ -20979,7 +20992,7 @@
         <v>Saturday</v>
       </c>
       <c r="C412" t="str">
-        <v>GEORGE THOMAS</v>
+        <v>George Thomas</v>
       </c>
       <c r="D412" t="str">
         <v>COMPLETED</v>
@@ -21029,7 +21042,7 @@
         <v>Saturday</v>
       </c>
       <c r="C413" t="str">
-        <v>GOKUL K</v>
+        <v>Gokul K</v>
       </c>
       <c r="D413" t="str">
         <v>ABSENT</v>
@@ -21079,7 +21092,7 @@
         <v>Saturday</v>
       </c>
       <c r="C414" t="str">
-        <v>Gokul Krishnan  E V</v>
+        <v>Gokul Krishnan E V</v>
       </c>
       <c r="D414" t="str">
         <v>ABSENT</v>
@@ -21129,7 +21142,7 @@
         <v>Saturday</v>
       </c>
       <c r="C415" t="str">
-        <v>Gopal (soma)</v>
+        <v>Gopal (Soma)</v>
       </c>
       <c r="D415" t="str">
         <v>ABSENT</v>
@@ -21179,7 +21192,7 @@
         <v>Saturday</v>
       </c>
       <c r="C416" t="str">
-        <v>James TM</v>
+        <v>James Tm</v>
       </c>
       <c r="D416" t="str">
         <v>ABSENT</v>
@@ -21429,7 +21442,7 @@
         <v>Saturday</v>
       </c>
       <c r="C421" t="str">
-        <v>Mahin KJ</v>
+        <v>Mahin Kj</v>
       </c>
       <c r="D421" t="str">
         <v>COMPLETED</v>
@@ -21579,7 +21592,7 @@
         <v>Saturday</v>
       </c>
       <c r="C424" t="str">
-        <v>NIJI MANOJ</v>
+        <v>Niji Manoj</v>
       </c>
       <c r="D424" t="str">
         <v>ABSENT</v>
@@ -21679,7 +21692,7 @@
         <v>Saturday</v>
       </c>
       <c r="C426" t="str">
-        <v>NOURIN SHAJI</v>
+        <v>Nourin Shaji</v>
       </c>
       <c r="D426" t="str">
         <v>ABSENT</v>
@@ -21779,7 +21792,7 @@
         <v>Saturday</v>
       </c>
       <c r="C428" t="str">
-        <v>PRASANTH E.M</v>
+        <v>Prasanth E.M</v>
       </c>
       <c r="D428" t="str">
         <v>COMPLETED</v>
@@ -21829,7 +21842,7 @@
         <v>Saturday</v>
       </c>
       <c r="C429" t="str">
-        <v>PRATHEESH K S</v>
+        <v>Pratheesh K S</v>
       </c>
       <c r="D429" t="str">
         <v>ABSENT</v>
@@ -21979,7 +21992,7 @@
         <v>Saturday</v>
       </c>
       <c r="C432" t="str">
-        <v>RAHUL SUNDARAN</v>
+        <v>Rahul Sundaran</v>
       </c>
       <c r="D432" t="str">
         <v>ABSENT</v>
@@ -22079,7 +22092,7 @@
         <v>Saturday</v>
       </c>
       <c r="C434" t="str">
-        <v>RAJI KANNAN</v>
+        <v>Raji Kannan</v>
       </c>
       <c r="D434" t="str">
         <v>ABSENT</v>
@@ -22379,7 +22392,7 @@
         <v>Saturday</v>
       </c>
       <c r="C440" t="str">
-        <v>REBEESH K S</v>
+        <v>Rebeesh K S</v>
       </c>
       <c r="D440" t="str">
         <v>LEAVE</v>
@@ -22429,7 +22442,7 @@
         <v>Saturday</v>
       </c>
       <c r="C441" t="str">
-        <v>REKHA MADHU</v>
+        <v>Rekha Madhu</v>
       </c>
       <c r="D441" t="str">
         <v>ABSENT</v>
@@ -22679,7 +22692,7 @@
         <v>Saturday</v>
       </c>
       <c r="C446" t="str">
-        <v>SHAHANA JABBAR</v>
+        <v>Shahana Jabbar</v>
       </c>
       <c r="D446" t="str">
         <v>ABSENT</v>
@@ -22729,7 +22742,7 @@
         <v>Saturday</v>
       </c>
       <c r="C447" t="str">
-        <v>SHINODH N T</v>
+        <v>Shinodh N T</v>
       </c>
       <c r="D447" t="str">
         <v>LEAVE</v>
@@ -22779,7 +22792,7 @@
         <v>Saturday</v>
       </c>
       <c r="C448" t="str">
-        <v>SHYAM MURALI</v>
+        <v>Shyam Murali</v>
       </c>
       <c r="D448" t="str">
         <v>ABSENT</v>
@@ -23729,7 +23742,7 @@
         <v>Sunday</v>
       </c>
       <c r="C467" t="str">
-        <v>AJEESH VIJAYAN</v>
+        <v>Ajeesh Vijayan</v>
       </c>
       <c r="D467" t="str">
         <v>ABSENT</v>
@@ -23929,7 +23942,7 @@
         <v>Sunday</v>
       </c>
       <c r="C471" t="str">
-        <v>Akhil AK</v>
+        <v>Akhil Ak</v>
       </c>
       <c r="D471" t="str">
         <v>ABSENT</v>
@@ -23979,7 +23992,7 @@
         <v>Sunday</v>
       </c>
       <c r="C472" t="str">
-        <v>AKHIL P KUMAR</v>
+        <v>Akhil P Kumar</v>
       </c>
       <c r="D472" t="str">
         <v>ABSENT</v>
@@ -24129,7 +24142,7 @@
         <v>Sunday</v>
       </c>
       <c r="C475" t="str">
-        <v>ANADHU SUNIL</v>
+        <v>Anadhu Sunil</v>
       </c>
       <c r="D475" t="str">
         <v>ABSENT</v>
@@ -24529,7 +24542,7 @@
         <v>Sunday</v>
       </c>
       <c r="C483" t="str">
-        <v>Arun P madhu</v>
+        <v>Arun P Madhu</v>
       </c>
       <c r="D483" t="str">
         <v>ABSENT</v>
@@ -24629,7 +24642,7 @@
         <v>Sunday</v>
       </c>
       <c r="C485" t="str">
-        <v>BINDHU JOSE</v>
+        <v>Bindhu Jose</v>
       </c>
       <c r="D485" t="str">
         <v>ABSENT</v>
@@ -24829,7 +24842,7 @@
         <v>Sunday</v>
       </c>
       <c r="C489" t="str">
-        <v>GEORGE THOMAS</v>
+        <v>George Thomas</v>
       </c>
       <c r="D489" t="str">
         <v>ABSENT</v>
@@ -24879,7 +24892,7 @@
         <v>Sunday</v>
       </c>
       <c r="C490" t="str">
-        <v>GOKUL K</v>
+        <v>Gokul K</v>
       </c>
       <c r="D490" t="str">
         <v>ABSENT</v>
@@ -24929,7 +24942,7 @@
         <v>Sunday</v>
       </c>
       <c r="C491" t="str">
-        <v>Gokul Krishnan  E V</v>
+        <v>Gokul Krishnan E V</v>
       </c>
       <c r="D491" t="str">
         <v>ABSENT</v>
@@ -24979,7 +24992,7 @@
         <v>Sunday</v>
       </c>
       <c r="C492" t="str">
-        <v>Gopal (soma)</v>
+        <v>Gopal (Soma)</v>
       </c>
       <c r="D492" t="str">
         <v>ABSENT</v>
@@ -25029,7 +25042,7 @@
         <v>Sunday</v>
       </c>
       <c r="C493" t="str">
-        <v>James TM</v>
+        <v>James Tm</v>
       </c>
       <c r="D493" t="str">
         <v>ABSENT</v>
@@ -25279,7 +25292,7 @@
         <v>Sunday</v>
       </c>
       <c r="C498" t="str">
-        <v>Mahin KJ</v>
+        <v>Mahin Kj</v>
       </c>
       <c r="D498" t="str">
         <v>ABSENT</v>
@@ -25429,7 +25442,7 @@
         <v>Sunday</v>
       </c>
       <c r="C501" t="str">
-        <v>NIJI MANOJ</v>
+        <v>Niji Manoj</v>
       </c>
       <c r="D501" t="str">
         <v>ABSENT</v>
@@ -25529,7 +25542,7 @@
         <v>Sunday</v>
       </c>
       <c r="C503" t="str">
-        <v>NOURIN SHAJI</v>
+        <v>Nourin Shaji</v>
       </c>
       <c r="D503" t="str">
         <v>ABSENT</v>
@@ -25629,7 +25642,7 @@
         <v>Sunday</v>
       </c>
       <c r="C505" t="str">
-        <v>PRASANTH E.M</v>
+        <v>Prasanth E.M</v>
       </c>
       <c r="D505" t="str">
         <v>ABSENT</v>
@@ -25679,7 +25692,7 @@
         <v>Sunday</v>
       </c>
       <c r="C506" t="str">
-        <v>PRATHEESH K S</v>
+        <v>Pratheesh K S</v>
       </c>
       <c r="D506" t="str">
         <v>ABSENT</v>
@@ -25829,7 +25842,7 @@
         <v>Sunday</v>
       </c>
       <c r="C509" t="str">
-        <v>RAHUL SUNDARAN</v>
+        <v>Rahul Sundaran</v>
       </c>
       <c r="D509" t="str">
         <v>ABSENT</v>
@@ -25929,7 +25942,7 @@
         <v>Sunday</v>
       </c>
       <c r="C511" t="str">
-        <v>RAJI KANNAN</v>
+        <v>Raji Kannan</v>
       </c>
       <c r="D511" t="str">
         <v>ABSENT</v>
@@ -26229,7 +26242,7 @@
         <v>Sunday</v>
       </c>
       <c r="C517" t="str">
-        <v>REBEESH K S</v>
+        <v>Rebeesh K S</v>
       </c>
       <c r="D517" t="str">
         <v>ABSENT</v>
@@ -26279,7 +26292,7 @@
         <v>Sunday</v>
       </c>
       <c r="C518" t="str">
-        <v>REKHA MADHU</v>
+        <v>Rekha Madhu</v>
       </c>
       <c r="D518" t="str">
         <v>ABSENT</v>
@@ -26529,7 +26542,7 @@
         <v>Sunday</v>
       </c>
       <c r="C523" t="str">
-        <v>SHAHANA JABBAR</v>
+        <v>Shahana Jabbar</v>
       </c>
       <c r="D523" t="str">
         <v>ABSENT</v>
@@ -26579,7 +26592,7 @@
         <v>Sunday</v>
       </c>
       <c r="C524" t="str">
-        <v>SHINODH N T</v>
+        <v>Shinodh N T</v>
       </c>
       <c r="D524" t="str">
         <v>ABSENT</v>
@@ -26629,7 +26642,7 @@
         <v>Sunday</v>
       </c>
       <c r="C525" t="str">
-        <v>SHYAM MURALI</v>
+        <v>Shyam Murali</v>
       </c>
       <c r="D525" t="str">
         <v>ABSENT</v>
@@ -27421,7 +27434,7 @@
         <v>Auto-Marked Absent (Missing text)</v>
       </c>
     </row>
-    <row r="541">
+    <row r="541" xml:space="preserve">
       <c r="A541" t="str">
         <v>2026-06-01</v>
       </c>
@@ -27464,8 +27477,10 @@
       <c r="N541">
         <v>1320</v>
       </c>
-      <c r="O541" t="str">
-        <v>Aamil, Sumesh Subodsha Anilrana Aneesh (Inter ext office. Quotes) (Provision house), (9-6 pm Chamakkala market)</v>
+      <c r="O541" t="str" xml:space="preserve">
+        <v xml:space="preserve">Aamil
+Thodupuzha 
+9-6</v>
       </c>
       <c r="P541" t="str">
         <v/>
@@ -27581,28 +27596,28 @@
         <v>Monday</v>
       </c>
       <c r="C544" t="str">
-        <v>AJEESH VIJAYAN</v>
+        <v>Ajeesh Vijayan</v>
       </c>
       <c r="D544" t="str">
-        <v>LEAVE</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E544" t="str">
         <v>INTEREXT OFFICE</v>
       </c>
       <c r="F544" t="str">
-        <v>—</v>
+        <v>05:31 PM</v>
       </c>
       <c r="G544" t="str">
-        <v>—</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H544">
-        <v>0</v>
+        <v>4.97</v>
       </c>
       <c r="I544">
         <v>0</v>
       </c>
       <c r="J544">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K544">
         <v>0</v>
@@ -27614,10 +27629,10 @@
         <v>0</v>
       </c>
       <c r="N544">
-        <v>0</v>
+        <v>533.34</v>
       </c>
       <c r="O544" t="str">
-        <v>Completed</v>
+        <v>Ajeesh | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P544" t="str">
         <v/>
@@ -27781,7 +27796,7 @@
         <v>Monday</v>
       </c>
       <c r="C548" t="str">
-        <v>Akhil AK</v>
+        <v>Akhil Ak</v>
       </c>
       <c r="D548" t="str">
         <v>ABSENT</v>
@@ -27831,7 +27846,7 @@
         <v>Monday</v>
       </c>
       <c r="C549" t="str">
-        <v>AKHIL P KUMAR</v>
+        <v>Akhil P Kumar</v>
       </c>
       <c r="D549" t="str">
         <v>COMPLETED</v>
@@ -27981,7 +27996,7 @@
         <v>Monday</v>
       </c>
       <c r="C552" t="str">
-        <v>ANADHU SUNIL</v>
+        <v>Anadhu Sunil</v>
       </c>
       <c r="D552" t="str">
         <v>COMPLETED</v>
@@ -28381,7 +28396,7 @@
         <v>Monday</v>
       </c>
       <c r="C560" t="str">
-        <v>Arun P madhu</v>
+        <v>Arun P Madhu</v>
       </c>
       <c r="D560" t="str">
         <v>ABSENT</v>
@@ -28481,7 +28496,7 @@
         <v>Monday</v>
       </c>
       <c r="C562" t="str">
-        <v>BINDHU JOSE</v>
+        <v>Bindhu Jose</v>
       </c>
       <c r="D562" t="str">
         <v>LEAVE</v>
@@ -28681,7 +28696,7 @@
         <v>Monday</v>
       </c>
       <c r="C566" t="str">
-        <v>GEORGE THOMAS</v>
+        <v>George Thomas</v>
       </c>
       <c r="D566" t="str">
         <v>ABSENT</v>
@@ -28731,7 +28746,7 @@
         <v>Monday</v>
       </c>
       <c r="C567" t="str">
-        <v>GOKUL K</v>
+        <v>Gokul K</v>
       </c>
       <c r="D567" t="str">
         <v>ABSENT</v>
@@ -28781,7 +28796,7 @@
         <v>Monday</v>
       </c>
       <c r="C568" t="str">
-        <v>Gokul Krishnan  E V</v>
+        <v>Gokul Krishnan E V</v>
       </c>
       <c r="D568" t="str">
         <v>ABSENT</v>
@@ -28831,7 +28846,7 @@
         <v>Monday</v>
       </c>
       <c r="C569" t="str">
-        <v>Gopal (soma)</v>
+        <v>Gopal (Soma)</v>
       </c>
       <c r="D569" t="str">
         <v>COMPLETED</v>
@@ -28881,7 +28896,7 @@
         <v>Monday</v>
       </c>
       <c r="C570" t="str">
-        <v>James TM</v>
+        <v>James Tm</v>
       </c>
       <c r="D570" t="str">
         <v>COMPLETED</v>
@@ -29073,7 +29088,7 @@
         <v>Auto-Marked Absent (Missing text)</v>
       </c>
     </row>
-    <row r="574">
+    <row r="574" xml:space="preserve">
       <c r="A574" t="str">
         <v>2026-06-01</v>
       </c>
@@ -29084,22 +29099,22 @@
         <v>M S Arjun</v>
       </c>
       <c r="D574" t="str">
-        <v>LEAVE</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E574" t="str">
         <v>INTEREXT OFFICE</v>
       </c>
       <c r="F574" t="str">
-        <v>—</v>
+        <v>09:00 AM</v>
       </c>
       <c r="G574" t="str">
-        <v>—</v>
+        <v>06:00 PM</v>
       </c>
       <c r="H574">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I574">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J574">
         <v>0</v>
@@ -29114,10 +29129,12 @@
         <v>0</v>
       </c>
       <c r="N574">
-        <v>0</v>
-      </c>
-      <c r="O574" t="str">
-        <v>https://interext-image-collection.vercel.app</v>
+        <v>1000</v>
+      </c>
+      <c r="O574" t="str" xml:space="preserve">
+        <v xml:space="preserve">Abishek
+Office 
+9-6</v>
       </c>
       <c r="P574" t="str">
         <v/>
@@ -29131,7 +29148,7 @@
         <v>Monday</v>
       </c>
       <c r="C575" t="str">
-        <v>Mahin KJ</v>
+        <v>Mahin Kj</v>
       </c>
       <c r="D575" t="str">
         <v>COMPLETED</v>
@@ -29281,7 +29298,7 @@
         <v>Monday</v>
       </c>
       <c r="C578" t="str">
-        <v>NIJI MANOJ</v>
+        <v>Niji Manoj</v>
       </c>
       <c r="D578" t="str">
         <v>LEAVE</v>
@@ -29381,7 +29398,7 @@
         <v>Monday</v>
       </c>
       <c r="C580" t="str">
-        <v>NOURIN SHAJI</v>
+        <v>Nourin Shaji</v>
       </c>
       <c r="D580" t="str">
         <v>LEAVE</v>
@@ -29481,7 +29498,7 @@
         <v>Monday</v>
       </c>
       <c r="C582" t="str">
-        <v>PRASANTH E.M</v>
+        <v>Prasanth E.M</v>
       </c>
       <c r="D582" t="str">
         <v>COMPLETED</v>
@@ -29531,7 +29548,7 @@
         <v>Monday</v>
       </c>
       <c r="C583" t="str">
-        <v>PRATHEESH K S</v>
+        <v>Pratheesh K S</v>
       </c>
       <c r="D583" t="str">
         <v>ABSENT</v>
@@ -29681,7 +29698,7 @@
         <v>Monday</v>
       </c>
       <c r="C586" t="str">
-        <v>RAHUL SUNDARAN</v>
+        <v>Rahul Sundaran</v>
       </c>
       <c r="D586" t="str">
         <v>ABSENT</v>
@@ -29781,7 +29798,7 @@
         <v>Monday</v>
       </c>
       <c r="C588" t="str">
-        <v>RAJI KANNAN</v>
+        <v>Raji Kannan</v>
       </c>
       <c r="D588" t="str">
         <v>LEAVE</v>
@@ -30081,7 +30098,7 @@
         <v>Monday</v>
       </c>
       <c r="C594" t="str">
-        <v>REBEESH K S</v>
+        <v>Rebeesh K S</v>
       </c>
       <c r="D594" t="str">
         <v>ABSENT</v>
@@ -30131,7 +30148,7 @@
         <v>Monday</v>
       </c>
       <c r="C595" t="str">
-        <v>REKHA MADHU</v>
+        <v>Rekha Madhu</v>
       </c>
       <c r="D595" t="str">
         <v>LEAVE</v>
@@ -30381,7 +30398,7 @@
         <v>Monday</v>
       </c>
       <c r="C600" t="str">
-        <v>SHAHANA JABBAR</v>
+        <v>Shahana Jabbar</v>
       </c>
       <c r="D600" t="str">
         <v>COMPLETED</v>
@@ -30431,7 +30448,7 @@
         <v>Monday</v>
       </c>
       <c r="C601" t="str">
-        <v>SHINODH N T</v>
+        <v>Shinodh N T</v>
       </c>
       <c r="D601" t="str">
         <v>LEAVE</v>
@@ -30481,7 +30498,7 @@
         <v>Monday</v>
       </c>
       <c r="C602" t="str">
-        <v>SHYAM MURALI</v>
+        <v>Shyam Murali</v>
       </c>
       <c r="D602" t="str">
         <v>ABSENT</v>
@@ -31431,7 +31448,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C621" t="str">
-        <v>AJEESH VIJAYAN</v>
+        <v>Ajeesh Vijayan</v>
       </c>
       <c r="D621" t="str">
         <v>COMPLETED</v>
@@ -31631,7 +31648,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C625" t="str">
-        <v>Akhil AK</v>
+        <v>Akhil Ak</v>
       </c>
       <c r="D625" t="str">
         <v>ABSENT</v>
@@ -31681,7 +31698,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C626" t="str">
-        <v>AKHIL P KUMAR</v>
+        <v>Akhil P Kumar</v>
       </c>
       <c r="D626" t="str">
         <v>COMPLETED</v>
@@ -31831,7 +31848,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C629" t="str">
-        <v>ANADHU SUNIL</v>
+        <v>Anadhu Sunil</v>
       </c>
       <c r="D629" t="str">
         <v>ABSENT</v>
@@ -32231,7 +32248,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C637" t="str">
-        <v>Arun P madhu</v>
+        <v>Arun P Madhu</v>
       </c>
       <c r="D637" t="str">
         <v>COMPLETED</v>
@@ -32331,7 +32348,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C639" t="str">
-        <v>BINDHU JOSE</v>
+        <v>Bindhu Jose</v>
       </c>
       <c r="D639" t="str">
         <v>COMPLETED</v>
@@ -32531,7 +32548,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C643" t="str">
-        <v>GEORGE THOMAS</v>
+        <v>George Thomas</v>
       </c>
       <c r="D643" t="str">
         <v>COMPLETED</v>
@@ -32581,7 +32598,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C644" t="str">
-        <v>GOKUL K</v>
+        <v>Gokul K</v>
       </c>
       <c r="D644" t="str">
         <v>COMPLETED</v>
@@ -32631,7 +32648,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C645" t="str">
-        <v>Gokul Krishnan  E V</v>
+        <v>Gokul Krishnan E V</v>
       </c>
       <c r="D645" t="str">
         <v>ABSENT</v>
@@ -32681,7 +32698,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C646" t="str">
-        <v>Gopal (soma)</v>
+        <v>Gopal (Soma)</v>
       </c>
       <c r="D646" t="str">
         <v>COMPLETED</v>
@@ -32731,7 +32748,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C647" t="str">
-        <v>James TM</v>
+        <v>James Tm</v>
       </c>
       <c r="D647" t="str">
         <v>COMPLETED</v>
@@ -32981,7 +32998,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C652" t="str">
-        <v>Mahin KJ</v>
+        <v>Mahin Kj</v>
       </c>
       <c r="D652" t="str">
         <v>COMPLETED</v>
@@ -33131,7 +33148,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C655" t="str">
-        <v>NIJI MANOJ</v>
+        <v>Niji Manoj</v>
       </c>
       <c r="D655" t="str">
         <v>COMPLETED</v>
@@ -33231,7 +33248,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C657" t="str">
-        <v>NOURIN SHAJI</v>
+        <v>Nourin Shaji</v>
       </c>
       <c r="D657" t="str">
         <v>ABSENT</v>
@@ -33331,7 +33348,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C659" t="str">
-        <v>PRASANTH E.M</v>
+        <v>Prasanth E.M</v>
       </c>
       <c r="D659" t="str">
         <v>COMPLETED</v>
@@ -33381,7 +33398,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C660" t="str">
-        <v>PRATHEESH K S</v>
+        <v>Pratheesh K S</v>
       </c>
       <c r="D660" t="str">
         <v>COMPLETED</v>
@@ -33531,7 +33548,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C663" t="str">
-        <v>RAHUL SUNDARAN</v>
+        <v>Rahul Sundaran</v>
       </c>
       <c r="D663" t="str">
         <v>COMPLETED</v>
@@ -33631,7 +33648,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C665" t="str">
-        <v>RAJI KANNAN</v>
+        <v>Raji Kannan</v>
       </c>
       <c r="D665" t="str">
         <v>COMPLETED</v>
@@ -33931,7 +33948,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C671" t="str">
-        <v>REBEESH K S</v>
+        <v>Rebeesh K S</v>
       </c>
       <c r="D671" t="str">
         <v>COMPLETED</v>
@@ -33981,7 +33998,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C672" t="str">
-        <v>REKHA MADHU</v>
+        <v>Rekha Madhu</v>
       </c>
       <c r="D672" t="str">
         <v>COMPLETED</v>
@@ -34231,7 +34248,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C677" t="str">
-        <v>SHAHANA JABBAR</v>
+        <v>Shahana Jabbar</v>
       </c>
       <c r="D677" t="str">
         <v>COMPLETED</v>
@@ -34281,7 +34298,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C678" t="str">
-        <v>SHINODH N T</v>
+        <v>Shinodh N T</v>
       </c>
       <c r="D678" t="str">
         <v>COMPLETED</v>
@@ -34331,7 +34348,7 @@
         <v>Tuesday</v>
       </c>
       <c r="C679" t="str">
-        <v>SHYAM MURALI</v>
+        <v>Shyam Murali</v>
       </c>
       <c r="D679" t="str">
         <v>COMPLETED</v>
@@ -35281,7 +35298,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C698" t="str">
-        <v>AJEESH VIJAYAN</v>
+        <v>Ajeesh Vijayan</v>
       </c>
       <c r="D698" t="str">
         <v>COMPLETED</v>
@@ -35481,7 +35498,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C702" t="str">
-        <v>Akhil AK</v>
+        <v>Akhil Ak</v>
       </c>
       <c r="D702" t="str">
         <v>COMPLETED</v>
@@ -35531,7 +35548,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C703" t="str">
-        <v>AKHIL P KUMAR</v>
+        <v>Akhil P Kumar</v>
       </c>
       <c r="D703" t="str">
         <v>COMPLETED</v>
@@ -35681,7 +35698,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C706" t="str">
-        <v>ANADHU SUNIL</v>
+        <v>Anadhu Sunil</v>
       </c>
       <c r="D706" t="str">
         <v>ABSENT</v>
@@ -36081,7 +36098,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C714" t="str">
-        <v>Arun P madhu</v>
+        <v>Arun P Madhu</v>
       </c>
       <c r="D714" t="str">
         <v>ABSENT</v>
@@ -36181,7 +36198,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C716" t="str">
-        <v>BINDHU JOSE</v>
+        <v>Bindhu Jose</v>
       </c>
       <c r="D716" t="str">
         <v>ABSENT</v>
@@ -36381,7 +36398,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C720" t="str">
-        <v>GEORGE THOMAS</v>
+        <v>George Thomas</v>
       </c>
       <c r="D720" t="str">
         <v>COMPLETED</v>
@@ -36431,7 +36448,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C721" t="str">
-        <v>GOKUL K</v>
+        <v>Gokul K</v>
       </c>
       <c r="D721" t="str">
         <v>COMPLETED</v>
@@ -36481,7 +36498,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C722" t="str">
-        <v>Gokul Krishnan  E V</v>
+        <v>Gokul Krishnan E V</v>
       </c>
       <c r="D722" t="str">
         <v>ABSENT</v>
@@ -36531,7 +36548,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C723" t="str">
-        <v>Gopal (soma)</v>
+        <v>Gopal (Soma)</v>
       </c>
       <c r="D723" t="str">
         <v>COMPLETED</v>
@@ -36581,7 +36598,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C724" t="str">
-        <v>James TM</v>
+        <v>James Tm</v>
       </c>
       <c r="D724" t="str">
         <v>COMPLETED</v>
@@ -36831,7 +36848,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C729" t="str">
-        <v>Mahin KJ</v>
+        <v>Mahin Kj</v>
       </c>
       <c r="D729" t="str">
         <v>COMPLETED</v>
@@ -36981,7 +36998,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C732" t="str">
-        <v>NIJI MANOJ</v>
+        <v>Niji Manoj</v>
       </c>
       <c r="D732" t="str">
         <v>COMPLETED</v>
@@ -37081,7 +37098,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C734" t="str">
-        <v>NOURIN SHAJI</v>
+        <v>Nourin Shaji</v>
       </c>
       <c r="D734" t="str">
         <v>COMPLETED</v>
@@ -37181,7 +37198,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C736" t="str">
-        <v>PRASANTH E.M</v>
+        <v>Prasanth E.M</v>
       </c>
       <c r="D736" t="str">
         <v>ABSENT</v>
@@ -37231,7 +37248,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C737" t="str">
-        <v>PRATHEESH K S</v>
+        <v>Pratheesh K S</v>
       </c>
       <c r="D737" t="str">
         <v>ABSENT</v>
@@ -37381,7 +37398,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C740" t="str">
-        <v>RAHUL SUNDARAN</v>
+        <v>Rahul Sundaran</v>
       </c>
       <c r="D740" t="str">
         <v>ABSENT</v>
@@ -37481,7 +37498,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C742" t="str">
-        <v>RAJI KANNAN</v>
+        <v>Raji Kannan</v>
       </c>
       <c r="D742" t="str">
         <v>ABSENT</v>
@@ -37781,7 +37798,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C748" t="str">
-        <v>REBEESH K S</v>
+        <v>Rebeesh K S</v>
       </c>
       <c r="D748" t="str">
         <v>ABSENT</v>
@@ -37831,7 +37848,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C749" t="str">
-        <v>REKHA MADHU</v>
+        <v>Rekha Madhu</v>
       </c>
       <c r="D749" t="str">
         <v>ABSENT</v>
@@ -38081,7 +38098,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C754" t="str">
-        <v>SHAHANA JABBAR</v>
+        <v>Shahana Jabbar</v>
       </c>
       <c r="D754" t="str">
         <v>ABSENT</v>
@@ -38131,7 +38148,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C755" t="str">
-        <v>SHINODH N T</v>
+        <v>Shinodh N T</v>
       </c>
       <c r="D755" t="str">
         <v>ABSENT</v>
@@ -38181,7 +38198,7 @@
         <v>Wednesday</v>
       </c>
       <c r="C756" t="str">
-        <v>SHYAM MURALI</v>
+        <v>Shyam Murali</v>
       </c>
       <c r="D756" t="str">
         <v>ABSENT</v>
@@ -39131,7 +39148,7 @@
         <v>Thursday</v>
       </c>
       <c r="C775" t="str">
-        <v>AJEESH VIJAYAN</v>
+        <v>Ajeesh Vijayan</v>
       </c>
       <c r="D775" t="str">
         <v>ABSENT</v>
@@ -39331,7 +39348,7 @@
         <v>Thursday</v>
       </c>
       <c r="C779" t="str">
-        <v>Akhil AK</v>
+        <v>Akhil Ak</v>
       </c>
       <c r="D779" t="str">
         <v>ABSENT</v>
@@ -39381,7 +39398,7 @@
         <v>Thursday</v>
       </c>
       <c r="C780" t="str">
-        <v>AKHIL P KUMAR</v>
+        <v>Akhil P Kumar</v>
       </c>
       <c r="D780" t="str">
         <v>ABSENT</v>
@@ -39531,7 +39548,7 @@
         <v>Thursday</v>
       </c>
       <c r="C783" t="str">
-        <v>ANADHU SUNIL</v>
+        <v>Anadhu Sunil</v>
       </c>
       <c r="D783" t="str">
         <v>ABSENT</v>
@@ -39931,7 +39948,7 @@
         <v>Thursday</v>
       </c>
       <c r="C791" t="str">
-        <v>Arun P madhu</v>
+        <v>Arun P Madhu</v>
       </c>
       <c r="D791" t="str">
         <v>ABSENT</v>
@@ -40031,7 +40048,7 @@
         <v>Thursday</v>
       </c>
       <c r="C793" t="str">
-        <v>BINDHU JOSE</v>
+        <v>Bindhu Jose</v>
       </c>
       <c r="D793" t="str">
         <v>ABSENT</v>
@@ -40231,7 +40248,7 @@
         <v>Thursday</v>
       </c>
       <c r="C797" t="str">
-        <v>GEORGE THOMAS</v>
+        <v>George Thomas</v>
       </c>
       <c r="D797" t="str">
         <v>ABSENT</v>
@@ -40281,7 +40298,7 @@
         <v>Thursday</v>
       </c>
       <c r="C798" t="str">
-        <v>GOKUL K</v>
+        <v>Gokul K</v>
       </c>
       <c r="D798" t="str">
         <v>ABSENT</v>
@@ -40331,7 +40348,7 @@
         <v>Thursday</v>
       </c>
       <c r="C799" t="str">
-        <v>Gokul Krishnan  E V</v>
+        <v>Gokul Krishnan E V</v>
       </c>
       <c r="D799" t="str">
         <v>ABSENT</v>
@@ -40381,7 +40398,7 @@
         <v>Thursday</v>
       </c>
       <c r="C800" t="str">
-        <v>Gopal (soma)</v>
+        <v>Gopal (Soma)</v>
       </c>
       <c r="D800" t="str">
         <v>ABSENT</v>
@@ -40431,7 +40448,7 @@
         <v>Thursday</v>
       </c>
       <c r="C801" t="str">
-        <v>James TM</v>
+        <v>James Tm</v>
       </c>
       <c r="D801" t="str">
         <v>ABSENT</v>
@@ -40681,7 +40698,7 @@
         <v>Thursday</v>
       </c>
       <c r="C806" t="str">
-        <v>Mahin KJ</v>
+        <v>Mahin Kj</v>
       </c>
       <c r="D806" t="str">
         <v>COMPLETED</v>
@@ -40831,7 +40848,7 @@
         <v>Thursday</v>
       </c>
       <c r="C809" t="str">
-        <v>NIJI MANOJ</v>
+        <v>Niji Manoj</v>
       </c>
       <c r="D809" t="str">
         <v>ABSENT</v>
@@ -40931,7 +40948,7 @@
         <v>Thursday</v>
       </c>
       <c r="C811" t="str">
-        <v>NOURIN SHAJI</v>
+        <v>Nourin Shaji</v>
       </c>
       <c r="D811" t="str">
         <v>ABSENT</v>
@@ -41031,7 +41048,7 @@
         <v>Thursday</v>
       </c>
       <c r="C813" t="str">
-        <v>PRASANTH E.M</v>
+        <v>Prasanth E.M</v>
       </c>
       <c r="D813" t="str">
         <v>ABSENT</v>
@@ -41081,7 +41098,7 @@
         <v>Thursday</v>
       </c>
       <c r="C814" t="str">
-        <v>PRATHEESH K S</v>
+        <v>Pratheesh K S</v>
       </c>
       <c r="D814" t="str">
         <v>ABSENT</v>
@@ -41231,7 +41248,7 @@
         <v>Thursday</v>
       </c>
       <c r="C817" t="str">
-        <v>RAHUL SUNDARAN</v>
+        <v>Rahul Sundaran</v>
       </c>
       <c r="D817" t="str">
         <v>ABSENT</v>
@@ -41331,7 +41348,7 @@
         <v>Thursday</v>
       </c>
       <c r="C819" t="str">
-        <v>RAJI KANNAN</v>
+        <v>Raji Kannan</v>
       </c>
       <c r="D819" t="str">
         <v>ABSENT</v>
@@ -41631,7 +41648,7 @@
         <v>Thursday</v>
       </c>
       <c r="C825" t="str">
-        <v>REBEESH K S</v>
+        <v>Rebeesh K S</v>
       </c>
       <c r="D825" t="str">
         <v>ABSENT</v>
@@ -41681,7 +41698,7 @@
         <v>Thursday</v>
       </c>
       <c r="C826" t="str">
-        <v>REKHA MADHU</v>
+        <v>Rekha Madhu</v>
       </c>
       <c r="D826" t="str">
         <v>ABSENT</v>
@@ -41931,7 +41948,7 @@
         <v>Thursday</v>
       </c>
       <c r="C831" t="str">
-        <v>SHAHANA JABBAR</v>
+        <v>Shahana Jabbar</v>
       </c>
       <c r="D831" t="str">
         <v>COMPLETED</v>
@@ -41981,7 +41998,7 @@
         <v>Thursday</v>
       </c>
       <c r="C832" t="str">
-        <v>SHINODH N T</v>
+        <v>Shinodh N T</v>
       </c>
       <c r="D832" t="str">
         <v>ABSENT</v>
@@ -42031,7 +42048,7 @@
         <v>Thursday</v>
       </c>
       <c r="C833" t="str">
-        <v>SHYAM MURALI</v>
+        <v>Shyam Murali</v>
       </c>
       <c r="D833" t="str">
         <v>ABSENT</v>
@@ -42981,7 +42998,7 @@
         <v>Friday</v>
       </c>
       <c r="C852" t="str">
-        <v>AJEESH VIJAYAN</v>
+        <v>Ajeesh Vijayan</v>
       </c>
       <c r="D852" t="str">
         <v>ABSENT</v>
@@ -43181,7 +43198,7 @@
         <v>Friday</v>
       </c>
       <c r="C856" t="str">
-        <v>Akhil AK</v>
+        <v>Akhil Ak</v>
       </c>
       <c r="D856" t="str">
         <v>COMPLETED</v>
@@ -43231,7 +43248,7 @@
         <v>Friday</v>
       </c>
       <c r="C857" t="str">
-        <v>AKHIL P KUMAR</v>
+        <v>Akhil P Kumar</v>
       </c>
       <c r="D857" t="str">
         <v>COMPLETED</v>
@@ -43240,13 +43257,13 @@
         <v>INTEREXT OFFICE</v>
       </c>
       <c r="F857" t="str">
-        <v>10:00 AM</v>
+        <v>09:00 AM</v>
       </c>
       <c r="G857" t="str">
-        <v>10:30 PM</v>
+        <v>06:00 PM</v>
       </c>
       <c r="H857">
-        <v>12.5</v>
+        <v>9</v>
       </c>
       <c r="I857">
         <v>1</v>
@@ -43267,7 +43284,7 @@
         <v>1200</v>
       </c>
       <c r="O857" t="str">
-        <v>I am 1 hr late to reach office today | [System Auto-Checkout: Missed check-out]</v>
+        <v>Akhil, Provision house Kothamangalam, 9 to 6</v>
       </c>
       <c r="P857" t="str">
         <v/>
@@ -43381,7 +43398,7 @@
         <v>Friday</v>
       </c>
       <c r="C860" t="str">
-        <v>ANADHU SUNIL</v>
+        <v>Anadhu Sunil</v>
       </c>
       <c r="D860" t="str">
         <v>ABSENT</v>
@@ -43781,7 +43798,7 @@
         <v>Friday</v>
       </c>
       <c r="C868" t="str">
-        <v>Arun P madhu</v>
+        <v>Arun P Madhu</v>
       </c>
       <c r="D868" t="str">
         <v>ABSENT</v>
@@ -43881,7 +43898,7 @@
         <v>Friday</v>
       </c>
       <c r="C870" t="str">
-        <v>BINDHU JOSE</v>
+        <v>Bindhu Jose</v>
       </c>
       <c r="D870" t="str">
         <v>ABSENT</v>
@@ -44081,7 +44098,7 @@
         <v>Friday</v>
       </c>
       <c r="C874" t="str">
-        <v>GEORGE THOMAS</v>
+        <v>George Thomas</v>
       </c>
       <c r="D874" t="str">
         <v>ABSENT</v>
@@ -44131,7 +44148,7 @@
         <v>Friday</v>
       </c>
       <c r="C875" t="str">
-        <v>GOKUL K</v>
+        <v>Gokul K</v>
       </c>
       <c r="D875" t="str">
         <v>ABSENT</v>
@@ -44181,7 +44198,7 @@
         <v>Friday</v>
       </c>
       <c r="C876" t="str">
-        <v>Gokul Krishnan  E V</v>
+        <v>Gokul Krishnan E V</v>
       </c>
       <c r="D876" t="str">
         <v>ABSENT</v>
@@ -44231,7 +44248,7 @@
         <v>Friday</v>
       </c>
       <c r="C877" t="str">
-        <v>Gopal (soma)</v>
+        <v>Gopal (Soma)</v>
       </c>
       <c r="D877" t="str">
         <v>ABSENT</v>
@@ -44281,7 +44298,7 @@
         <v>Friday</v>
       </c>
       <c r="C878" t="str">
-        <v>James TM</v>
+        <v>James Tm</v>
       </c>
       <c r="D878" t="str">
         <v>ABSENT</v>
@@ -44531,7 +44548,7 @@
         <v>Friday</v>
       </c>
       <c r="C883" t="str">
-        <v>Mahin KJ</v>
+        <v>Mahin Kj</v>
       </c>
       <c r="D883" t="str">
         <v>COMPLETED</v>
@@ -44681,7 +44698,7 @@
         <v>Friday</v>
       </c>
       <c r="C886" t="str">
-        <v>NIJI MANOJ</v>
+        <v>Niji Manoj</v>
       </c>
       <c r="D886" t="str">
         <v>LEAVE</v>
@@ -44781,7 +44798,7 @@
         <v>Friday</v>
       </c>
       <c r="C888" t="str">
-        <v>NOURIN SHAJI</v>
+        <v>Nourin Shaji</v>
       </c>
       <c r="D888" t="str">
         <v>ABSENT</v>
@@ -44881,7 +44898,7 @@
         <v>Friday</v>
       </c>
       <c r="C890" t="str">
-        <v>PRASANTH E.M</v>
+        <v>Prasanth E.M</v>
       </c>
       <c r="D890" t="str">
         <v>ABSENT</v>
@@ -44931,7 +44948,7 @@
         <v>Friday</v>
       </c>
       <c r="C891" t="str">
-        <v>PRATHEESH K S</v>
+        <v>Pratheesh K S</v>
       </c>
       <c r="D891" t="str">
         <v>ABSENT</v>
@@ -45081,7 +45098,7 @@
         <v>Friday</v>
       </c>
       <c r="C894" t="str">
-        <v>RAHUL SUNDARAN</v>
+        <v>Rahul Sundaran</v>
       </c>
       <c r="D894" t="str">
         <v>ABSENT</v>
@@ -45181,7 +45198,7 @@
         <v>Friday</v>
       </c>
       <c r="C896" t="str">
-        <v>RAJI KANNAN</v>
+        <v>Raji Kannan</v>
       </c>
       <c r="D896" t="str">
         <v>ABSENT</v>
@@ -45481,7 +45498,7 @@
         <v>Friday</v>
       </c>
       <c r="C902" t="str">
-        <v>REBEESH K S</v>
+        <v>Rebeesh K S</v>
       </c>
       <c r="D902" t="str">
         <v>ABSENT</v>
@@ -45531,7 +45548,7 @@
         <v>Friday</v>
       </c>
       <c r="C903" t="str">
-        <v>REKHA MADHU</v>
+        <v>Rekha Madhu</v>
       </c>
       <c r="D903" t="str">
         <v>ABSENT</v>
@@ -45781,7 +45798,7 @@
         <v>Friday</v>
       </c>
       <c r="C908" t="str">
-        <v>SHAHANA JABBAR</v>
+        <v>Shahana Jabbar</v>
       </c>
       <c r="D908" t="str">
         <v>ABSENT</v>
@@ -45831,7 +45848,7 @@
         <v>Friday</v>
       </c>
       <c r="C909" t="str">
-        <v>SHINODH N T</v>
+        <v>Shinodh N T</v>
       </c>
       <c r="D909" t="str">
         <v>ABSENT</v>
@@ -45881,7 +45898,7 @@
         <v>Friday</v>
       </c>
       <c r="C910" t="str">
-        <v>SHYAM MURALI</v>
+        <v>Shyam Murali</v>
       </c>
       <c r="D910" t="str">
         <v>ABSENT</v>
@@ -46484,22 +46501,22 @@
         <v>Sunil Rana</v>
       </c>
       <c r="D922" t="str">
-        <v>ABSENT</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E922" t="str">
-        <v>—</v>
+        <v>INTEREXT OFFICE</v>
       </c>
       <c r="F922" t="str">
-        <v>—</v>
+        <v>09:00 AM</v>
       </c>
       <c r="G922" t="str">
-        <v>—</v>
+        <v>06:00 PM</v>
       </c>
       <c r="H922">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I922">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J922">
         <v>0</v>
@@ -46508,19 +46525,19 @@
         <v>0</v>
       </c>
       <c r="L922">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M922">
         <v>0</v>
       </c>
       <c r="N922">
-        <v>0</v>
+        <v>1320</v>
       </c>
       <c r="O922" t="str">
-        <v>—</v>
+        <v>Sunilrana, Provision house Kothamangalam, 9 to 6</v>
       </c>
       <c r="P922" t="str">
-        <v>Auto-Marked Absent (Missing text)</v>
+        <v/>
       </c>
     </row>
     <row r="923">
@@ -46634,22 +46651,22 @@
         <v>Vijesh A V</v>
       </c>
       <c r="D925" t="str">
-        <v>ABSENT</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E925" t="str">
-        <v>—</v>
+        <v>INTEREXT OFFICE</v>
       </c>
       <c r="F925" t="str">
-        <v>—</v>
+        <v>09:00 AM</v>
       </c>
       <c r="G925" t="str">
-        <v>—</v>
+        <v>06:00 PM</v>
       </c>
       <c r="H925">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I925">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J925">
         <v>0</v>
@@ -46664,13 +46681,13 @@
         <v>0</v>
       </c>
       <c r="N925">
-        <v>0</v>
+        <v>1153.85</v>
       </c>
       <c r="O925" t="str">
-        <v>—</v>
+        <v>Vijesh A V, Provision house Kothamangalam, 9 to 6</v>
       </c>
       <c r="P925" t="str">
-        <v>Auto-Marked Absent (Missing text)</v>
+        <v/>
       </c>
     </row>
     <row r="926">
@@ -46831,7 +46848,7 @@
         <v>Saturday</v>
       </c>
       <c r="C929" t="str">
-        <v>AJEESH VIJAYAN</v>
+        <v>Ajeesh Vijayan</v>
       </c>
       <c r="D929" t="str">
         <v>ABSENT</v>
@@ -47031,7 +47048,7 @@
         <v>Saturday</v>
       </c>
       <c r="C933" t="str">
-        <v>Akhil AK</v>
+        <v>Akhil Ak</v>
       </c>
       <c r="D933" t="str">
         <v>ABSENT</v>
@@ -47081,7 +47098,7 @@
         <v>Saturday</v>
       </c>
       <c r="C934" t="str">
-        <v>AKHIL P KUMAR</v>
+        <v>Akhil P Kumar</v>
       </c>
       <c r="D934" t="str">
         <v>ABSENT</v>
@@ -47231,7 +47248,7 @@
         <v>Saturday</v>
       </c>
       <c r="C937" t="str">
-        <v>ANADHU SUNIL</v>
+        <v>Anadhu Sunil</v>
       </c>
       <c r="D937" t="str">
         <v>ABSENT</v>
@@ -47631,7 +47648,7 @@
         <v>Saturday</v>
       </c>
       <c r="C945" t="str">
-        <v>Arun P madhu</v>
+        <v>Arun P Madhu</v>
       </c>
       <c r="D945" t="str">
         <v>ABSENT</v>
@@ -47731,7 +47748,7 @@
         <v>Saturday</v>
       </c>
       <c r="C947" t="str">
-        <v>BINDHU JOSE</v>
+        <v>Bindhu Jose</v>
       </c>
       <c r="D947" t="str">
         <v>ABSENT</v>
@@ -47931,7 +47948,7 @@
         <v>Saturday</v>
       </c>
       <c r="C951" t="str">
-        <v>GEORGE THOMAS</v>
+        <v>George Thomas</v>
       </c>
       <c r="D951" t="str">
         <v>ABSENT</v>
@@ -47981,7 +47998,7 @@
         <v>Saturday</v>
       </c>
       <c r="C952" t="str">
-        <v>GOKUL K</v>
+        <v>Gokul K</v>
       </c>
       <c r="D952" t="str">
         <v>ABSENT</v>
@@ -48031,7 +48048,7 @@
         <v>Saturday</v>
       </c>
       <c r="C953" t="str">
-        <v>Gokul Krishnan  E V</v>
+        <v>Gokul Krishnan E V</v>
       </c>
       <c r="D953" t="str">
         <v>ABSENT</v>
@@ -48081,7 +48098,7 @@
         <v>Saturday</v>
       </c>
       <c r="C954" t="str">
-        <v>Gopal (soma)</v>
+        <v>Gopal (Soma)</v>
       </c>
       <c r="D954" t="str">
         <v>ABSENT</v>
@@ -48131,7 +48148,7 @@
         <v>Saturday</v>
       </c>
       <c r="C955" t="str">
-        <v>James TM</v>
+        <v>James Tm</v>
       </c>
       <c r="D955" t="str">
         <v>LEAVE</v>
@@ -48381,7 +48398,7 @@
         <v>Saturday</v>
       </c>
       <c r="C960" t="str">
-        <v>Mahin KJ</v>
+        <v>Mahin Kj</v>
       </c>
       <c r="D960" t="str">
         <v>CHECKED-IN</v>
@@ -48531,7 +48548,7 @@
         <v>Saturday</v>
       </c>
       <c r="C963" t="str">
-        <v>NIJI MANOJ</v>
+        <v>Niji Manoj</v>
       </c>
       <c r="D963" t="str">
         <v>ABSENT</v>
@@ -48631,7 +48648,7 @@
         <v>Saturday</v>
       </c>
       <c r="C965" t="str">
-        <v>NOURIN SHAJI</v>
+        <v>Nourin Shaji</v>
       </c>
       <c r="D965" t="str">
         <v>ABSENT</v>
@@ -48731,7 +48748,7 @@
         <v>Saturday</v>
       </c>
       <c r="C967" t="str">
-        <v>PRASANTH E.M</v>
+        <v>Prasanth E.M</v>
       </c>
       <c r="D967" t="str">
         <v>CHECKED-IN</v>
@@ -48781,7 +48798,7 @@
         <v>Saturday</v>
       </c>
       <c r="C968" t="str">
-        <v>PRATHEESH K S</v>
+        <v>Pratheesh K S</v>
       </c>
       <c r="D968" t="str">
         <v>CHECKED-IN</v>
@@ -48931,19 +48948,19 @@
         <v>Saturday</v>
       </c>
       <c r="C971" t="str">
-        <v>RAHUL SUNDARAN</v>
+        <v>Rahul Sundaran</v>
       </c>
       <c r="D971" t="str">
-        <v>ABSENT</v>
+        <v>CHECKED-IN</v>
       </c>
       <c r="E971" t="str">
-        <v>—</v>
+        <v>INTEREXT OFFICE</v>
       </c>
       <c r="F971" t="str">
-        <v>—</v>
+        <v>09:00 AM</v>
       </c>
       <c r="G971" t="str">
-        <v>—</v>
+        <v>Currently Checked-In</v>
       </c>
       <c r="H971">
         <v>0</v>
@@ -48970,7 +48987,7 @@
         <v>—</v>
       </c>
       <c r="P971" t="str">
-        <v>Auto-Marked Absent (Missing text)</v>
+        <v/>
       </c>
     </row>
     <row r="972">
@@ -49031,7 +49048,7 @@
         <v>Saturday</v>
       </c>
       <c r="C973" t="str">
-        <v>RAJI KANNAN</v>
+        <v>Raji Kannan</v>
       </c>
       <c r="D973" t="str">
         <v>ABSENT</v>
@@ -49331,7 +49348,7 @@
         <v>Saturday</v>
       </c>
       <c r="C979" t="str">
-        <v>REBEESH K S</v>
+        <v>Rebeesh K S</v>
       </c>
       <c r="D979" t="str">
         <v>ABSENT</v>
@@ -49381,7 +49398,7 @@
         <v>Saturday</v>
       </c>
       <c r="C980" t="str">
-        <v>REKHA MADHU</v>
+        <v>Rekha Madhu</v>
       </c>
       <c r="D980" t="str">
         <v>ABSENT</v>
@@ -49631,7 +49648,7 @@
         <v>Saturday</v>
       </c>
       <c r="C985" t="str">
-        <v>SHAHANA JABBAR</v>
+        <v>Shahana Jabbar</v>
       </c>
       <c r="D985" t="str">
         <v>ABSENT</v>
@@ -49681,7 +49698,7 @@
         <v>Saturday</v>
       </c>
       <c r="C986" t="str">
-        <v>SHINODH N T</v>
+        <v>Shinodh N T</v>
       </c>
       <c r="D986" t="str">
         <v>ABSENT</v>
@@ -49731,7 +49748,7 @@
         <v>Saturday</v>
       </c>
       <c r="C987" t="str">
-        <v>SHYAM MURALI</v>
+        <v>Shyam Murali</v>
       </c>
       <c r="D987" t="str">
         <v>ABSENT</v>
@@ -49884,16 +49901,16 @@
         <v>Sona Francis</v>
       </c>
       <c r="D990" t="str">
-        <v>CHECKED-IN</v>
+        <v>LEAVE</v>
       </c>
       <c r="E990" t="str">
         <v>INTEREXT OFFICE</v>
       </c>
       <c r="F990" t="str">
-        <v>09:30 AM</v>
+        <v>—</v>
       </c>
       <c r="G990" t="str">
-        <v>Currently Checked-In</v>
+        <v>—</v>
       </c>
       <c r="H990">
         <v>0</v>
@@ -49917,7 +49934,7 @@
         <v>0</v>
       </c>
       <c r="O990" t="str">
-        <v>I'm half hour late to reach office</v>
+        <v>I'm on leave afternoon session</v>
       </c>
       <c r="P990" t="str">
         <v/>
@@ -50384,16 +50401,16 @@
         <v>Sunil. C. M</v>
       </c>
       <c r="D1000" t="str">
-        <v>ABSENT</v>
+        <v>CHECKED-IN</v>
       </c>
       <c r="E1000" t="str">
-        <v>—</v>
+        <v>INTEREXT OFFICE</v>
       </c>
       <c r="F1000" t="str">
-        <v>—</v>
+        <v>09:30 AM</v>
       </c>
       <c r="G1000" t="str">
-        <v>—</v>
+        <v>Currently Checked-In</v>
       </c>
       <c r="H1000">
         <v>0</v>
@@ -50417,10 +50434,10 @@
         <v>0</v>
       </c>
       <c r="O1000" t="str">
-        <v>—</v>
+        <v>[RESOLVED] Selfie verification pending admin approval</v>
       </c>
       <c r="P1000" t="str">
-        <v>Auto-Marked Absent (Missing text)</v>
+        <v/>
       </c>
     </row>
     <row r="1001">

</xml_diff>

<commit_message>
fix: restore correct check-out time and full-day calculations for M S Arjun
</commit_message>
<xml_diff>
--- a/Attendance_Payroll.xlsx
+++ b/Attendance_Payroll.xlsx
@@ -48351,22 +48351,22 @@
         <v>M S Arjun</v>
       </c>
       <c r="D959" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E959" t="str">
-        <v>INTEREXT OFFICE</v>
+        <v/>
       </c>
       <c r="F959" t="str">
         <v>09:00 AM</v>
       </c>
       <c r="G959" t="str">
-        <v>Currently Checked-In</v>
+        <v>06:00 PM</v>
       </c>
       <c r="H959">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I959">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J959">
         <v>0</v>
@@ -48381,10 +48381,10 @@
         <v>0</v>
       </c>
       <c r="N959">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="O959" t="str">
-        <v>Face recognized - auto entry</v>
+        <v>Face recognized - auto exit</v>
       </c>
       <c r="P959" t="str">
         <v>Face recognized</v>

</xml_diff>

<commit_message>
chore: update database records and payroll calculations
</commit_message>
<xml_diff>
--- a/Attendance_Payroll.xlsx
+++ b/Attendance_Payroll.xlsx
@@ -54901,16 +54901,16 @@
         <v>Alex Rajan</v>
       </c>
       <c r="D1090" t="str">
-        <v>LEAVE</v>
+        <v>CHECKED-IN</v>
       </c>
       <c r="E1090" t="str">
-        <v>INTEREXT OFFICE</v>
+        <v>Webcam Scan</v>
       </c>
       <c r="F1090" t="str">
-        <v>—</v>
+        <v>01:16 PM</v>
       </c>
       <c r="G1090" t="str">
-        <v>—</v>
+        <v>Currently Checked-In</v>
       </c>
       <c r="H1090">
         <v>0</v>
@@ -54934,7 +54934,7 @@
         <v>0</v>
       </c>
       <c r="O1090" t="str">
-        <v>Today i am half day leave due to sickness</v>
+        <v>Face recognized - auto entry</v>
       </c>
       <c r="P1090" t="str">
         <v/>
@@ -55051,7 +55051,7 @@
         <v>Aneesh Ahammed</v>
       </c>
       <c r="D1093" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E1093" t="str">
         <v>INTEREXT OFFICE</v>
@@ -55060,13 +55060,13 @@
         <v>08:35 AM</v>
       </c>
       <c r="G1093" t="str">
-        <v>Currently Checked-In</v>
+        <v>06:00 PM</v>
       </c>
       <c r="H1093">
-        <v>0</v>
+        <v>9.42</v>
       </c>
       <c r="I1093">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J1093">
         <v>0</v>
@@ -55075,13 +55075,13 @@
         <v>0</v>
       </c>
       <c r="L1093">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M1093">
         <v>0</v>
       </c>
       <c r="N1093">
-        <v>0</v>
+        <v>1210</v>
       </c>
       <c r="O1093" t="str">
         <v>8:35AM</v>
@@ -55154,7 +55154,7 @@
         <v>ABSENT</v>
       </c>
       <c r="E1095" t="str">
-        <v>—</v>
+        <v/>
       </c>
       <c r="F1095" t="str">
         <v>—</v>
@@ -55184,10 +55184,10 @@
         <v>0</v>
       </c>
       <c r="O1095" t="str">
-        <v>—</v>
+        <v>Face recognized - auto lunch-out</v>
       </c>
       <c r="P1095" t="str">
-        <v>Auto-Marked Absent (Missing text)</v>
+        <v>Face recognized</v>
       </c>
     </row>
     <row r="1096">

</xml_diff>

<commit_message>
Update payroll data, CCTV processor, and backend APIs
</commit_message>
<xml_diff>
--- a/Attendance_Payroll.xlsx
+++ b/Attendance_Payroll.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P1369"/>
+  <dimension ref="A1:P1445"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="13.83203125" customWidth="1"/>
@@ -49401,22 +49401,22 @@
         <v>Sreeraj V S</v>
       </c>
       <c r="D980" t="str">
-        <v>ABSENT</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E980" t="str">
-        <v>—</v>
+        <v>INTEREXT OFFICE</v>
       </c>
       <c r="F980" t="str">
-        <v>—</v>
+        <v>09:00 AM</v>
       </c>
       <c r="G980" t="str">
-        <v>—</v>
+        <v>06:00 PM</v>
       </c>
       <c r="H980">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I980">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J980">
         <v>0</v>
@@ -49425,19 +49425,19 @@
         <v>0</v>
       </c>
       <c r="L980">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M980">
         <v>0</v>
       </c>
       <c r="N980">
-        <v>0</v>
+        <v>1155</v>
       </c>
       <c r="O980" t="str">
-        <v>—</v>
+        <v>Sreeraj, —, (9-6 pm pearl royal)</v>
       </c>
       <c r="P980" t="str">
-        <v>Auto-Marked Absent (Missing text)</v>
+        <v/>
       </c>
     </row>
     <row r="981">
@@ -65554,16 +65554,16 @@
         <v>EARLY CHECK-OUT</v>
       </c>
       <c r="E1303" t="str">
-        <v>Webcam Scan</v>
+        <v>Main Gate</v>
       </c>
       <c r="F1303" t="str">
-        <v>12:32 PM</v>
+        <v>05:55 PM</v>
       </c>
       <c r="G1303" t="str">
         <v>12:34 PM</v>
       </c>
       <c r="H1303">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="I1303">
         <v>0</v>
@@ -65581,10 +65581,10 @@
         <v>0</v>
       </c>
       <c r="N1303">
-        <v>1.63</v>
+        <v>0</v>
       </c>
       <c r="O1303" t="str">
-        <v>Face recognized - auto exit</v>
+        <v>Face recognized - auto exit | CCTV Face recognized - auto entry</v>
       </c>
       <c r="P1303" t="str">
         <v>Face recognized</v>
@@ -65751,19 +65751,19 @@
         <v>Aneesh Ahammed</v>
       </c>
       <c r="D1307" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E1307" t="str">
         <v>INTEREXT OFFICE</v>
       </c>
       <c r="F1307" t="str">
-        <v>08:53 AM</v>
+        <v>07:40 PM</v>
       </c>
       <c r="G1307" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H1307">
-        <v>0</v>
+        <v>2.83</v>
       </c>
       <c r="I1307">
         <v>0</v>
@@ -65781,10 +65781,10 @@
         <v>0</v>
       </c>
       <c r="N1307">
-        <v>0</v>
+        <v>389.13</v>
       </c>
       <c r="O1307" t="str">
-        <v xml:space="preserve">Aneesh, Company quarters, </v>
+        <v>7:40PM | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P1307" t="str">
         <v/>
@@ -65801,7 +65801,7 @@
         <v>Anil Rana</v>
       </c>
       <c r="D1308" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E1308" t="str">
         <v>INTEREXT OFFICE</v>
@@ -65810,13 +65810,13 @@
         <v>08:53 AM</v>
       </c>
       <c r="G1308" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H1308">
-        <v>0</v>
+        <v>13.6</v>
       </c>
       <c r="I1308">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J1308">
         <v>0</v>
@@ -65825,16 +65825,16 @@
         <v>0</v>
       </c>
       <c r="L1308">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="M1308">
         <v>0</v>
       </c>
       <c r="N1308">
-        <v>0</v>
+        <v>1575</v>
       </c>
       <c r="O1308" t="str">
-        <v xml:space="preserve">Anil rana, Company quarters, </v>
+        <v>Anil rana, Company quarters,  | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P1308" t="str">
         <v/>
@@ -66001,22 +66001,22 @@
         <v>Arun George</v>
       </c>
       <c r="D1312" t="str">
-        <v>ABSENT</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E1312" t="str">
-        <v>—</v>
+        <v>INTEREXT OFFICE</v>
       </c>
       <c r="F1312" t="str">
-        <v>—</v>
+        <v>09:00 AM</v>
       </c>
       <c r="G1312" t="str">
-        <v>—</v>
+        <v>06:00 PM</v>
       </c>
       <c r="H1312">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I1312">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J1312">
         <v>0</v>
@@ -66025,19 +66025,19 @@
         <v>0</v>
       </c>
       <c r="L1312">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M1312">
         <v>0</v>
       </c>
       <c r="N1312">
-        <v>0</v>
+        <v>1320</v>
       </c>
       <c r="O1312" t="str">
-        <v>—</v>
+        <v>Sreeraj, Aneesh Anilrana Subodsha Anadhu Arun George Aamil Sanjaya behara Remanan (Chamakkala market. Quotes Office), (9-6 pm Chamakkala market)</v>
       </c>
       <c r="P1312" t="str">
-        <v>Auto-Marked Absent (Missing text)</v>
+        <v/>
       </c>
     </row>
     <row r="1313">
@@ -66251,7 +66251,7 @@
         <v>Devadas E K</v>
       </c>
       <c r="D1317" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E1317" t="str">
         <v>Webcam Scan</v>
@@ -66260,13 +66260,13 @@
         <v>11:04 AM</v>
       </c>
       <c r="G1317" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H1317">
-        <v>0</v>
+        <v>11.42</v>
       </c>
       <c r="I1317">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J1317">
         <v>0</v>
@@ -66275,16 +66275,16 @@
         <v>0</v>
       </c>
       <c r="L1317">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M1317">
         <v>0</v>
       </c>
       <c r="N1317">
-        <v>0</v>
+        <v>1650</v>
       </c>
       <c r="O1317" t="str">
-        <v>Face recognized - auto entry</v>
+        <v>Face recognized - auto entry | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P1317" t="str">
         <v/>
@@ -66401,7 +66401,7 @@
         <v>Gokul K</v>
       </c>
       <c r="D1320" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E1320" t="str">
         <v>Webcam Scan</v>
@@ -66410,13 +66410,13 @@
         <v>11:05 AM</v>
       </c>
       <c r="G1320" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H1320">
-        <v>0</v>
+        <v>11.4</v>
       </c>
       <c r="I1320">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J1320">
         <v>0</v>
@@ -66431,10 +66431,10 @@
         <v>0</v>
       </c>
       <c r="N1320">
-        <v>0</v>
+        <v>900</v>
       </c>
       <c r="O1320" t="str">
-        <v>Face recognized - auto entry</v>
+        <v>Face recognized - auto entry | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P1320" t="str">
         <v/>
@@ -66501,22 +66501,22 @@
         <v>Gopal (Soma)</v>
       </c>
       <c r="D1322" t="str">
-        <v>ABSENT</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E1322" t="str">
-        <v>—</v>
+        <v>INTEREXT OFFICE</v>
       </c>
       <c r="F1322" t="str">
-        <v>—</v>
+        <v>09:00 AM</v>
       </c>
       <c r="G1322" t="str">
-        <v>—</v>
+        <v>06:00 PM</v>
       </c>
       <c r="H1322">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I1322">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J1322">
         <v>0</v>
@@ -66525,19 +66525,19 @@
         <v>0</v>
       </c>
       <c r="L1322">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M1322">
         <v>0</v>
       </c>
       <c r="N1322">
-        <v>0</v>
+        <v>1155</v>
       </c>
       <c r="O1322" t="str">
-        <v>—</v>
+        <v>Gopal, —, 9am to 6pm Gokulam coorg</v>
       </c>
       <c r="P1322" t="str">
-        <v>Auto-Marked Absent (Missing text)</v>
+        <v/>
       </c>
     </row>
     <row r="1323">
@@ -66751,19 +66751,19 @@
         <v>Mahin Kj</v>
       </c>
       <c r="D1327" t="str">
-        <v>EARLY CHECK-OUT</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E1327" t="str">
-        <v>Webcam Scan</v>
+        <v>INTEREXT OFFICE</v>
       </c>
       <c r="F1327" t="str">
-        <v>08:31 AM</v>
+        <v>07:00 PM</v>
       </c>
       <c r="G1327" t="str">
-        <v>11:06 AM</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H1327">
-        <v>2.58</v>
+        <v>3.5</v>
       </c>
       <c r="I1327">
         <v>0</v>
@@ -66781,10 +66781,10 @@
         <v>0</v>
       </c>
       <c r="N1327">
-        <v>334.91</v>
+        <v>454.34</v>
       </c>
       <c r="O1327" t="str">
-        <v>Face recognized - auto exit</v>
+        <v>7.00pm | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P1327" t="str">
         <v/>
@@ -67101,22 +67101,22 @@
         <v>Prasanth E.M</v>
       </c>
       <c r="D1334" t="str">
-        <v>LATE CHECK-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E1334" t="str">
-        <v>Webcam Scan</v>
+        <v>INTEREXT OFFICE</v>
       </c>
       <c r="F1334" t="str">
-        <v>11:59 AM</v>
+        <v>09:00 AM</v>
       </c>
       <c r="G1334" t="str">
-        <v>—</v>
+        <v>06:00 PM</v>
       </c>
       <c r="H1334">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I1334">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J1334">
         <v>0</v>
@@ -67131,10 +67131,10 @@
         <v>0</v>
       </c>
       <c r="N1334">
-        <v>0</v>
+        <v>1192.31</v>
       </c>
       <c r="O1334" t="str">
-        <v>Face recognized - auto entry</v>
+        <v>9am to 6pm cavli wireless</v>
       </c>
       <c r="P1334" t="str">
         <v>Face recognized</v>
@@ -67201,19 +67201,19 @@
         <v>Rahul Das</v>
       </c>
       <c r="D1336" t="str">
-        <v>ABSENT</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E1336" t="str">
-        <v>—</v>
+        <v>INTEREXT OFFICE</v>
       </c>
       <c r="F1336" t="str">
-        <v>—</v>
+        <v>07:00 PM</v>
       </c>
       <c r="G1336" t="str">
-        <v>—</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H1336">
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="I1336">
         <v>0</v>
@@ -67231,13 +67231,13 @@
         <v>0</v>
       </c>
       <c r="N1336">
-        <v>0</v>
+        <v>370.19</v>
       </c>
       <c r="O1336" t="str">
-        <v>—</v>
+        <v>7:00 pm | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P1336" t="str">
-        <v>Auto-Marked Absent (Missing text)</v>
+        <v/>
       </c>
     </row>
     <row r="1337">
@@ -67401,7 +67401,7 @@
         <v>Raji Kannan</v>
       </c>
       <c r="D1340" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E1340" t="str">
         <v>Webcam Scan</v>
@@ -67410,13 +67410,13 @@
         <v>11:29 AM</v>
       </c>
       <c r="G1340" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H1340">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="I1340">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J1340">
         <v>0</v>
@@ -67425,16 +67425,16 @@
         <v>0</v>
       </c>
       <c r="L1340">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M1340">
         <v>0</v>
       </c>
       <c r="N1340">
-        <v>0</v>
+        <v>750</v>
       </c>
       <c r="O1340" t="str">
-        <v>Face recognized - auto entry</v>
+        <v>Face recognized - auto entry | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P1340" t="str">
         <v/>
@@ -67851,22 +67851,22 @@
         <v>Sabu (Joseph Antony)</v>
       </c>
       <c r="D1349" t="str">
-        <v>ABSENT</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E1349" t="str">
-        <v>—</v>
+        <v>INTEREXT OFFICE</v>
       </c>
       <c r="F1349" t="str">
-        <v>—</v>
+        <v>09:00 AM</v>
       </c>
       <c r="G1349" t="str">
-        <v>—</v>
+        <v>06:00 PM</v>
       </c>
       <c r="H1349">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I1349">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J1349">
         <v>0</v>
@@ -67875,19 +67875,19 @@
         <v>0</v>
       </c>
       <c r="L1349">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M1349">
         <v>0</v>
       </c>
       <c r="N1349">
-        <v>0</v>
+        <v>1430</v>
       </c>
       <c r="O1349" t="str">
-        <v>—</v>
+        <v>Joseph Antony, —, 9am to 6pm Gokulam coorg</v>
       </c>
       <c r="P1349" t="str">
-        <v>Auto-Marked Absent (Missing text)</v>
+        <v/>
       </c>
     </row>
     <row r="1350">
@@ -67951,22 +67951,22 @@
         <v>Sandeep C</v>
       </c>
       <c r="D1351" t="str">
-        <v>ABSENT</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E1351" t="str">
-        <v>—</v>
+        <v>INTEREXT OFFICE</v>
       </c>
       <c r="F1351" t="str">
-        <v>—</v>
+        <v>09:00 AM</v>
       </c>
       <c r="G1351" t="str">
-        <v>—</v>
+        <v>06:00 PM</v>
       </c>
       <c r="H1351">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I1351">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J1351">
         <v>0</v>
@@ -67975,19 +67975,19 @@
         <v>0</v>
       </c>
       <c r="L1351">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M1351">
         <v>0</v>
       </c>
       <c r="N1351">
-        <v>0</v>
+        <v>1320</v>
       </c>
       <c r="O1351" t="str">
-        <v>—</v>
+        <v>Sandeep c, —, 9am to 6pm Gokulam coorg</v>
       </c>
       <c r="P1351" t="str">
-        <v>Auto-Marked Absent (Missing text)</v>
+        <v/>
       </c>
     </row>
     <row r="1352">
@@ -68251,7 +68251,7 @@
         <v>Sona Francis</v>
       </c>
       <c r="D1357" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E1357" t="str">
         <v>Webcam Scan</v>
@@ -68260,13 +68260,13 @@
         <v>11:38 AM</v>
       </c>
       <c r="G1357" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H1357">
-        <v>0</v>
+        <v>10.85</v>
       </c>
       <c r="I1357">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J1357">
         <v>0</v>
@@ -68281,10 +68281,10 @@
         <v>0</v>
       </c>
       <c r="N1357">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="O1357" t="str">
-        <v>Face recognized - auto entry</v>
+        <v>Face recognized - auto entry | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P1357" t="str">
         <v/>
@@ -68451,7 +68451,7 @@
         <v>Stephin Pious</v>
       </c>
       <c r="D1361" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E1361" t="str">
         <v>Webcam Scan</v>
@@ -68460,13 +68460,13 @@
         <v>11:38 AM</v>
       </c>
       <c r="G1361" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H1361">
-        <v>0</v>
+        <v>10.85</v>
       </c>
       <c r="I1361">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J1361">
         <v>0</v>
@@ -68481,10 +68481,10 @@
         <v>0</v>
       </c>
       <c r="N1361">
-        <v>0</v>
+        <v>961.54</v>
       </c>
       <c r="O1361" t="str">
-        <v>Face recognized - auto entry</v>
+        <v>Face recognized - auto entry | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P1361" t="str">
         <v/>
@@ -68501,7 +68501,7 @@
         <v>Subodh Sha</v>
       </c>
       <c r="D1362" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E1362" t="str">
         <v>INTEREXT OFFICE</v>
@@ -68510,13 +68510,13 @@
         <v>08:53 AM</v>
       </c>
       <c r="G1362" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H1362">
-        <v>0</v>
+        <v>13.6</v>
       </c>
       <c r="I1362">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J1362">
         <v>0</v>
@@ -68525,16 +68525,16 @@
         <v>0</v>
       </c>
       <c r="L1362">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="M1362">
         <v>0</v>
       </c>
       <c r="N1362">
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c r="O1362" t="str">
-        <v xml:space="preserve">Subodsha, Company quarters, </v>
+        <v>Subodsha, Company quarters,  | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P1362" t="str">
         <v/>
@@ -68651,7 +68651,7 @@
         <v>Sunil Aliyar</v>
       </c>
       <c r="D1365" t="str">
-        <v>CHECKED-IN</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E1365" t="str">
         <v>INTEREXT OFFICE</v>
@@ -68660,13 +68660,13 @@
         <v>08:53 AM</v>
       </c>
       <c r="G1365" t="str">
-        <v>Currently Checked-In</v>
+        <v>10:30 PM</v>
       </c>
       <c r="H1365">
-        <v>0</v>
+        <v>13.6</v>
       </c>
       <c r="I1365">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J1365">
         <v>0</v>
@@ -68675,16 +68675,16 @@
         <v>0</v>
       </c>
       <c r="L1365">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="M1365">
         <v>0</v>
       </c>
       <c r="N1365">
-        <v>0</v>
+        <v>2025</v>
       </c>
       <c r="O1365" t="str">
-        <v xml:space="preserve">Sunil aliyar, Company quarters, </v>
+        <v>Sunil aliyar, Company quarters,  | [System Auto-Checkout: Missed check-out]</v>
       </c>
       <c r="P1365" t="str">
         <v/>
@@ -68890,9 +68890,3810 @@
         <v>Face recognized</v>
       </c>
     </row>
+    <row r="1370">
+      <c r="A1370" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1370" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1370" t="str">
+        <v>Aamil</v>
+      </c>
+      <c r="D1370" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1370" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1370" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1370" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1370">
+        <v>0</v>
+      </c>
+      <c r="I1370">
+        <v>0</v>
+      </c>
+      <c r="J1370">
+        <v>0</v>
+      </c>
+      <c r="K1370">
+        <v>0</v>
+      </c>
+      <c r="L1370">
+        <v>0</v>
+      </c>
+      <c r="M1370">
+        <v>0</v>
+      </c>
+      <c r="N1370">
+        <v>0</v>
+      </c>
+      <c r="O1370" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1370" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1371">
+      <c r="A1371" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1371" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1371" t="str">
+        <v>Abhishek Shaji</v>
+      </c>
+      <c r="D1371" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1371" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1371" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1371" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1371">
+        <v>0</v>
+      </c>
+      <c r="I1371">
+        <v>0</v>
+      </c>
+      <c r="J1371">
+        <v>0</v>
+      </c>
+      <c r="K1371">
+        <v>0</v>
+      </c>
+      <c r="L1371">
+        <v>0</v>
+      </c>
+      <c r="M1371">
+        <v>0</v>
+      </c>
+      <c r="N1371">
+        <v>0</v>
+      </c>
+      <c r="O1371" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1371" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1372">
+      <c r="A1372" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1372" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1372" t="str">
+        <v>Abin Mathew</v>
+      </c>
+      <c r="D1372" t="str">
+        <v>LEAVE</v>
+      </c>
+      <c r="E1372" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F1372" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1372" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1372">
+        <v>0</v>
+      </c>
+      <c r="I1372">
+        <v>0</v>
+      </c>
+      <c r="J1372">
+        <v>0</v>
+      </c>
+      <c r="K1372">
+        <v>0</v>
+      </c>
+      <c r="L1372">
+        <v>0</v>
+      </c>
+      <c r="M1372">
+        <v>0</v>
+      </c>
+      <c r="N1372">
+        <v>0</v>
+      </c>
+      <c r="O1372" t="str">
+        <v>I am on leave today</v>
+      </c>
+      <c r="P1372" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="1373">
+      <c r="A1373" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1373" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1373" t="str">
+        <v>Ajeesh Vijayan</v>
+      </c>
+      <c r="D1373" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1373" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1373" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1373" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1373">
+        <v>0</v>
+      </c>
+      <c r="I1373">
+        <v>0</v>
+      </c>
+      <c r="J1373">
+        <v>0</v>
+      </c>
+      <c r="K1373">
+        <v>0</v>
+      </c>
+      <c r="L1373">
+        <v>0</v>
+      </c>
+      <c r="M1373">
+        <v>0</v>
+      </c>
+      <c r="N1373">
+        <v>0</v>
+      </c>
+      <c r="O1373" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1373" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1374">
+      <c r="A1374" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1374" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1374" t="str">
+        <v>Ajith Reghunath</v>
+      </c>
+      <c r="D1374" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1374" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1374" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1374" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1374">
+        <v>0</v>
+      </c>
+      <c r="I1374">
+        <v>0</v>
+      </c>
+      <c r="J1374">
+        <v>0</v>
+      </c>
+      <c r="K1374">
+        <v>0</v>
+      </c>
+      <c r="L1374">
+        <v>0</v>
+      </c>
+      <c r="M1374">
+        <v>0</v>
+      </c>
+      <c r="N1374">
+        <v>0</v>
+      </c>
+      <c r="O1374" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1374" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1375">
+      <c r="A1375" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1375" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1375" t="str">
+        <v>Ajmal K H</v>
+      </c>
+      <c r="D1375" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1375" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1375" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1375" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1375">
+        <v>0</v>
+      </c>
+      <c r="I1375">
+        <v>0</v>
+      </c>
+      <c r="J1375">
+        <v>0</v>
+      </c>
+      <c r="K1375">
+        <v>0</v>
+      </c>
+      <c r="L1375">
+        <v>0</v>
+      </c>
+      <c r="M1375">
+        <v>0</v>
+      </c>
+      <c r="N1375">
+        <v>0</v>
+      </c>
+      <c r="O1375" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1375" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1376">
+      <c r="A1376" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1376" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1376" t="str">
+        <v>Akash Rana</v>
+      </c>
+      <c r="D1376" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1376" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1376" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1376" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1376">
+        <v>0</v>
+      </c>
+      <c r="I1376">
+        <v>0</v>
+      </c>
+      <c r="J1376">
+        <v>0</v>
+      </c>
+      <c r="K1376">
+        <v>0</v>
+      </c>
+      <c r="L1376">
+        <v>0</v>
+      </c>
+      <c r="M1376">
+        <v>0</v>
+      </c>
+      <c r="N1376">
+        <v>0</v>
+      </c>
+      <c r="O1376" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1376" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1377">
+      <c r="A1377" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1377" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1377" t="str">
+        <v>Akhil Ak</v>
+      </c>
+      <c r="D1377" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1377" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1377" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1377" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1377">
+        <v>0</v>
+      </c>
+      <c r="I1377">
+        <v>0</v>
+      </c>
+      <c r="J1377">
+        <v>0</v>
+      </c>
+      <c r="K1377">
+        <v>0</v>
+      </c>
+      <c r="L1377">
+        <v>0</v>
+      </c>
+      <c r="M1377">
+        <v>0</v>
+      </c>
+      <c r="N1377">
+        <v>0</v>
+      </c>
+      <c r="O1377" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1377" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1378">
+      <c r="A1378" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1378" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1378" t="str">
+        <v>Akhil P Kumar</v>
+      </c>
+      <c r="D1378" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1378" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1378" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1378" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1378">
+        <v>0</v>
+      </c>
+      <c r="I1378">
+        <v>0</v>
+      </c>
+      <c r="J1378">
+        <v>0</v>
+      </c>
+      <c r="K1378">
+        <v>0</v>
+      </c>
+      <c r="L1378">
+        <v>0</v>
+      </c>
+      <c r="M1378">
+        <v>0</v>
+      </c>
+      <c r="N1378">
+        <v>0</v>
+      </c>
+      <c r="O1378" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1378" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1379">
+      <c r="A1379" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1379" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1379" t="str">
+        <v>Alex Gigi</v>
+      </c>
+      <c r="D1379" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1379" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1379" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1379" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1379">
+        <v>0</v>
+      </c>
+      <c r="I1379">
+        <v>0</v>
+      </c>
+      <c r="J1379">
+        <v>0</v>
+      </c>
+      <c r="K1379">
+        <v>0</v>
+      </c>
+      <c r="L1379">
+        <v>0</v>
+      </c>
+      <c r="M1379">
+        <v>0</v>
+      </c>
+      <c r="N1379">
+        <v>0</v>
+      </c>
+      <c r="O1379" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1379" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1380">
+      <c r="A1380" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1380" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1380" t="str">
+        <v>Alex Rajan</v>
+      </c>
+      <c r="D1380" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1380" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1380" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1380" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1380">
+        <v>0</v>
+      </c>
+      <c r="I1380">
+        <v>0</v>
+      </c>
+      <c r="J1380">
+        <v>0</v>
+      </c>
+      <c r="K1380">
+        <v>0</v>
+      </c>
+      <c r="L1380">
+        <v>0</v>
+      </c>
+      <c r="M1380">
+        <v>0</v>
+      </c>
+      <c r="N1380">
+        <v>0</v>
+      </c>
+      <c r="O1380" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1380" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1381">
+      <c r="A1381" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1381" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1381" t="str">
+        <v>Anandhu Raj</v>
+      </c>
+      <c r="D1381" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1381" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1381" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1381" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1381">
+        <v>0</v>
+      </c>
+      <c r="I1381">
+        <v>0</v>
+      </c>
+      <c r="J1381">
+        <v>0</v>
+      </c>
+      <c r="K1381">
+        <v>0</v>
+      </c>
+      <c r="L1381">
+        <v>0</v>
+      </c>
+      <c r="M1381">
+        <v>0</v>
+      </c>
+      <c r="N1381">
+        <v>0</v>
+      </c>
+      <c r="O1381" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1381" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1382">
+      <c r="A1382" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1382" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1382" t="str">
+        <v>Anandhu Sunil</v>
+      </c>
+      <c r="D1382" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1382" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1382" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1382" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1382">
+        <v>0</v>
+      </c>
+      <c r="I1382">
+        <v>0</v>
+      </c>
+      <c r="J1382">
+        <v>0</v>
+      </c>
+      <c r="K1382">
+        <v>0</v>
+      </c>
+      <c r="L1382">
+        <v>0</v>
+      </c>
+      <c r="M1382">
+        <v>0</v>
+      </c>
+      <c r="N1382">
+        <v>0</v>
+      </c>
+      <c r="O1382" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1382" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1383">
+      <c r="A1383" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1383" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1383" t="str">
+        <v>Aneesh Ahammed</v>
+      </c>
+      <c r="D1383" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E1383" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F1383" t="str">
+        <v>08:54 AM</v>
+      </c>
+      <c r="G1383" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H1383">
+        <v>0</v>
+      </c>
+      <c r="I1383">
+        <v>0</v>
+      </c>
+      <c r="J1383">
+        <v>0</v>
+      </c>
+      <c r="K1383">
+        <v>0</v>
+      </c>
+      <c r="L1383">
+        <v>0</v>
+      </c>
+      <c r="M1383">
+        <v>0</v>
+      </c>
+      <c r="N1383">
+        <v>0</v>
+      </c>
+      <c r="O1383" t="str">
+        <v>8:54am</v>
+      </c>
+      <c r="P1383" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="1384">
+      <c r="A1384" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1384" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1384" t="str">
+        <v>Anil Rana</v>
+      </c>
+      <c r="D1384" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1384" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1384" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1384" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1384">
+        <v>0</v>
+      </c>
+      <c r="I1384">
+        <v>0</v>
+      </c>
+      <c r="J1384">
+        <v>0</v>
+      </c>
+      <c r="K1384">
+        <v>0</v>
+      </c>
+      <c r="L1384">
+        <v>0</v>
+      </c>
+      <c r="M1384">
+        <v>0</v>
+      </c>
+      <c r="N1384">
+        <v>0</v>
+      </c>
+      <c r="O1384" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1384" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1385">
+      <c r="A1385" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1385" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1385" t="str">
+        <v>Anish Viswanathan</v>
+      </c>
+      <c r="D1385" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1385" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1385" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1385" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1385">
+        <v>0</v>
+      </c>
+      <c r="I1385">
+        <v>0</v>
+      </c>
+      <c r="J1385">
+        <v>0</v>
+      </c>
+      <c r="K1385">
+        <v>0</v>
+      </c>
+      <c r="L1385">
+        <v>0</v>
+      </c>
+      <c r="M1385">
+        <v>0</v>
+      </c>
+      <c r="N1385">
+        <v>0</v>
+      </c>
+      <c r="O1385" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1385" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1386">
+      <c r="A1386" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1386" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1386" t="str">
+        <v>Anoop (Ancil K Grace)</v>
+      </c>
+      <c r="D1386" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1386" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1386" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1386" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1386">
+        <v>0</v>
+      </c>
+      <c r="I1386">
+        <v>0</v>
+      </c>
+      <c r="J1386">
+        <v>0</v>
+      </c>
+      <c r="K1386">
+        <v>0</v>
+      </c>
+      <c r="L1386">
+        <v>0</v>
+      </c>
+      <c r="M1386">
+        <v>0</v>
+      </c>
+      <c r="N1386">
+        <v>0</v>
+      </c>
+      <c r="O1386" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1386" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1387">
+      <c r="A1387" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1387" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1387" t="str">
+        <v>Anusree Subramanian</v>
+      </c>
+      <c r="D1387" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1387" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1387" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1387" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1387">
+        <v>0</v>
+      </c>
+      <c r="I1387">
+        <v>0</v>
+      </c>
+      <c r="J1387">
+        <v>0</v>
+      </c>
+      <c r="K1387">
+        <v>0</v>
+      </c>
+      <c r="L1387">
+        <v>0</v>
+      </c>
+      <c r="M1387">
+        <v>0</v>
+      </c>
+      <c r="N1387">
+        <v>0</v>
+      </c>
+      <c r="O1387" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1387" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1388">
+      <c r="A1388" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1388" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1388" t="str">
+        <v>Arun George</v>
+      </c>
+      <c r="D1388" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1388" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1388" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1388" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1388">
+        <v>0</v>
+      </c>
+      <c r="I1388">
+        <v>0</v>
+      </c>
+      <c r="J1388">
+        <v>0</v>
+      </c>
+      <c r="K1388">
+        <v>0</v>
+      </c>
+      <c r="L1388">
+        <v>0</v>
+      </c>
+      <c r="M1388">
+        <v>0</v>
+      </c>
+      <c r="N1388">
+        <v>0</v>
+      </c>
+      <c r="O1388" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1388" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1389">
+      <c r="A1389" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1389" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1389" t="str">
+        <v>Arun P Madhu</v>
+      </c>
+      <c r="D1389" t="str">
+        <v>LEAVE</v>
+      </c>
+      <c r="E1389" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F1389" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1389" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1389">
+        <v>0</v>
+      </c>
+      <c r="I1389">
+        <v>0</v>
+      </c>
+      <c r="J1389">
+        <v>0</v>
+      </c>
+      <c r="K1389">
+        <v>0</v>
+      </c>
+      <c r="L1389">
+        <v>0</v>
+      </c>
+      <c r="M1389">
+        <v>0</v>
+      </c>
+      <c r="N1389">
+        <v>0</v>
+      </c>
+      <c r="O1389" t="str">
+        <v>I am leave today</v>
+      </c>
+      <c r="P1389" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="1390">
+      <c r="A1390" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1390" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1390" t="str">
+        <v>Bimal Rana</v>
+      </c>
+      <c r="D1390" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1390" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1390" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1390" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1390">
+        <v>0</v>
+      </c>
+      <c r="I1390">
+        <v>0</v>
+      </c>
+      <c r="J1390">
+        <v>0</v>
+      </c>
+      <c r="K1390">
+        <v>0</v>
+      </c>
+      <c r="L1390">
+        <v>0</v>
+      </c>
+      <c r="M1390">
+        <v>0</v>
+      </c>
+      <c r="N1390">
+        <v>0</v>
+      </c>
+      <c r="O1390" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1390" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1391">
+      <c r="A1391" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1391" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1391" t="str">
+        <v>Bindhu Jose</v>
+      </c>
+      <c r="D1391" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1391" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1391" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1391" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1391">
+        <v>0</v>
+      </c>
+      <c r="I1391">
+        <v>0</v>
+      </c>
+      <c r="J1391">
+        <v>0</v>
+      </c>
+      <c r="K1391">
+        <v>0</v>
+      </c>
+      <c r="L1391">
+        <v>0</v>
+      </c>
+      <c r="M1391">
+        <v>0</v>
+      </c>
+      <c r="N1391">
+        <v>0</v>
+      </c>
+      <c r="O1391" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1391" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1392">
+      <c r="A1392" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1392" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1392" t="str">
+        <v>Binu</v>
+      </c>
+      <c r="D1392" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1392" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1392" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1392" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1392">
+        <v>0</v>
+      </c>
+      <c r="I1392">
+        <v>0</v>
+      </c>
+      <c r="J1392">
+        <v>0</v>
+      </c>
+      <c r="K1392">
+        <v>0</v>
+      </c>
+      <c r="L1392">
+        <v>0</v>
+      </c>
+      <c r="M1392">
+        <v>0</v>
+      </c>
+      <c r="N1392">
+        <v>0</v>
+      </c>
+      <c r="O1392" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1392" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1393">
+      <c r="A1393" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1393" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1393" t="str">
+        <v>Devadas E K</v>
+      </c>
+      <c r="D1393" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1393" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1393" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1393" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1393">
+        <v>0</v>
+      </c>
+      <c r="I1393">
+        <v>0</v>
+      </c>
+      <c r="J1393">
+        <v>0</v>
+      </c>
+      <c r="K1393">
+        <v>0</v>
+      </c>
+      <c r="L1393">
+        <v>0</v>
+      </c>
+      <c r="M1393">
+        <v>0</v>
+      </c>
+      <c r="N1393">
+        <v>0</v>
+      </c>
+      <c r="O1393" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1393" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1394">
+      <c r="A1394" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1394" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1394" t="str">
+        <v>Faiyaj Ansari</v>
+      </c>
+      <c r="D1394" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1394" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1394" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1394" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1394">
+        <v>0</v>
+      </c>
+      <c r="I1394">
+        <v>0</v>
+      </c>
+      <c r="J1394">
+        <v>0</v>
+      </c>
+      <c r="K1394">
+        <v>0</v>
+      </c>
+      <c r="L1394">
+        <v>0</v>
+      </c>
+      <c r="M1394">
+        <v>0</v>
+      </c>
+      <c r="N1394">
+        <v>0</v>
+      </c>
+      <c r="O1394" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1394" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1395">
+      <c r="A1395" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1395" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1395" t="str">
+        <v>George Thomas</v>
+      </c>
+      <c r="D1395" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1395" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1395" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1395" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1395">
+        <v>0</v>
+      </c>
+      <c r="I1395">
+        <v>0</v>
+      </c>
+      <c r="J1395">
+        <v>0</v>
+      </c>
+      <c r="K1395">
+        <v>0</v>
+      </c>
+      <c r="L1395">
+        <v>0</v>
+      </c>
+      <c r="M1395">
+        <v>0</v>
+      </c>
+      <c r="N1395">
+        <v>0</v>
+      </c>
+      <c r="O1395" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1395" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1396">
+      <c r="A1396" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1396" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1396" t="str">
+        <v>Gokul K</v>
+      </c>
+      <c r="D1396" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1396" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1396" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1396" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1396">
+        <v>0</v>
+      </c>
+      <c r="I1396">
+        <v>0</v>
+      </c>
+      <c r="J1396">
+        <v>0</v>
+      </c>
+      <c r="K1396">
+        <v>0</v>
+      </c>
+      <c r="L1396">
+        <v>0</v>
+      </c>
+      <c r="M1396">
+        <v>0</v>
+      </c>
+      <c r="N1396">
+        <v>0</v>
+      </c>
+      <c r="O1396" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1396" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1397">
+      <c r="A1397" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1397" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1397" t="str">
+        <v>Gokul Krishnan E V</v>
+      </c>
+      <c r="D1397" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1397" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1397" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1397" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1397">
+        <v>0</v>
+      </c>
+      <c r="I1397">
+        <v>0</v>
+      </c>
+      <c r="J1397">
+        <v>0</v>
+      </c>
+      <c r="K1397">
+        <v>0</v>
+      </c>
+      <c r="L1397">
+        <v>0</v>
+      </c>
+      <c r="M1397">
+        <v>0</v>
+      </c>
+      <c r="N1397">
+        <v>0</v>
+      </c>
+      <c r="O1397" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1397" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1398">
+      <c r="A1398" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1398" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1398" t="str">
+        <v>Gopal (Soma)</v>
+      </c>
+      <c r="D1398" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1398" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1398" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1398" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1398">
+        <v>0</v>
+      </c>
+      <c r="I1398">
+        <v>0</v>
+      </c>
+      <c r="J1398">
+        <v>0</v>
+      </c>
+      <c r="K1398">
+        <v>0</v>
+      </c>
+      <c r="L1398">
+        <v>0</v>
+      </c>
+      <c r="M1398">
+        <v>0</v>
+      </c>
+      <c r="N1398">
+        <v>0</v>
+      </c>
+      <c r="O1398" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1398" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1399">
+      <c r="A1399" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1399" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1399" t="str">
+        <v>James Tm</v>
+      </c>
+      <c r="D1399" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1399" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1399" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1399" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1399">
+        <v>0</v>
+      </c>
+      <c r="I1399">
+        <v>0</v>
+      </c>
+      <c r="J1399">
+        <v>0</v>
+      </c>
+      <c r="K1399">
+        <v>0</v>
+      </c>
+      <c r="L1399">
+        <v>0</v>
+      </c>
+      <c r="M1399">
+        <v>0</v>
+      </c>
+      <c r="N1399">
+        <v>0</v>
+      </c>
+      <c r="O1399" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1399" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1400">
+      <c r="A1400" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1400" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1400" t="str">
+        <v>Jitendra Rana</v>
+      </c>
+      <c r="D1400" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1400" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1400" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1400" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1400">
+        <v>0</v>
+      </c>
+      <c r="I1400">
+        <v>0</v>
+      </c>
+      <c r="J1400">
+        <v>0</v>
+      </c>
+      <c r="K1400">
+        <v>0</v>
+      </c>
+      <c r="L1400">
+        <v>0</v>
+      </c>
+      <c r="M1400">
+        <v>0</v>
+      </c>
+      <c r="N1400">
+        <v>0</v>
+      </c>
+      <c r="O1400" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1400" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1401">
+      <c r="A1401" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1401" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1401" t="str">
+        <v>Joshy</v>
+      </c>
+      <c r="D1401" t="str">
+        <v>LEAVE</v>
+      </c>
+      <c r="E1401" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F1401" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1401" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1401">
+        <v>0</v>
+      </c>
+      <c r="I1401">
+        <v>0</v>
+      </c>
+      <c r="J1401">
+        <v>0</v>
+      </c>
+      <c r="K1401">
+        <v>0</v>
+      </c>
+      <c r="L1401">
+        <v>0</v>
+      </c>
+      <c r="M1401">
+        <v>0</v>
+      </c>
+      <c r="N1401">
+        <v>0</v>
+      </c>
+      <c r="O1401" t="str">
+        <v>I am leave today</v>
+      </c>
+      <c r="P1401" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="1402">
+      <c r="A1402" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1402" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1402" t="str">
+        <v>M S Arjun</v>
+      </c>
+      <c r="D1402" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E1402" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F1402" t="str">
+        <v>09:00 AM</v>
+      </c>
+      <c r="G1402" t="str">
+        <v>06:00 PM</v>
+      </c>
+      <c r="H1402">
+        <v>0</v>
+      </c>
+      <c r="I1402">
+        <v>0</v>
+      </c>
+      <c r="J1402">
+        <v>0</v>
+      </c>
+      <c r="K1402">
+        <v>0</v>
+      </c>
+      <c r="L1402">
+        <v>0</v>
+      </c>
+      <c r="M1402">
+        <v>0</v>
+      </c>
+      <c r="N1402">
+        <v>0</v>
+      </c>
+      <c r="O1402" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1402" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="1403">
+      <c r="A1403" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1403" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1403" t="str">
+        <v>Mahin Kj</v>
+      </c>
+      <c r="D1403" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E1403" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F1403" t="str">
+        <v>07:28 AM</v>
+      </c>
+      <c r="G1403" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H1403">
+        <v>0</v>
+      </c>
+      <c r="I1403">
+        <v>0</v>
+      </c>
+      <c r="J1403">
+        <v>0</v>
+      </c>
+      <c r="K1403">
+        <v>0</v>
+      </c>
+      <c r="L1403">
+        <v>0</v>
+      </c>
+      <c r="M1403">
+        <v>0</v>
+      </c>
+      <c r="N1403">
+        <v>0</v>
+      </c>
+      <c r="O1403" t="str">
+        <v>7.28am</v>
+      </c>
+      <c r="P1403" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="1404">
+      <c r="A1404" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1404" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1404" t="str">
+        <v>Manu Mahesh</v>
+      </c>
+      <c r="D1404" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1404" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1404" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1404" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1404">
+        <v>0</v>
+      </c>
+      <c r="I1404">
+        <v>0</v>
+      </c>
+      <c r="J1404">
+        <v>0</v>
+      </c>
+      <c r="K1404">
+        <v>0</v>
+      </c>
+      <c r="L1404">
+        <v>0</v>
+      </c>
+      <c r="M1404">
+        <v>0</v>
+      </c>
+      <c r="N1404">
+        <v>0</v>
+      </c>
+      <c r="O1404" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1404" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1405">
+      <c r="A1405" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1405" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1405" t="str">
+        <v>Mohammed Gulfam</v>
+      </c>
+      <c r="D1405" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1405" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1405" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1405" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1405">
+        <v>0</v>
+      </c>
+      <c r="I1405">
+        <v>0</v>
+      </c>
+      <c r="J1405">
+        <v>0</v>
+      </c>
+      <c r="K1405">
+        <v>0</v>
+      </c>
+      <c r="L1405">
+        <v>0</v>
+      </c>
+      <c r="M1405">
+        <v>0</v>
+      </c>
+      <c r="N1405">
+        <v>0</v>
+      </c>
+      <c r="O1405" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1405" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1406">
+      <c r="A1406" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1406" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1406" t="str">
+        <v>Niji Manoj</v>
+      </c>
+      <c r="D1406" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1406" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1406" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1406" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1406">
+        <v>0</v>
+      </c>
+      <c r="I1406">
+        <v>0</v>
+      </c>
+      <c r="J1406">
+        <v>0</v>
+      </c>
+      <c r="K1406">
+        <v>0</v>
+      </c>
+      <c r="L1406">
+        <v>0</v>
+      </c>
+      <c r="M1406">
+        <v>0</v>
+      </c>
+      <c r="N1406">
+        <v>0</v>
+      </c>
+      <c r="O1406" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1406" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1407">
+      <c r="A1407" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1407" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1407" t="str">
+        <v>Niranjan Bose</v>
+      </c>
+      <c r="D1407" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1407" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1407" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1407" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1407">
+        <v>0</v>
+      </c>
+      <c r="I1407">
+        <v>0</v>
+      </c>
+      <c r="J1407">
+        <v>0</v>
+      </c>
+      <c r="K1407">
+        <v>0</v>
+      </c>
+      <c r="L1407">
+        <v>0</v>
+      </c>
+      <c r="M1407">
+        <v>0</v>
+      </c>
+      <c r="N1407">
+        <v>0</v>
+      </c>
+      <c r="O1407" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1407" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1408">
+      <c r="A1408" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1408" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1408" t="str">
+        <v>Nourin Shaji</v>
+      </c>
+      <c r="D1408" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1408" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1408" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1408" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1408">
+        <v>0</v>
+      </c>
+      <c r="I1408">
+        <v>0</v>
+      </c>
+      <c r="J1408">
+        <v>0</v>
+      </c>
+      <c r="K1408">
+        <v>0</v>
+      </c>
+      <c r="L1408">
+        <v>0</v>
+      </c>
+      <c r="M1408">
+        <v>0</v>
+      </c>
+      <c r="N1408">
+        <v>0</v>
+      </c>
+      <c r="O1408" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1408" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1409">
+      <c r="A1409" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1409" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1409" t="str">
+        <v>Pappu Kumar Rana</v>
+      </c>
+      <c r="D1409" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1409" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1409" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1409" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1409">
+        <v>0</v>
+      </c>
+      <c r="I1409">
+        <v>0</v>
+      </c>
+      <c r="J1409">
+        <v>0</v>
+      </c>
+      <c r="K1409">
+        <v>0</v>
+      </c>
+      <c r="L1409">
+        <v>0</v>
+      </c>
+      <c r="M1409">
+        <v>0</v>
+      </c>
+      <c r="N1409">
+        <v>0</v>
+      </c>
+      <c r="O1409" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1409" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1410">
+      <c r="A1410" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1410" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1410" t="str">
+        <v>Prasanth E.M</v>
+      </c>
+      <c r="D1410" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1410" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1410" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1410" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1410">
+        <v>0</v>
+      </c>
+      <c r="I1410">
+        <v>0</v>
+      </c>
+      <c r="J1410">
+        <v>0</v>
+      </c>
+      <c r="K1410">
+        <v>0</v>
+      </c>
+      <c r="L1410">
+        <v>0</v>
+      </c>
+      <c r="M1410">
+        <v>0</v>
+      </c>
+      <c r="N1410">
+        <v>0</v>
+      </c>
+      <c r="O1410" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1410" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1411">
+      <c r="A1411" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1411" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1411" t="str">
+        <v>Pratheesh K S</v>
+      </c>
+      <c r="D1411" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1411" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1411" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1411" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1411">
+        <v>0</v>
+      </c>
+      <c r="I1411">
+        <v>0</v>
+      </c>
+      <c r="J1411">
+        <v>0</v>
+      </c>
+      <c r="K1411">
+        <v>0</v>
+      </c>
+      <c r="L1411">
+        <v>0</v>
+      </c>
+      <c r="M1411">
+        <v>0</v>
+      </c>
+      <c r="N1411">
+        <v>0</v>
+      </c>
+      <c r="O1411" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1411" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1412">
+      <c r="A1412" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1412" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1412" t="str">
+        <v>Rahul Das</v>
+      </c>
+      <c r="D1412" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E1412" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F1412" t="str">
+        <v>08:40 AM</v>
+      </c>
+      <c r="G1412" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H1412">
+        <v>0</v>
+      </c>
+      <c r="I1412">
+        <v>0</v>
+      </c>
+      <c r="J1412">
+        <v>0</v>
+      </c>
+      <c r="K1412">
+        <v>0</v>
+      </c>
+      <c r="L1412">
+        <v>0</v>
+      </c>
+      <c r="M1412">
+        <v>0</v>
+      </c>
+      <c r="N1412">
+        <v>0</v>
+      </c>
+      <c r="O1412" t="str">
+        <v>8:40am</v>
+      </c>
+      <c r="P1412" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="1413">
+      <c r="A1413" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1413" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1413" t="str">
+        <v>Rahul R Nair</v>
+      </c>
+      <c r="D1413" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1413" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1413" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1413" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1413">
+        <v>0</v>
+      </c>
+      <c r="I1413">
+        <v>0</v>
+      </c>
+      <c r="J1413">
+        <v>0</v>
+      </c>
+      <c r="K1413">
+        <v>0</v>
+      </c>
+      <c r="L1413">
+        <v>0</v>
+      </c>
+      <c r="M1413">
+        <v>0</v>
+      </c>
+      <c r="N1413">
+        <v>0</v>
+      </c>
+      <c r="O1413" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1413" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1414">
+      <c r="A1414" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1414" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1414" t="str">
+        <v>Rahul Sundaran</v>
+      </c>
+      <c r="D1414" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1414" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1414" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1414" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1414">
+        <v>0</v>
+      </c>
+      <c r="I1414">
+        <v>0</v>
+      </c>
+      <c r="J1414">
+        <v>0</v>
+      </c>
+      <c r="K1414">
+        <v>0</v>
+      </c>
+      <c r="L1414">
+        <v>0</v>
+      </c>
+      <c r="M1414">
+        <v>0</v>
+      </c>
+      <c r="N1414">
+        <v>0</v>
+      </c>
+      <c r="O1414" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1414" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1415">
+      <c r="A1415" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1415" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1415" t="str">
+        <v>Raj Kumar Rana</v>
+      </c>
+      <c r="D1415" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1415" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1415" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1415" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1415">
+        <v>0</v>
+      </c>
+      <c r="I1415">
+        <v>0</v>
+      </c>
+      <c r="J1415">
+        <v>0</v>
+      </c>
+      <c r="K1415">
+        <v>0</v>
+      </c>
+      <c r="L1415">
+        <v>0</v>
+      </c>
+      <c r="M1415">
+        <v>0</v>
+      </c>
+      <c r="N1415">
+        <v>0</v>
+      </c>
+      <c r="O1415" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1415" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1416">
+      <c r="A1416" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1416" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1416" t="str">
+        <v>Raji Kannan</v>
+      </c>
+      <c r="D1416" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1416" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1416" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1416" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1416">
+        <v>0</v>
+      </c>
+      <c r="I1416">
+        <v>0</v>
+      </c>
+      <c r="J1416">
+        <v>0</v>
+      </c>
+      <c r="K1416">
+        <v>0</v>
+      </c>
+      <c r="L1416">
+        <v>0</v>
+      </c>
+      <c r="M1416">
+        <v>0</v>
+      </c>
+      <c r="N1416">
+        <v>0</v>
+      </c>
+      <c r="O1416" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1416" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1417">
+      <c r="A1417" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1417" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1417" t="str">
+        <v>Raju Rana</v>
+      </c>
+      <c r="D1417" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1417" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1417" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1417" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1417">
+        <v>0</v>
+      </c>
+      <c r="I1417">
+        <v>0</v>
+      </c>
+      <c r="J1417">
+        <v>0</v>
+      </c>
+      <c r="K1417">
+        <v>0</v>
+      </c>
+      <c r="L1417">
+        <v>0</v>
+      </c>
+      <c r="M1417">
+        <v>0</v>
+      </c>
+      <c r="N1417">
+        <v>0</v>
+      </c>
+      <c r="O1417" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1417" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1418">
+      <c r="A1418" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1418" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1418" t="str">
+        <v>Rakesh Sadhukha</v>
+      </c>
+      <c r="D1418" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1418" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1418" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1418" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1418">
+        <v>0</v>
+      </c>
+      <c r="I1418">
+        <v>0</v>
+      </c>
+      <c r="J1418">
+        <v>0</v>
+      </c>
+      <c r="K1418">
+        <v>0</v>
+      </c>
+      <c r="L1418">
+        <v>0</v>
+      </c>
+      <c r="M1418">
+        <v>0</v>
+      </c>
+      <c r="N1418">
+        <v>0</v>
+      </c>
+      <c r="O1418" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1418" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1419">
+      <c r="A1419" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1419" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1419" t="str">
+        <v>Ramsy Rasheed</v>
+      </c>
+      <c r="D1419" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1419" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1419" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1419" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1419">
+        <v>0</v>
+      </c>
+      <c r="I1419">
+        <v>0</v>
+      </c>
+      <c r="J1419">
+        <v>0</v>
+      </c>
+      <c r="K1419">
+        <v>0</v>
+      </c>
+      <c r="L1419">
+        <v>0</v>
+      </c>
+      <c r="M1419">
+        <v>0</v>
+      </c>
+      <c r="N1419">
+        <v>0</v>
+      </c>
+      <c r="O1419" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1419" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1420">
+      <c r="A1420" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1420" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1420" t="str">
+        <v>Ratheesh K S</v>
+      </c>
+      <c r="D1420" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1420" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1420" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1420" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1420">
+        <v>0</v>
+      </c>
+      <c r="I1420">
+        <v>0</v>
+      </c>
+      <c r="J1420">
+        <v>0</v>
+      </c>
+      <c r="K1420">
+        <v>0</v>
+      </c>
+      <c r="L1420">
+        <v>0</v>
+      </c>
+      <c r="M1420">
+        <v>0</v>
+      </c>
+      <c r="N1420">
+        <v>0</v>
+      </c>
+      <c r="O1420" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1420" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1421">
+      <c r="A1421" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1421" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1421" t="str">
+        <v>Ratheesh P R</v>
+      </c>
+      <c r="D1421" t="str">
+        <v>LATE</v>
+      </c>
+      <c r="E1421" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F1421" t="str">
+        <v>11:00 AM</v>
+      </c>
+      <c r="G1421" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1421">
+        <v>0</v>
+      </c>
+      <c r="I1421">
+        <v>0</v>
+      </c>
+      <c r="J1421">
+        <v>0</v>
+      </c>
+      <c r="K1421">
+        <v>0</v>
+      </c>
+      <c r="L1421">
+        <v>0</v>
+      </c>
+      <c r="M1421">
+        <v>0</v>
+      </c>
+      <c r="N1421">
+        <v>0</v>
+      </c>
+      <c r="O1421" t="str">
+        <v>Two hour late today morning session</v>
+      </c>
+      <c r="P1421" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="1422">
+      <c r="A1422" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1422" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1422" t="str">
+        <v>Rebeesh K S</v>
+      </c>
+      <c r="D1422" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1422" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1422" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1422" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1422">
+        <v>0</v>
+      </c>
+      <c r="I1422">
+        <v>0</v>
+      </c>
+      <c r="J1422">
+        <v>0</v>
+      </c>
+      <c r="K1422">
+        <v>0</v>
+      </c>
+      <c r="L1422">
+        <v>0</v>
+      </c>
+      <c r="M1422">
+        <v>0</v>
+      </c>
+      <c r="N1422">
+        <v>0</v>
+      </c>
+      <c r="O1422" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1422" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1423">
+      <c r="A1423" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1423" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1423" t="str">
+        <v>Rekha Madhu</v>
+      </c>
+      <c r="D1423" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1423" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1423" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1423" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1423">
+        <v>0</v>
+      </c>
+      <c r="I1423">
+        <v>0</v>
+      </c>
+      <c r="J1423">
+        <v>0</v>
+      </c>
+      <c r="K1423">
+        <v>0</v>
+      </c>
+      <c r="L1423">
+        <v>0</v>
+      </c>
+      <c r="M1423">
+        <v>0</v>
+      </c>
+      <c r="N1423">
+        <v>0</v>
+      </c>
+      <c r="O1423" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1423" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1424">
+      <c r="A1424" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1424" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1424" t="str">
+        <v>Remanan N N</v>
+      </c>
+      <c r="D1424" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1424" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1424" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1424" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1424">
+        <v>0</v>
+      </c>
+      <c r="I1424">
+        <v>0</v>
+      </c>
+      <c r="J1424">
+        <v>0</v>
+      </c>
+      <c r="K1424">
+        <v>0</v>
+      </c>
+      <c r="L1424">
+        <v>0</v>
+      </c>
+      <c r="M1424">
+        <v>0</v>
+      </c>
+      <c r="N1424">
+        <v>0</v>
+      </c>
+      <c r="O1424" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1424" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1425">
+      <c r="A1425" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1425" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1425" t="str">
+        <v>Sabu (Joseph Antony)</v>
+      </c>
+      <c r="D1425" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1425" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1425" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1425" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1425">
+        <v>0</v>
+      </c>
+      <c r="I1425">
+        <v>0</v>
+      </c>
+      <c r="J1425">
+        <v>0</v>
+      </c>
+      <c r="K1425">
+        <v>0</v>
+      </c>
+      <c r="L1425">
+        <v>0</v>
+      </c>
+      <c r="M1425">
+        <v>0</v>
+      </c>
+      <c r="N1425">
+        <v>0</v>
+      </c>
+      <c r="O1425" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1425" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1426">
+      <c r="A1426" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1426" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1426" t="str">
+        <v>Samshad Aalam</v>
+      </c>
+      <c r="D1426" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1426" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1426" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1426" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1426">
+        <v>0</v>
+      </c>
+      <c r="I1426">
+        <v>0</v>
+      </c>
+      <c r="J1426">
+        <v>0</v>
+      </c>
+      <c r="K1426">
+        <v>0</v>
+      </c>
+      <c r="L1426">
+        <v>0</v>
+      </c>
+      <c r="M1426">
+        <v>0</v>
+      </c>
+      <c r="N1426">
+        <v>0</v>
+      </c>
+      <c r="O1426" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1426" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1427">
+      <c r="A1427" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1427" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1427" t="str">
+        <v>Sandeep C</v>
+      </c>
+      <c r="D1427" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1427" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1427" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1427" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1427">
+        <v>0</v>
+      </c>
+      <c r="I1427">
+        <v>0</v>
+      </c>
+      <c r="J1427">
+        <v>0</v>
+      </c>
+      <c r="K1427">
+        <v>0</v>
+      </c>
+      <c r="L1427">
+        <v>0</v>
+      </c>
+      <c r="M1427">
+        <v>0</v>
+      </c>
+      <c r="N1427">
+        <v>0</v>
+      </c>
+      <c r="O1427" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1427" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1428">
+      <c r="A1428" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1428" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1428" t="str">
+        <v>Shahana Jabbar</v>
+      </c>
+      <c r="D1428" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1428" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1428" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1428" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1428">
+        <v>0</v>
+      </c>
+      <c r="I1428">
+        <v>0</v>
+      </c>
+      <c r="J1428">
+        <v>0</v>
+      </c>
+      <c r="K1428">
+        <v>0</v>
+      </c>
+      <c r="L1428">
+        <v>0</v>
+      </c>
+      <c r="M1428">
+        <v>0</v>
+      </c>
+      <c r="N1428">
+        <v>0</v>
+      </c>
+      <c r="O1428" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1428" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1429">
+      <c r="A1429" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1429" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1429" t="str">
+        <v>Shinodh N T</v>
+      </c>
+      <c r="D1429" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1429" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1429" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1429" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1429">
+        <v>0</v>
+      </c>
+      <c r="I1429">
+        <v>0</v>
+      </c>
+      <c r="J1429">
+        <v>0</v>
+      </c>
+      <c r="K1429">
+        <v>0</v>
+      </c>
+      <c r="L1429">
+        <v>0</v>
+      </c>
+      <c r="M1429">
+        <v>0</v>
+      </c>
+      <c r="N1429">
+        <v>0</v>
+      </c>
+      <c r="O1429" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1429" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1430">
+      <c r="A1430" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1430" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1430" t="str">
+        <v>Shyam Murali</v>
+      </c>
+      <c r="D1430" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1430" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1430" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1430" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1430">
+        <v>0</v>
+      </c>
+      <c r="I1430">
+        <v>0</v>
+      </c>
+      <c r="J1430">
+        <v>0</v>
+      </c>
+      <c r="K1430">
+        <v>0</v>
+      </c>
+      <c r="L1430">
+        <v>0</v>
+      </c>
+      <c r="M1430">
+        <v>0</v>
+      </c>
+      <c r="N1430">
+        <v>0</v>
+      </c>
+      <c r="O1430" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1430" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1431" xml:space="preserve">
+      <c r="A1431" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1431" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1431" t="str">
+        <v>Siju Thomas</v>
+      </c>
+      <c r="D1431" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E1431" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F1431" t="str">
+        <v>06:30 PM</v>
+      </c>
+      <c r="G1431" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H1431">
+        <v>0</v>
+      </c>
+      <c r="I1431">
+        <v>0</v>
+      </c>
+      <c r="J1431">
+        <v>0</v>
+      </c>
+      <c r="K1431">
+        <v>0</v>
+      </c>
+      <c r="L1431">
+        <v>0</v>
+      </c>
+      <c r="M1431">
+        <v>0</v>
+      </c>
+      <c r="N1431">
+        <v>0</v>
+      </c>
+      <c r="O1431" t="str" xml:space="preserve">
+        <v xml:space="preserve">10/06/2026
+6.30 pm</v>
+      </c>
+      <c r="P1431" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="1432">
+      <c r="A1432" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1432" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1432" t="str">
+        <v>Sineesh Sasi</v>
+      </c>
+      <c r="D1432" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1432" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1432" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1432" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1432">
+        <v>0</v>
+      </c>
+      <c r="I1432">
+        <v>0</v>
+      </c>
+      <c r="J1432">
+        <v>0</v>
+      </c>
+      <c r="K1432">
+        <v>0</v>
+      </c>
+      <c r="L1432">
+        <v>0</v>
+      </c>
+      <c r="M1432">
+        <v>0</v>
+      </c>
+      <c r="N1432">
+        <v>0</v>
+      </c>
+      <c r="O1432" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1432" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1433">
+      <c r="A1433" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1433" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1433" t="str">
+        <v>Sona Francis</v>
+      </c>
+      <c r="D1433" t="str">
+        <v>LEAVE</v>
+      </c>
+      <c r="E1433" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F1433" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1433" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1433">
+        <v>0</v>
+      </c>
+      <c r="I1433">
+        <v>0</v>
+      </c>
+      <c r="J1433">
+        <v>0</v>
+      </c>
+      <c r="K1433">
+        <v>0</v>
+      </c>
+      <c r="L1433">
+        <v>0</v>
+      </c>
+      <c r="M1433">
+        <v>0</v>
+      </c>
+      <c r="N1433">
+        <v>0</v>
+      </c>
+      <c r="O1433" t="str">
+        <v>I'm on leave today due to health issues</v>
+      </c>
+      <c r="P1433" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="1434">
+      <c r="A1434" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1434" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1434" t="str">
+        <v>Sreelakshmi R</v>
+      </c>
+      <c r="D1434" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1434" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1434" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1434" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1434">
+        <v>0</v>
+      </c>
+      <c r="I1434">
+        <v>0</v>
+      </c>
+      <c r="J1434">
+        <v>0</v>
+      </c>
+      <c r="K1434">
+        <v>0</v>
+      </c>
+      <c r="L1434">
+        <v>0</v>
+      </c>
+      <c r="M1434">
+        <v>0</v>
+      </c>
+      <c r="N1434">
+        <v>0</v>
+      </c>
+      <c r="O1434" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1434" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1435">
+      <c r="A1435" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1435" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1435" t="str">
+        <v>Sreenath C V</v>
+      </c>
+      <c r="D1435" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1435" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1435" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1435" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1435">
+        <v>0</v>
+      </c>
+      <c r="I1435">
+        <v>0</v>
+      </c>
+      <c r="J1435">
+        <v>0</v>
+      </c>
+      <c r="K1435">
+        <v>0</v>
+      </c>
+      <c r="L1435">
+        <v>0</v>
+      </c>
+      <c r="M1435">
+        <v>0</v>
+      </c>
+      <c r="N1435">
+        <v>0</v>
+      </c>
+      <c r="O1435" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1435" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1436">
+      <c r="A1436" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1436" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1436" t="str">
+        <v>Sreeraj V S</v>
+      </c>
+      <c r="D1436" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1436" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1436" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1436" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1436">
+        <v>0</v>
+      </c>
+      <c r="I1436">
+        <v>0</v>
+      </c>
+      <c r="J1436">
+        <v>0</v>
+      </c>
+      <c r="K1436">
+        <v>0</v>
+      </c>
+      <c r="L1436">
+        <v>0</v>
+      </c>
+      <c r="M1436">
+        <v>0</v>
+      </c>
+      <c r="N1436">
+        <v>0</v>
+      </c>
+      <c r="O1436" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1436" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1437">
+      <c r="A1437" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1437" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1437" t="str">
+        <v>Stephin Pious</v>
+      </c>
+      <c r="D1437" t="str">
+        <v>CHECKED-IN</v>
+      </c>
+      <c r="E1437" t="str">
+        <v>INTEREXT OFFICE</v>
+      </c>
+      <c r="F1437" t="str">
+        <v>08:55 AM</v>
+      </c>
+      <c r="G1437" t="str">
+        <v>Currently Checked-In</v>
+      </c>
+      <c r="H1437">
+        <v>0</v>
+      </c>
+      <c r="I1437">
+        <v>0</v>
+      </c>
+      <c r="J1437">
+        <v>0</v>
+      </c>
+      <c r="K1437">
+        <v>0</v>
+      </c>
+      <c r="L1437">
+        <v>0</v>
+      </c>
+      <c r="M1437">
+        <v>0</v>
+      </c>
+      <c r="N1437">
+        <v>0</v>
+      </c>
+      <c r="O1437" t="str">
+        <v>8.55 am</v>
+      </c>
+      <c r="P1437" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="1438">
+      <c r="A1438" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1438" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1438" t="str">
+        <v>Subodh Sha</v>
+      </c>
+      <c r="D1438" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1438" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1438" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1438" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1438">
+        <v>0</v>
+      </c>
+      <c r="I1438">
+        <v>0</v>
+      </c>
+      <c r="J1438">
+        <v>0</v>
+      </c>
+      <c r="K1438">
+        <v>0</v>
+      </c>
+      <c r="L1438">
+        <v>0</v>
+      </c>
+      <c r="M1438">
+        <v>0</v>
+      </c>
+      <c r="N1438">
+        <v>0</v>
+      </c>
+      <c r="O1438" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1438" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1439">
+      <c r="A1439" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1439" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1439" t="str">
+        <v>Sukanto Mishal</v>
+      </c>
+      <c r="D1439" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1439" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1439" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1439" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1439">
+        <v>0</v>
+      </c>
+      <c r="I1439">
+        <v>0</v>
+      </c>
+      <c r="J1439">
+        <v>0</v>
+      </c>
+      <c r="K1439">
+        <v>0</v>
+      </c>
+      <c r="L1439">
+        <v>0</v>
+      </c>
+      <c r="M1439">
+        <v>0</v>
+      </c>
+      <c r="N1439">
+        <v>0</v>
+      </c>
+      <c r="O1439" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1439" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1440">
+      <c r="A1440" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1440" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1440" t="str">
+        <v>Sumesh B</v>
+      </c>
+      <c r="D1440" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1440" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1440" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1440" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1440">
+        <v>0</v>
+      </c>
+      <c r="I1440">
+        <v>0</v>
+      </c>
+      <c r="J1440">
+        <v>0</v>
+      </c>
+      <c r="K1440">
+        <v>0</v>
+      </c>
+      <c r="L1440">
+        <v>0</v>
+      </c>
+      <c r="M1440">
+        <v>0</v>
+      </c>
+      <c r="N1440">
+        <v>0</v>
+      </c>
+      <c r="O1440" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1440" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1441">
+      <c r="A1441" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1441" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1441" t="str">
+        <v>Sunil Aliyar</v>
+      </c>
+      <c r="D1441" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1441" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1441" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1441" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1441">
+        <v>0</v>
+      </c>
+      <c r="I1441">
+        <v>0</v>
+      </c>
+      <c r="J1441">
+        <v>0</v>
+      </c>
+      <c r="K1441">
+        <v>0</v>
+      </c>
+      <c r="L1441">
+        <v>0</v>
+      </c>
+      <c r="M1441">
+        <v>0</v>
+      </c>
+      <c r="N1441">
+        <v>0</v>
+      </c>
+      <c r="O1441" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1441" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1442">
+      <c r="A1442" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1442" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1442" t="str">
+        <v>Sunil Rana</v>
+      </c>
+      <c r="D1442" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1442" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1442" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1442" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1442">
+        <v>0</v>
+      </c>
+      <c r="I1442">
+        <v>0</v>
+      </c>
+      <c r="J1442">
+        <v>0</v>
+      </c>
+      <c r="K1442">
+        <v>0</v>
+      </c>
+      <c r="L1442">
+        <v>0</v>
+      </c>
+      <c r="M1442">
+        <v>0</v>
+      </c>
+      <c r="N1442">
+        <v>0</v>
+      </c>
+      <c r="O1442" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1442" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1443">
+      <c r="A1443" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1443" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1443" t="str">
+        <v>Sunil. C. M</v>
+      </c>
+      <c r="D1443" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1443" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1443" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1443" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1443">
+        <v>0</v>
+      </c>
+      <c r="I1443">
+        <v>0</v>
+      </c>
+      <c r="J1443">
+        <v>0</v>
+      </c>
+      <c r="K1443">
+        <v>0</v>
+      </c>
+      <c r="L1443">
+        <v>0</v>
+      </c>
+      <c r="M1443">
+        <v>0</v>
+      </c>
+      <c r="N1443">
+        <v>0</v>
+      </c>
+      <c r="O1443" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1443" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1444">
+      <c r="A1444" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1444" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1444" t="str">
+        <v>Tufail Alam Danish</v>
+      </c>
+      <c r="D1444" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1444" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1444" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1444" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1444">
+        <v>0</v>
+      </c>
+      <c r="I1444">
+        <v>0</v>
+      </c>
+      <c r="J1444">
+        <v>0</v>
+      </c>
+      <c r="K1444">
+        <v>0</v>
+      </c>
+      <c r="L1444">
+        <v>0</v>
+      </c>
+      <c r="M1444">
+        <v>0</v>
+      </c>
+      <c r="N1444">
+        <v>0</v>
+      </c>
+      <c r="O1444" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1444" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
+    <row r="1445">
+      <c r="A1445" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="B1445" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C1445" t="str">
+        <v>Vijesh A V</v>
+      </c>
+      <c r="D1445" t="str">
+        <v>ABSENT</v>
+      </c>
+      <c r="E1445" t="str">
+        <v>—</v>
+      </c>
+      <c r="F1445" t="str">
+        <v>—</v>
+      </c>
+      <c r="G1445" t="str">
+        <v>—</v>
+      </c>
+      <c r="H1445">
+        <v>0</v>
+      </c>
+      <c r="I1445">
+        <v>0</v>
+      </c>
+      <c r="J1445">
+        <v>0</v>
+      </c>
+      <c r="K1445">
+        <v>0</v>
+      </c>
+      <c r="L1445">
+        <v>0</v>
+      </c>
+      <c r="M1445">
+        <v>0</v>
+      </c>
+      <c r="N1445">
+        <v>0</v>
+      </c>
+      <c r="O1445" t="str">
+        <v>—</v>
+      </c>
+      <c r="P1445" t="str">
+        <v>Auto-Marked Absent (Missing text)</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P1369"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P1445"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>